<commit_message>
Price check — 03/20/2026
</commit_message>
<xml_diff>
--- a/PriceBook_Combined_Final.xlsx
+++ b/PriceBook_Combined_Final.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="🧊 Refrigerators" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="📺 TVs" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="🧊 Refrigerators" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="📺 TVs" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21,7 +21,7 @@
     <numFmt numFmtId="164" formatCode="$#,##0.00"/>
     <numFmt numFmtId="165" formatCode="$#,##0"/>
   </numFmts>
-  <fonts count="18">
+  <fonts count="19">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -129,6 +129,11 @@
       <color rgb="00F59E0B"/>
       <sz val="9"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="0000897B"/>
+      <sz val="10"/>
+    </font>
   </fonts>
   <fills count="15">
     <fill>
@@ -229,7 +234,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -326,6 +331,15 @@
     </xf>
     <xf numFmtId="0" fontId="17" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="18" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -692,7 +706,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:O67"/>
+  <dimension ref="B1:P67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -710,6 +724,7 @@
     <col width="44" customWidth="1" min="13" max="13"/>
     <col width="14" customWidth="1" min="14" max="14"/>
     <col width="12" customWidth="1" min="15" max="15"/>
+    <col width="12" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1" ht="8" customHeight="1"/>
@@ -799,6 +814,11 @@
           <t>3/20</t>
         </is>
       </c>
+      <c r="P5" s="33" t="inlineStr">
+        <is>
+          <t>3/20</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="22" customHeight="1">
       <c r="B6" s="5" t="inlineStr">
@@ -866,6 +886,9 @@
       <c r="O7" s="14" t="n">
         <v>449.99</v>
       </c>
+      <c r="P7" s="34" t="n">
+        <v>449.99</v>
+      </c>
     </row>
     <row r="8" ht="18" customHeight="1">
       <c r="B8" s="15" t="n">
@@ -926,6 +949,11 @@
       <c r="O8" s="14" t="n">
         <v>659.99</v>
       </c>
+      <c r="P8" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="18" customHeight="1">
       <c r="B9" s="6" t="n">
@@ -986,6 +1014,11 @@
       <c r="O9" s="14" t="n">
         <v>659.99</v>
       </c>
+      <c r="P9" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="18" customHeight="1">
       <c r="B10" s="15" t="n">
@@ -1046,6 +1079,9 @@
       <c r="O10" s="14" t="n">
         <v>449.99</v>
       </c>
+      <c r="P10" s="34" t="n">
+        <v>449.99</v>
+      </c>
     </row>
     <row r="11" ht="18" customHeight="1">
       <c r="B11" s="6" t="n">
@@ -1106,6 +1142,11 @@
       <c r="O11" s="14" t="n">
         <v>659.99</v>
       </c>
+      <c r="P11" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="18" customHeight="1">
       <c r="B12" s="15" t="n">
@@ -1166,6 +1207,9 @@
       <c r="O12" s="14" t="n">
         <v>729.99</v>
       </c>
+      <c r="P12" s="34" t="n">
+        <v>729.99</v>
+      </c>
     </row>
     <row r="13" ht="5" customHeight="1"/>
     <row r="14" ht="22" customHeight="1">
@@ -1234,6 +1278,9 @@
       <c r="O15" s="14" t="n">
         <v>599.99</v>
       </c>
+      <c r="P15" s="34" t="n">
+        <v>599.99</v>
+      </c>
     </row>
     <row r="16" ht="18" customHeight="1">
       <c r="B16" s="15" t="n">
@@ -1294,6 +1341,9 @@
       <c r="O16" s="14" t="n">
         <v>749.99</v>
       </c>
+      <c r="P16" s="13" t="n">
+        <v>62.99</v>
+      </c>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="B17" s="6" t="n">
@@ -1354,6 +1404,9 @@
       <c r="O17" s="14" t="n">
         <v>899.99</v>
       </c>
+      <c r="P17" s="13" t="n">
+        <v>56.99</v>
+      </c>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="B18" s="15" t="n">
@@ -1470,6 +1523,9 @@
       <c r="O19" s="14" t="n">
         <v>2199.99</v>
       </c>
+      <c r="P19" s="34" t="n">
+        <v>2199.99</v>
+      </c>
     </row>
     <row r="20" ht="5" customHeight="1"/>
     <row r="21" ht="22" customHeight="1">
@@ -1538,6 +1594,9 @@
       <c r="O22" s="14" t="n">
         <v>1098.99</v>
       </c>
+      <c r="P22" s="34" t="n">
+        <v>1098.99</v>
+      </c>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="B23" s="6" t="n">
@@ -1598,6 +1657,11 @@
       <c r="O23" s="14" t="n">
         <v>1199.99</v>
       </c>
+      <c r="P23" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="B24" s="15" t="n">
@@ -1658,6 +1722,11 @@
       <c r="O24" s="14" t="n">
         <v>1199.99</v>
       </c>
+      <c r="P24" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="18" customHeight="1">
       <c r="B25" s="6" t="n">
@@ -1774,6 +1843,11 @@
       <c r="O26" s="14" t="n">
         <v>1599.99</v>
       </c>
+      <c r="P26" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="18" customHeight="1">
       <c r="B27" s="6" t="n">
@@ -1834,6 +1908,9 @@
       <c r="O27" s="14" t="n">
         <v>1799.99</v>
       </c>
+      <c r="P27" s="34" t="n">
+        <v>1799.99</v>
+      </c>
     </row>
     <row r="28" ht="18" customHeight="1">
       <c r="B28" s="15" t="n">
@@ -1894,6 +1971,9 @@
       <c r="O28" s="14" t="n">
         <v>1479.99</v>
       </c>
+      <c r="P28" s="34" t="n">
+        <v>1479.99</v>
+      </c>
     </row>
     <row r="29" ht="18" customHeight="1">
       <c r="B29" s="6" t="n">
@@ -1954,6 +2034,9 @@
       <c r="O29" s="14" t="n">
         <v>1799.99</v>
       </c>
+      <c r="P29" s="34" t="n">
+        <v>1799.99</v>
+      </c>
     </row>
     <row r="30" ht="18" customHeight="1">
       <c r="B30" s="15" t="n">
@@ -2014,6 +2097,9 @@
       <c r="O30" s="14" t="n">
         <v>1799.99</v>
       </c>
+      <c r="P30" s="34" t="n">
+        <v>1799.99</v>
+      </c>
     </row>
     <row r="31" ht="5" customHeight="1"/>
     <row r="32" ht="22" customHeight="1">
@@ -2082,6 +2168,9 @@
       <c r="O33" s="14" t="n">
         <v>1029.99</v>
       </c>
+      <c r="P33" s="34" t="n">
+        <v>1029.99</v>
+      </c>
     </row>
     <row r="34" ht="18" customHeight="1">
       <c r="B34" s="15" t="n">
@@ -2142,6 +2231,9 @@
       <c r="O34" s="14" t="n">
         <v>1029.99</v>
       </c>
+      <c r="P34" s="34" t="n">
+        <v>1029.99</v>
+      </c>
     </row>
     <row r="35" ht="18" customHeight="1">
       <c r="B35" s="6" t="n">
@@ -2202,6 +2294,11 @@
       <c r="O35" s="14" t="n">
         <v>1599.99</v>
       </c>
+      <c r="P35" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="18" customHeight="1">
       <c r="B36" s="15" t="n">
@@ -2262,6 +2359,9 @@
       <c r="O36" s="14" t="n">
         <v>1699.99</v>
       </c>
+      <c r="P36" s="34" t="n">
+        <v>1699.99</v>
+      </c>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="B37" s="6" t="n">
@@ -2322,6 +2422,9 @@
       <c r="O37" s="14" t="n">
         <v>2499.99</v>
       </c>
+      <c r="P37" s="34" t="n">
+        <v>2499.99</v>
+      </c>
     </row>
     <row r="38" ht="18" customHeight="1">
       <c r="B38" s="15" t="n">
@@ -2382,6 +2485,9 @@
       <c r="O38" s="14" t="n">
         <v>2898.99</v>
       </c>
+      <c r="P38" s="34" t="n">
+        <v>2898.99</v>
+      </c>
     </row>
     <row r="39" ht="18" customHeight="1">
       <c r="B39" s="6" t="n">
@@ -2442,6 +2548,9 @@
       <c r="O39" s="14" t="n">
         <v>2499.99</v>
       </c>
+      <c r="P39" s="34" t="n">
+        <v>2499.99</v>
+      </c>
     </row>
     <row r="40" ht="18" customHeight="1">
       <c r="B40" s="15" t="n">
@@ -2502,6 +2611,9 @@
       <c r="O40" s="14" t="n">
         <v>1029.99</v>
       </c>
+      <c r="P40" s="34" t="n">
+        <v>1029.99</v>
+      </c>
     </row>
     <row r="41" ht="18" customHeight="1">
       <c r="B41" s="6" t="n">
@@ -2562,6 +2674,9 @@
       <c r="O41" s="14" t="n">
         <v>1749.99</v>
       </c>
+      <c r="P41" s="34" t="n">
+        <v>1749.99</v>
+      </c>
     </row>
     <row r="42" ht="18" customHeight="1">
       <c r="B42" s="15" t="n">
@@ -2622,6 +2737,9 @@
       <c r="O42" s="14" t="n">
         <v>1899.99</v>
       </c>
+      <c r="P42" s="34" t="n">
+        <v>1899.99</v>
+      </c>
     </row>
     <row r="43" ht="18" customHeight="1">
       <c r="B43" s="6" t="n">
@@ -2738,6 +2856,9 @@
       <c r="O44" s="14" t="n">
         <v>3599.99</v>
       </c>
+      <c r="P44" s="34" t="n">
+        <v>3599.99</v>
+      </c>
     </row>
     <row r="45" ht="5" customHeight="1"/>
     <row r="46" ht="22" customHeight="1">
@@ -2806,6 +2927,9 @@
       <c r="O47" s="14" t="n">
         <v>1899.99</v>
       </c>
+      <c r="P47" s="34" t="n">
+        <v>1899.99</v>
+      </c>
     </row>
     <row r="48" ht="18" customHeight="1">
       <c r="B48" s="15" t="n">
@@ -2866,6 +2990,11 @@
       <c r="O48" s="14" t="n">
         <v>1599.99</v>
       </c>
+      <c r="P48" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="49" ht="18" customHeight="1">
       <c r="B49" s="6" t="n">
@@ -2926,6 +3055,11 @@
       <c r="O49" s="14" t="n">
         <v>1849.99</v>
       </c>
+      <c r="P49" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="50" ht="18" customHeight="1">
       <c r="B50" s="15" t="n">
@@ -2986,6 +3120,9 @@
       <c r="O50" s="14" t="n">
         <v>2599.99</v>
       </c>
+      <c r="P50" s="34" t="n">
+        <v>2599.99</v>
+      </c>
     </row>
     <row r="51" ht="18" customHeight="1">
       <c r="B51" s="6" t="n">
@@ -3102,6 +3239,9 @@
       <c r="O52" s="14" t="n">
         <v>2599.99</v>
       </c>
+      <c r="P52" s="34" t="n">
+        <v>2599.99</v>
+      </c>
     </row>
     <row r="53" ht="18" customHeight="1">
       <c r="B53" s="6" t="n">
@@ -3162,6 +3302,9 @@
       <c r="O53" s="14" t="n">
         <v>3499.99</v>
       </c>
+      <c r="P53" s="34" t="n">
+        <v>3499.99</v>
+      </c>
     </row>
     <row r="54" ht="5" customHeight="1"/>
     <row r="55" ht="22" customHeight="1">
@@ -3230,6 +3373,9 @@
       <c r="O56" s="14" t="n">
         <v>3599.99</v>
       </c>
+      <c r="P56" s="34" t="n">
+        <v>3599.99</v>
+      </c>
     </row>
     <row r="57" ht="18" customHeight="1">
       <c r="B57" s="26" t="n">
@@ -3466,6 +3612,11 @@
       <c r="O62" s="14" t="n">
         <v>127.99</v>
       </c>
+      <c r="P62" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="63" ht="18" customHeight="1">
       <c r="B63" s="6" t="n">
@@ -3526,6 +3677,9 @@
       <c r="O63" s="14" t="n">
         <v>279.99</v>
       </c>
+      <c r="P63" s="13" t="n">
+        <v>39.99</v>
+      </c>
     </row>
     <row r="64" ht="18" customHeight="1">
       <c r="B64" s="15" t="n">
@@ -3585,6 +3739,9 @@
       </c>
       <c r="O64" s="14" t="n">
         <v>379.99</v>
+      </c>
+      <c r="P64" s="13" t="n">
+        <v>21.99</v>
       </c>
     </row>
     <row r="65" ht="18" customHeight="1">
@@ -3818,7 +3975,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:O70"/>
+  <dimension ref="B1:P70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -3836,6 +3993,7 @@
     <col width="44" customWidth="1" min="13" max="13"/>
     <col width="14" customWidth="1" min="14" max="14"/>
     <col width="12" customWidth="1" min="15" max="15"/>
+    <col width="12" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1" ht="8" customHeight="1"/>
@@ -3925,6 +4083,11 @@
           <t>3/20</t>
         </is>
       </c>
+      <c r="P5" s="33" t="inlineStr">
+        <is>
+          <t>3/20</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="22" customHeight="1">
       <c r="B6" s="5" t="inlineStr">
@@ -3992,6 +4155,9 @@
       <c r="O7" s="14" t="n">
         <v>89.98999999999999</v>
       </c>
+      <c r="P7" s="34" t="n">
+        <v>89.98999999999999</v>
+      </c>
     </row>
     <row r="8" ht="18" customHeight="1">
       <c r="B8" s="15" t="n">
@@ -4052,6 +4218,9 @@
       <c r="O8" s="14" t="n">
         <v>194.99</v>
       </c>
+      <c r="P8" s="34" t="n">
+        <v>194.99</v>
+      </c>
     </row>
     <row r="9" ht="18" customHeight="1">
       <c r="B9" s="6" t="n">
@@ -4112,6 +4281,9 @@
       <c r="O9" s="14" t="n">
         <v>299.99</v>
       </c>
+      <c r="P9" s="13" t="n">
+        <v>34.99</v>
+      </c>
     </row>
     <row r="10" ht="18" customHeight="1">
       <c r="B10" s="15" t="n">
@@ -4228,6 +4400,9 @@
       <c r="O11" s="14" t="n">
         <v>219.99</v>
       </c>
+      <c r="P11" s="34" t="n">
+        <v>219.99</v>
+      </c>
     </row>
     <row r="12" ht="18" customHeight="1">
       <c r="B12" s="15" t="n">
@@ -4288,6 +4463,11 @@
       <c r="O12" s="14" t="n">
         <v>349.99</v>
       </c>
+      <c r="P12" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="18" customHeight="1">
       <c r="B13" s="6" t="n">
@@ -4348,6 +4528,9 @@
       <c r="O13" s="14" t="n">
         <v>597.99</v>
       </c>
+      <c r="P13" s="13" t="n">
+        <v>39.99</v>
+      </c>
     </row>
     <row r="14" ht="5" customHeight="1"/>
     <row r="15" ht="22" customHeight="1">
@@ -4416,6 +4599,9 @@
       <c r="O16" s="14" t="n">
         <v>299.99</v>
       </c>
+      <c r="P16" s="13" t="n">
+        <v>34.99</v>
+      </c>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="B17" s="6" t="n">
@@ -4476,6 +4662,9 @@
       <c r="O17" s="14" t="n">
         <v>279.99</v>
       </c>
+      <c r="P17" s="34" t="n">
+        <v>279.99</v>
+      </c>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="B18" s="15" t="n">
@@ -4536,6 +4725,9 @@
       <c r="O18" s="14" t="n">
         <v>399.99</v>
       </c>
+      <c r="P18" s="34" t="n">
+        <v>399.99</v>
+      </c>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="B19" s="6" t="n">
@@ -4596,6 +4788,9 @@
       <c r="O19" s="14" t="n">
         <v>249.99</v>
       </c>
+      <c r="P19" s="34" t="n">
+        <v>249.99</v>
+      </c>
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="B20" s="15" t="n">
@@ -4656,6 +4851,11 @@
       <c r="O20" s="14" t="n">
         <v>427.99</v>
       </c>
+      <c r="P20" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="B21" s="6" t="n">
@@ -4716,6 +4916,9 @@
       <c r="O21" s="14" t="n">
         <v>478.99</v>
       </c>
+      <c r="P21" s="34" t="n">
+        <v>478.99</v>
+      </c>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="B22" s="15" t="n">
@@ -4776,6 +4979,11 @@
       <c r="O22" s="14" t="n">
         <v>599.99</v>
       </c>
+      <c r="P22" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="B23" s="6" t="n">
@@ -4836,6 +5044,9 @@
       <c r="O23" s="14" t="n">
         <v>999.99</v>
       </c>
+      <c r="P23" s="34" t="n">
+        <v>999.99</v>
+      </c>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="B24" s="15" t="n">
@@ -4896,6 +5107,9 @@
       <c r="O24" s="14" t="n">
         <v>1296.99</v>
       </c>
+      <c r="P24" s="13" t="n">
+        <v>29.99</v>
+      </c>
     </row>
     <row r="25" ht="18" customHeight="1">
       <c r="B25" s="6" t="n">
@@ -4956,6 +5170,9 @@
       <c r="O25" s="14" t="n">
         <v>1199.99</v>
       </c>
+      <c r="P25" s="34" t="n">
+        <v>1199.99</v>
+      </c>
     </row>
     <row r="26" ht="18" customHeight="1">
       <c r="B26" s="15" t="n">
@@ -5016,6 +5233,9 @@
       <c r="O26" s="14" t="n">
         <v>1274.99</v>
       </c>
+      <c r="P26" s="34" t="n">
+        <v>1274.99</v>
+      </c>
     </row>
     <row r="27" ht="5" customHeight="1"/>
     <row r="28" ht="22" customHeight="1">
@@ -5084,6 +5304,9 @@
       <c r="O29" s="14" t="n">
         <v>369.99</v>
       </c>
+      <c r="P29" s="34" t="n">
+        <v>369.99</v>
+      </c>
     </row>
     <row r="30" ht="18" customHeight="1">
       <c r="B30" s="15" t="n">
@@ -5144,6 +5367,9 @@
       <c r="O30" s="14" t="n">
         <v>579.99</v>
       </c>
+      <c r="P30" s="34" t="n">
+        <v>579.99</v>
+      </c>
     </row>
     <row r="31" ht="18" customHeight="1">
       <c r="B31" s="6" t="n">
@@ -5204,6 +5430,11 @@
       <c r="O31" s="14" t="n">
         <v>746.99</v>
       </c>
+      <c r="P31" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="18" customHeight="1">
       <c r="B32" s="15" t="n">
@@ -5264,6 +5495,9 @@
       <c r="O32" s="14" t="n">
         <v>759.99</v>
       </c>
+      <c r="P32" s="34" t="n">
+        <v>759.99</v>
+      </c>
     </row>
     <row r="33" ht="18" customHeight="1">
       <c r="B33" s="6" t="n">
@@ -5324,6 +5558,9 @@
       <c r="O33" s="14" t="n">
         <v>799.99</v>
       </c>
+      <c r="P33" s="34" t="n">
+        <v>799.99</v>
+      </c>
     </row>
     <row r="34" ht="18" customHeight="1">
       <c r="B34" s="15" t="n">
@@ -5384,6 +5621,9 @@
       <c r="O34" s="14" t="n">
         <v>1274.99</v>
       </c>
+      <c r="P34" s="34" t="n">
+        <v>1274.99</v>
+      </c>
     </row>
     <row r="35" ht="18" customHeight="1">
       <c r="B35" s="6" t="n">
@@ -5444,6 +5684,9 @@
       <c r="O35" s="14" t="n">
         <v>1799.99</v>
       </c>
+      <c r="P35" s="34" t="n">
+        <v>1799.99</v>
+      </c>
     </row>
     <row r="36" ht="18" customHeight="1">
       <c r="B36" s="15" t="n">
@@ -5504,6 +5747,9 @@
       <c r="O36" s="14" t="n">
         <v>1975.99</v>
       </c>
+      <c r="P36" s="34" t="n">
+        <v>1975.99</v>
+      </c>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="B37" s="6" t="n">
@@ -5564,6 +5810,9 @@
       <c r="O37" s="14" t="n">
         <v>2699.99</v>
       </c>
+      <c r="P37" s="34" t="n">
+        <v>2699.99</v>
+      </c>
     </row>
     <row r="38" ht="5" customHeight="1"/>
     <row r="39" ht="22" customHeight="1">
@@ -5632,6 +5881,9 @@
       <c r="O40" s="14" t="n">
         <v>740.99</v>
       </c>
+      <c r="P40" s="34" t="n">
+        <v>740.99</v>
+      </c>
     </row>
     <row r="41" ht="18" customHeight="1">
       <c r="B41" s="6" t="n">
@@ -5692,6 +5944,9 @@
       <c r="O41" s="14" t="n">
         <v>649.99</v>
       </c>
+      <c r="P41" s="34" t="n">
+        <v>649.99</v>
+      </c>
     </row>
     <row r="42" ht="18" customHeight="1">
       <c r="B42" s="15" t="n">
@@ -5752,6 +6007,9 @@
       <c r="O42" s="14" t="n">
         <v>799.99</v>
       </c>
+      <c r="P42" s="34" t="n">
+        <v>799.99</v>
+      </c>
     </row>
     <row r="43" ht="18" customHeight="1">
       <c r="B43" s="6" t="n">
@@ -5812,6 +6070,9 @@
       <c r="O43" s="14" t="n">
         <v>949.99</v>
       </c>
+      <c r="P43" s="34" t="n">
+        <v>949.99</v>
+      </c>
     </row>
     <row r="44" ht="18" customHeight="1">
       <c r="B44" s="15" t="n">
@@ -5872,6 +6133,9 @@
       <c r="O44" s="14" t="n">
         <v>1139.99</v>
       </c>
+      <c r="P44" s="34" t="n">
+        <v>1139.99</v>
+      </c>
     </row>
     <row r="45" ht="18" customHeight="1">
       <c r="B45" s="6" t="n">
@@ -5932,6 +6196,9 @@
       <c r="O45" s="14" t="n">
         <v>1529.99</v>
       </c>
+      <c r="P45" s="34" t="n">
+        <v>1529.99</v>
+      </c>
     </row>
     <row r="46" ht="18" customHeight="1">
       <c r="B46" s="15" t="n">
@@ -5992,6 +6259,9 @@
       <c r="O46" s="14" t="n">
         <v>2199.99</v>
       </c>
+      <c r="P46" s="13" t="n">
+        <v>59.99</v>
+      </c>
     </row>
     <row r="47" ht="18" customHeight="1">
       <c r="B47" s="6" t="n">
@@ -6052,6 +6322,9 @@
       <c r="O47" s="14" t="n">
         <v>2999.99</v>
       </c>
+      <c r="P47" s="34" t="n">
+        <v>2999.99</v>
+      </c>
     </row>
     <row r="48" ht="18" customHeight="1">
       <c r="B48" s="15" t="n">
@@ -6112,6 +6385,11 @@
       <c r="O48" s="14" t="n">
         <v>3499.99</v>
       </c>
+      <c r="P48" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="49" ht="5" customHeight="1"/>
     <row r="50" ht="22" customHeight="1">
@@ -6180,6 +6458,9 @@
       <c r="O51" s="14" t="n">
         <v>798.99</v>
       </c>
+      <c r="P51" s="34" t="n">
+        <v>798.99</v>
+      </c>
     </row>
     <row r="52" ht="18" customHeight="1">
       <c r="B52" s="15" t="n">
@@ -6240,6 +6521,9 @@
       <c r="O52" s="14" t="n">
         <v>798.99</v>
       </c>
+      <c r="P52" s="34" t="n">
+        <v>798.99</v>
+      </c>
     </row>
     <row r="53" ht="18" customHeight="1">
       <c r="B53" s="6" t="n">
@@ -6300,6 +6584,11 @@
       <c r="O53" s="14" t="n">
         <v>1499.99</v>
       </c>
+      <c r="P53" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="54" ht="18" customHeight="1">
       <c r="B54" s="15" t="n">
@@ -6360,6 +6649,9 @@
       <c r="O54" s="14" t="n">
         <v>899.99</v>
       </c>
+      <c r="P54" s="34" t="n">
+        <v>899.99</v>
+      </c>
     </row>
     <row r="55" ht="18" customHeight="1">
       <c r="B55" s="6" t="n">
@@ -6420,6 +6712,9 @@
       <c r="O55" s="14" t="n">
         <v>1397.99</v>
       </c>
+      <c r="P55" s="34" t="n">
+        <v>1397.99</v>
+      </c>
     </row>
     <row r="56" ht="18" customHeight="1">
       <c r="B56" s="15" t="n">
@@ -6480,6 +6775,9 @@
       <c r="O56" s="14" t="n">
         <v>2799.99</v>
       </c>
+      <c r="P56" s="34" t="n">
+        <v>2799.99</v>
+      </c>
     </row>
     <row r="57" ht="18" customHeight="1">
       <c r="B57" s="6" t="n">
@@ -6540,6 +6838,11 @@
       <c r="O57" s="14" t="n">
         <v>3199.99</v>
       </c>
+      <c r="P57" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="58" ht="18" customHeight="1">
       <c r="B58" s="26" t="n">
@@ -6664,6 +6967,9 @@
       <c r="O61" s="14" t="n">
         <v>999.99</v>
       </c>
+      <c r="P61" s="34" t="n">
+        <v>999.99</v>
+      </c>
     </row>
     <row r="62" ht="18" customHeight="1">
       <c r="B62" s="15" t="n">
@@ -6780,6 +7086,9 @@
       <c r="O63" s="14" t="n">
         <v>1658.99</v>
       </c>
+      <c r="P63" s="34" t="n">
+        <v>1658.99</v>
+      </c>
     </row>
     <row r="64" ht="18" customHeight="1">
       <c r="B64" s="15" t="n">
@@ -6840,6 +7149,9 @@
       <c r="O64" s="14" t="n">
         <v>2549.99</v>
       </c>
+      <c r="P64" s="34" t="n">
+        <v>2549.99</v>
+      </c>
     </row>
     <row r="65" ht="18" customHeight="1">
       <c r="B65" s="26" t="n">
@@ -7074,6 +7386,9 @@
         <v>1899.99</v>
       </c>
       <c r="O70" s="14" t="n">
+        <v>1899.99</v>
+      </c>
+      <c r="P70" s="34" t="n">
         <v>1899.99</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Price check — 03/22/2026
</commit_message>
<xml_diff>
--- a/PriceBook_Combined_Final.xlsx
+++ b/PriceBook_Combined_Final.xlsx
@@ -709,7 +709,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:Z67"/>
+  <dimension ref="B1:AA67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -738,6 +738,7 @@
     <col width="12" customWidth="1" min="24" max="24"/>
     <col width="12" customWidth="1" min="25" max="25"/>
     <col width="12" customWidth="1" min="26" max="26"/>
+    <col width="12" customWidth="1" min="27" max="27"/>
   </cols>
   <sheetData>
     <row r="1" ht="8" customHeight="1"/>
@@ -882,6 +883,11 @@
           <t>3/21</t>
         </is>
       </c>
+      <c r="AA5" s="33" t="inlineStr">
+        <is>
+          <t>3/22</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="22" customHeight="1">
       <c r="B6" s="5" t="inlineStr">
@@ -982,6 +988,9 @@
       <c r="Z7" s="34" t="n">
         <v>449.99</v>
       </c>
+      <c r="AA7" s="34" t="n">
+        <v>449.99</v>
+      </c>
     </row>
     <row r="8" ht="18" customHeight="1">
       <c r="B8" s="15" t="n">
@@ -1093,6 +1102,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AA8" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="18" customHeight="1">
       <c r="B9" s="6" t="n">
@@ -1204,6 +1218,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AA9" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="18" customHeight="1">
       <c r="B10" s="15" t="n">
@@ -1297,6 +1316,9 @@
       <c r="Z10" s="34" t="n">
         <v>449.99</v>
       </c>
+      <c r="AA10" s="34" t="n">
+        <v>449.99</v>
+      </c>
     </row>
     <row r="11" ht="18" customHeight="1">
       <c r="B11" s="6" t="n">
@@ -1408,6 +1430,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AA11" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="18" customHeight="1">
       <c r="B12" s="15" t="n">
@@ -1505,6 +1532,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AA12" s="34" t="n">
+        <v>729.99</v>
+      </c>
     </row>
     <row r="13" ht="5" customHeight="1"/>
     <row r="14" ht="22" customHeight="1">
@@ -1614,6 +1644,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AA15" s="34" t="n">
+        <v>599.99</v>
+      </c>
     </row>
     <row r="16" ht="18" customHeight="1">
       <c r="B16" s="15" t="n">
@@ -1711,6 +1744,11 @@
       <c r="Z16" s="13" t="n">
         <v>659.99</v>
       </c>
+      <c r="AA16" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="B17" s="6" t="n">
@@ -1822,6 +1860,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AA17" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="B18" s="15" t="n">
@@ -1977,6 +2020,9 @@
       <c r="Z19" s="34" t="n">
         <v>2199.99</v>
       </c>
+      <c r="AA19" s="34" t="n">
+        <v>2199.99</v>
+      </c>
     </row>
     <row r="20" ht="5" customHeight="1"/>
     <row r="21" ht="22" customHeight="1">
@@ -2084,6 +2130,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AA22" s="34" t="n">
+        <v>1098.99</v>
+      </c>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="B23" s="6" t="n">
@@ -2187,6 +2236,9 @@
       <c r="Z23" s="34" t="n">
         <v>1199.99</v>
       </c>
+      <c r="AA23" s="34" t="n">
+        <v>1199.99</v>
+      </c>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="B24" s="15" t="n">
@@ -2290,6 +2342,9 @@
       <c r="Z24" s="34" t="n">
         <v>1199.99</v>
       </c>
+      <c r="AA24" s="34" t="n">
+        <v>1199.99</v>
+      </c>
     </row>
     <row r="25" ht="18" customHeight="1">
       <c r="B25" s="6" t="n">
@@ -2451,6 +2506,9 @@
       <c r="Z26" s="34" t="n">
         <v>1599.99</v>
       </c>
+      <c r="AA26" s="34" t="n">
+        <v>1599.99</v>
+      </c>
     </row>
     <row r="27" ht="18" customHeight="1">
       <c r="B27" s="6" t="n">
@@ -2548,6 +2606,11 @@
       <c r="Z27" s="34" t="n">
         <v>1799.99</v>
       </c>
+      <c r="AA27" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="18" customHeight="1">
       <c r="B28" s="15" t="n">
@@ -2643,6 +2706,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AA28" s="34" t="n">
+        <v>1479.99</v>
+      </c>
     </row>
     <row r="29" ht="18" customHeight="1">
       <c r="B29" s="6" t="n">
@@ -2740,6 +2806,11 @@
       <c r="Z29" s="34" t="n">
         <v>1799.99</v>
       </c>
+      <c r="AA29" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="18" customHeight="1">
       <c r="B30" s="15" t="n">
@@ -2837,6 +2908,11 @@
       <c r="Z30" s="34" t="n">
         <v>1799.99</v>
       </c>
+      <c r="AA30" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="5" customHeight="1"/>
     <row r="32" ht="22" customHeight="1">
@@ -2942,6 +3018,11 @@
       <c r="Z33" s="34" t="n">
         <v>1029.99</v>
       </c>
+      <c r="AA33" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="18" customHeight="1">
       <c r="B34" s="15" t="n">
@@ -3039,6 +3120,11 @@
       <c r="Z34" s="34" t="n">
         <v>1029.99</v>
       </c>
+      <c r="AA34" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="18" customHeight="1">
       <c r="B35" s="6" t="n">
@@ -3144,6 +3230,9 @@
       <c r="Z35" s="34" t="n">
         <v>1599.99</v>
       </c>
+      <c r="AA35" s="34" t="n">
+        <v>1599.99</v>
+      </c>
     </row>
     <row r="36" ht="18" customHeight="1">
       <c r="B36" s="15" t="n">
@@ -3245,6 +3334,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AA36" s="34" t="n">
+        <v>1699.99</v>
+      </c>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="B37" s="6" t="n">
@@ -3344,6 +3436,9 @@
       <c r="Z37" s="34" t="n">
         <v>2499.99</v>
       </c>
+      <c r="AA37" s="34" t="n">
+        <v>2499.99</v>
+      </c>
     </row>
     <row r="38" ht="18" customHeight="1">
       <c r="B38" s="15" t="n">
@@ -3443,6 +3538,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AA38" s="34" t="n">
+        <v>2898.99</v>
+      </c>
     </row>
     <row r="39" ht="18" customHeight="1">
       <c r="B39" s="6" t="n">
@@ -3542,6 +3640,9 @@
       <c r="Z39" s="34" t="n">
         <v>2499.99</v>
       </c>
+      <c r="AA39" s="34" t="n">
+        <v>2499.99</v>
+      </c>
     </row>
     <row r="40" ht="18" customHeight="1">
       <c r="B40" s="15" t="n">
@@ -3639,6 +3740,11 @@
       <c r="Z40" s="34" t="n">
         <v>1029.99</v>
       </c>
+      <c r="AA40" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="18" customHeight="1">
       <c r="B41" s="6" t="n">
@@ -3736,6 +3842,9 @@
       <c r="Z41" s="34" t="n">
         <v>1749.99</v>
       </c>
+      <c r="AA41" s="34" t="n">
+        <v>1749.99</v>
+      </c>
     </row>
     <row r="42" ht="18" customHeight="1">
       <c r="B42" s="15" t="n">
@@ -3843,6 +3952,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AA42" s="34" t="n">
+        <v>1899.99</v>
+      </c>
     </row>
     <row r="43" ht="18" customHeight="1">
       <c r="B43" s="6" t="n">
@@ -3996,6 +4108,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AA44" s="34" t="n">
+        <v>3599.99</v>
+      </c>
     </row>
     <row r="45" ht="5" customHeight="1"/>
     <row r="46" ht="22" customHeight="1">
@@ -4111,6 +4226,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AA47" s="34" t="n">
+        <v>1899.99</v>
+      </c>
     </row>
     <row r="48" ht="18" customHeight="1">
       <c r="B48" s="15" t="n">
@@ -4216,6 +4334,9 @@
       <c r="Z48" s="34" t="n">
         <v>1599.99</v>
       </c>
+      <c r="AA48" s="34" t="n">
+        <v>1599.99</v>
+      </c>
     </row>
     <row r="49" ht="18" customHeight="1">
       <c r="B49" s="6" t="n">
@@ -4317,6 +4438,9 @@
       <c r="Z49" s="34" t="n">
         <v>1849.99</v>
       </c>
+      <c r="AA49" s="34" t="n">
+        <v>1849.99</v>
+      </c>
     </row>
     <row r="50" ht="18" customHeight="1">
       <c r="B50" s="15" t="n">
@@ -4414,6 +4538,9 @@
       <c r="Z50" s="34" t="n">
         <v>2599.99</v>
       </c>
+      <c r="AA50" s="34" t="n">
+        <v>2599.99</v>
+      </c>
     </row>
     <row r="51" ht="18" customHeight="1">
       <c r="B51" s="6" t="n">
@@ -4567,6 +4694,9 @@
       <c r="Z52" s="34" t="n">
         <v>2599.99</v>
       </c>
+      <c r="AA52" s="34" t="n">
+        <v>2599.99</v>
+      </c>
     </row>
     <row r="53" ht="18" customHeight="1">
       <c r="B53" s="6" t="n">
@@ -4664,6 +4794,9 @@
       <c r="Z53" s="34" t="n">
         <v>3499.99</v>
       </c>
+      <c r="AA53" s="34" t="n">
+        <v>3499.99</v>
+      </c>
     </row>
     <row r="54" ht="5" customHeight="1"/>
     <row r="55" ht="22" customHeight="1">
@@ -4769,6 +4902,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AA56" s="34" t="n">
+        <v>3599.99</v>
+      </c>
     </row>
     <row r="57" ht="18" customHeight="1">
       <c r="B57" s="26" t="n">
@@ -5046,6 +5182,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AA62" s="34" t="n">
+        <v>127.99</v>
+      </c>
     </row>
     <row r="63" ht="18" customHeight="1">
       <c r="B63" s="6" t="n">
@@ -5151,6 +5290,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AA63" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="64" ht="18" customHeight="1">
       <c r="B64" s="15" t="n">
@@ -5252,6 +5396,9 @@
         <v>499.99</v>
       </c>
       <c r="Z64" s="36" t="n">
+        <v>499.99</v>
+      </c>
+      <c r="AA64" s="36" t="n">
         <v>499.99</v>
       </c>
     </row>
@@ -5486,7 +5633,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:Z70"/>
+  <dimension ref="B1:AA70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -5515,6 +5662,7 @@
     <col width="12" customWidth="1" min="24" max="24"/>
     <col width="12" customWidth="1" min="25" max="25"/>
     <col width="12" customWidth="1" min="26" max="26"/>
+    <col width="12" customWidth="1" min="27" max="27"/>
   </cols>
   <sheetData>
     <row r="1" ht="8" customHeight="1"/>
@@ -5659,6 +5807,11 @@
           <t>3/21</t>
         </is>
       </c>
+      <c r="AA5" s="33" t="inlineStr">
+        <is>
+          <t>3/22</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="22" customHeight="1">
       <c r="B6" s="5" t="inlineStr">
@@ -5767,6 +5920,9 @@
       <c r="Z7" s="34" t="n">
         <v>89.98999999999999</v>
       </c>
+      <c r="AA7" s="34" t="n">
+        <v>89.98999999999999</v>
+      </c>
     </row>
     <row r="8" ht="18" customHeight="1">
       <c r="B8" s="15" t="n">
@@ -5866,6 +6022,9 @@
       <c r="Z8" s="34" t="n">
         <v>194.99</v>
       </c>
+      <c r="AA8" s="34" t="n">
+        <v>194.99</v>
+      </c>
     </row>
     <row r="9" ht="18" customHeight="1">
       <c r="B9" s="6" t="n">
@@ -5975,6 +6134,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AA9" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="18" customHeight="1">
       <c r="B10" s="15" t="n">
@@ -6124,6 +6288,9 @@
       <c r="Z11" s="34" t="n">
         <v>219.99</v>
       </c>
+      <c r="AA11" s="34" t="n">
+        <v>219.99</v>
+      </c>
     </row>
     <row r="12" ht="18" customHeight="1">
       <c r="B12" s="15" t="n">
@@ -6227,6 +6394,9 @@
       <c r="Z12" s="34" t="n">
         <v>349.99</v>
       </c>
+      <c r="AA12" s="34" t="n">
+        <v>349.99</v>
+      </c>
     </row>
     <row r="13" ht="18" customHeight="1">
       <c r="B13" s="6" t="n">
@@ -6334,6 +6504,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AA13" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="5" customHeight="1"/>
     <row r="15" ht="22" customHeight="1">
@@ -6451,6 +6626,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AA16" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="B17" s="6" t="n">
@@ -6544,6 +6724,9 @@
       <c r="Z17" s="34" t="n">
         <v>279.99</v>
       </c>
+      <c r="AA17" s="34" t="n">
+        <v>279.99</v>
+      </c>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="B18" s="15" t="n">
@@ -6645,6 +6828,9 @@
       <c r="Z18" s="34" t="n">
         <v>399.99</v>
       </c>
+      <c r="AA18" s="34" t="n">
+        <v>399.99</v>
+      </c>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="B19" s="6" t="n">
@@ -6744,6 +6930,9 @@
       <c r="Z19" s="34" t="n">
         <v>249.99</v>
       </c>
+      <c r="AA19" s="34" t="n">
+        <v>249.99</v>
+      </c>
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="B20" s="15" t="n">
@@ -6841,6 +7030,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AA20" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="B21" s="6" t="n">
@@ -6934,6 +7128,9 @@
       <c r="Z21" s="34" t="n">
         <v>478.99</v>
       </c>
+      <c r="AA21" s="34" t="n">
+        <v>478.99</v>
+      </c>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="B22" s="15" t="n">
@@ -7041,6 +7238,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AA22" s="34" t="n">
+        <v>599.99</v>
+      </c>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="B23" s="6" t="n">
@@ -7138,6 +7338,11 @@
       <c r="Z23" s="34" t="n">
         <v>999.99</v>
       </c>
+      <c r="AA23" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="B24" s="15" t="n">
@@ -7245,6 +7450,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AA24" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="18" customHeight="1">
       <c r="B25" s="6" t="n">
@@ -7348,6 +7558,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AA25" s="34" t="n">
+        <v>1199.99</v>
+      </c>
     </row>
     <row r="26" ht="18" customHeight="1">
       <c r="B26" s="15" t="n">
@@ -7447,6 +7660,9 @@
       <c r="Z26" s="34" t="n">
         <v>1274.99</v>
       </c>
+      <c r="AA26" s="34" t="n">
+        <v>1274.99</v>
+      </c>
     </row>
     <row r="27" ht="5" customHeight="1"/>
     <row r="28" ht="22" customHeight="1">
@@ -7558,6 +7774,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AA29" s="34" t="n">
+        <v>369.99</v>
+      </c>
     </row>
     <row r="30" ht="18" customHeight="1">
       <c r="B30" s="15" t="n">
@@ -7657,6 +7876,9 @@
       <c r="Z30" s="34" t="n">
         <v>579.99</v>
       </c>
+      <c r="AA30" s="34" t="n">
+        <v>579.99</v>
+      </c>
     </row>
     <row r="31" ht="18" customHeight="1">
       <c r="B31" s="6" t="n">
@@ -7758,6 +7980,11 @@
       <c r="Z31" s="34" t="n">
         <v>746.99</v>
       </c>
+      <c r="AA31" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="18" customHeight="1">
       <c r="B32" s="15" t="n">
@@ -7857,6 +8084,9 @@
       <c r="Z32" s="34" t="n">
         <v>759.99</v>
       </c>
+      <c r="AA32" s="34" t="n">
+        <v>759.99</v>
+      </c>
     </row>
     <row r="33" ht="18" customHeight="1">
       <c r="B33" s="6" t="n">
@@ -7958,6 +8188,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AA33" s="34" t="n">
+        <v>799.99</v>
+      </c>
     </row>
     <row r="34" ht="18" customHeight="1">
       <c r="B34" s="15" t="n">
@@ -8057,6 +8290,9 @@
       <c r="Z34" s="34" t="n">
         <v>1274.99</v>
       </c>
+      <c r="AA34" s="34" t="n">
+        <v>1274.99</v>
+      </c>
     </row>
     <row r="35" ht="18" customHeight="1">
       <c r="B35" s="6" t="n">
@@ -8156,6 +8392,9 @@
       <c r="Z35" s="34" t="n">
         <v>1799.99</v>
       </c>
+      <c r="AA35" s="34" t="n">
+        <v>1799.99</v>
+      </c>
     </row>
     <row r="36" ht="18" customHeight="1">
       <c r="B36" s="15" t="n">
@@ -8253,6 +8492,9 @@
       <c r="Z36" s="34" t="n">
         <v>1975.99</v>
       </c>
+      <c r="AA36" s="34" t="n">
+        <v>1975.99</v>
+      </c>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="B37" s="6" t="n">
@@ -8354,6 +8596,9 @@
       <c r="Z37" s="34" t="n">
         <v>2699.99</v>
       </c>
+      <c r="AA37" s="34" t="n">
+        <v>2699.99</v>
+      </c>
     </row>
     <row r="38" ht="5" customHeight="1"/>
     <row r="39" ht="22" customHeight="1">
@@ -8461,6 +8706,9 @@
       <c r="Z40" s="34" t="n">
         <v>740.99</v>
       </c>
+      <c r="AA40" s="34" t="n">
+        <v>740.99</v>
+      </c>
     </row>
     <row r="41" ht="18" customHeight="1">
       <c r="B41" s="6" t="n">
@@ -8562,6 +8810,11 @@
       <c r="Z41" s="34" t="n">
         <v>649.99</v>
       </c>
+      <c r="AA41" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="18" customHeight="1">
       <c r="B42" s="15" t="n">
@@ -8663,6 +8916,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AA42" s="34" t="n">
+        <v>799.99</v>
+      </c>
     </row>
     <row r="43" ht="18" customHeight="1">
       <c r="B43" s="6" t="n">
@@ -8766,6 +9022,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AA43" s="34" t="n">
+        <v>949.99</v>
+      </c>
     </row>
     <row r="44" ht="18" customHeight="1">
       <c r="B44" s="15" t="n">
@@ -8859,6 +9118,11 @@
       <c r="Z44" s="34" t="n">
         <v>1139.99</v>
       </c>
+      <c r="AA44" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="45" ht="18" customHeight="1">
       <c r="B45" s="6" t="n">
@@ -8954,6 +9218,9 @@
       <c r="Z45" s="34" t="n">
         <v>1529.99</v>
       </c>
+      <c r="AA45" s="34" t="n">
+        <v>1529.99</v>
+      </c>
     </row>
     <row r="46" ht="18" customHeight="1">
       <c r="B46" s="15" t="n">
@@ -9061,6 +9328,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AA46" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="47" ht="18" customHeight="1">
       <c r="B47" s="6" t="n">
@@ -9160,6 +9432,9 @@
       <c r="Z47" s="34" t="n">
         <v>2999.99</v>
       </c>
+      <c r="AA47" s="34" t="n">
+        <v>2999.99</v>
+      </c>
     </row>
     <row r="48" ht="18" customHeight="1">
       <c r="B48" s="15" t="n">
@@ -9261,6 +9536,9 @@
       <c r="Z48" s="34" t="n">
         <v>3499.99</v>
       </c>
+      <c r="AA48" s="34" t="n">
+        <v>3499.99</v>
+      </c>
     </row>
     <row r="49" ht="5" customHeight="1"/>
     <row r="50" ht="22" customHeight="1">
@@ -9364,6 +9642,11 @@
       <c r="Z51" s="34" t="n">
         <v>798.99</v>
       </c>
+      <c r="AA51" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="52" ht="18" customHeight="1">
       <c r="B52" s="15" t="n">
@@ -9459,6 +9742,11 @@
       <c r="Z52" s="34" t="n">
         <v>798.99</v>
       </c>
+      <c r="AA52" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="53" ht="18" customHeight="1">
       <c r="B53" s="6" t="n">
@@ -9558,6 +9846,9 @@
       <c r="Z53" s="34" t="n">
         <v>1499.99</v>
       </c>
+      <c r="AA53" s="34" t="n">
+        <v>1499.99</v>
+      </c>
     </row>
     <row r="54" ht="18" customHeight="1">
       <c r="B54" s="15" t="n">
@@ -9653,6 +9944,9 @@
       <c r="Z54" s="34" t="n">
         <v>899.99</v>
       </c>
+      <c r="AA54" s="34" t="n">
+        <v>899.99</v>
+      </c>
     </row>
     <row r="55" ht="18" customHeight="1">
       <c r="B55" s="6" t="n">
@@ -9752,6 +10046,9 @@
       <c r="Z55" s="34" t="n">
         <v>1397.99</v>
       </c>
+      <c r="AA55" s="34" t="n">
+        <v>1397.99</v>
+      </c>
     </row>
     <row r="56" ht="18" customHeight="1">
       <c r="B56" s="15" t="n">
@@ -9851,6 +10148,9 @@
       <c r="Z56" s="34" t="n">
         <v>2799.99</v>
       </c>
+      <c r="AA56" s="34" t="n">
+        <v>2799.99</v>
+      </c>
     </row>
     <row r="57" ht="18" customHeight="1">
       <c r="B57" s="6" t="n">
@@ -9948,6 +10248,11 @@
       <c r="Z57" s="34" t="n">
         <v>3199.99</v>
       </c>
+      <c r="AA57" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="58" ht="18" customHeight="1">
       <c r="B58" s="26" t="n">
@@ -10109,6 +10414,11 @@
       <c r="Z61" s="34" t="n">
         <v>999.99</v>
       </c>
+      <c r="AA61" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="62" ht="18" customHeight="1">
       <c r="B62" s="15" t="n">
@@ -10266,6 +10576,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AA63" s="34" t="n">
+        <v>1658.99</v>
+      </c>
     </row>
     <row r="64" ht="18" customHeight="1">
       <c r="B64" s="15" t="n">
@@ -10363,6 +10676,9 @@
       <c r="Z64" s="34" t="n">
         <v>2549.99</v>
       </c>
+      <c r="AA64" s="34" t="n">
+        <v>2549.99</v>
+      </c>
     </row>
     <row r="65" ht="18" customHeight="1">
       <c r="B65" s="26" t="n">
@@ -10634,6 +10950,9 @@
         <v>1899.99</v>
       </c>
       <c r="Z70" s="34" t="n">
+        <v>1899.99</v>
+      </c>
+      <c r="AA70" s="34" t="n">
         <v>1899.99</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Price check — 03/23/2026
</commit_message>
<xml_diff>
--- a/PriceBook_Combined_Final.xlsx
+++ b/PriceBook_Combined_Final.xlsx
@@ -709,7 +709,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:AA67"/>
+  <dimension ref="B1:AB67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -739,6 +739,7 @@
     <col width="12" customWidth="1" min="25" max="25"/>
     <col width="12" customWidth="1" min="26" max="26"/>
     <col width="12" customWidth="1" min="27" max="27"/>
+    <col width="12" customWidth="1" min="28" max="28"/>
   </cols>
   <sheetData>
     <row r="1" ht="8" customHeight="1"/>
@@ -888,6 +889,11 @@
           <t>3/22</t>
         </is>
       </c>
+      <c r="AB5" s="33" t="inlineStr">
+        <is>
+          <t>3/23</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="22" customHeight="1">
       <c r="B6" s="5" t="inlineStr">
@@ -991,6 +997,9 @@
       <c r="AA7" s="34" t="n">
         <v>449.99</v>
       </c>
+      <c r="AB7" s="34" t="n">
+        <v>449.99</v>
+      </c>
     </row>
     <row r="8" ht="18" customHeight="1">
       <c r="B8" s="15" t="n">
@@ -1107,6 +1116,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AB8" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="18" customHeight="1">
       <c r="B9" s="6" t="n">
@@ -1223,6 +1237,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AB9" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="18" customHeight="1">
       <c r="B10" s="15" t="n">
@@ -1319,6 +1338,9 @@
       <c r="AA10" s="34" t="n">
         <v>449.99</v>
       </c>
+      <c r="AB10" s="34" t="n">
+        <v>449.99</v>
+      </c>
     </row>
     <row r="11" ht="18" customHeight="1">
       <c r="B11" s="6" t="n">
@@ -1435,6 +1457,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AB11" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="18" customHeight="1">
       <c r="B12" s="15" t="n">
@@ -1535,6 +1562,9 @@
       <c r="AA12" s="34" t="n">
         <v>729.99</v>
       </c>
+      <c r="AB12" s="34" t="n">
+        <v>729.99</v>
+      </c>
     </row>
     <row r="13" ht="5" customHeight="1"/>
     <row r="14" ht="22" customHeight="1">
@@ -1647,6 +1677,11 @@
       <c r="AA15" s="34" t="n">
         <v>599.99</v>
       </c>
+      <c r="AB15" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="18" customHeight="1">
       <c r="B16" s="15" t="n">
@@ -1749,6 +1784,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AB16" s="13" t="n">
+        <v>659.99</v>
+      </c>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="B17" s="6" t="n">
@@ -1865,6 +1903,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AB17" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="B18" s="15" t="n">
@@ -2023,6 +2066,9 @@
       <c r="AA19" s="34" t="n">
         <v>2199.99</v>
       </c>
+      <c r="AB19" s="34" t="n">
+        <v>2199.99</v>
+      </c>
     </row>
     <row r="20" ht="5" customHeight="1"/>
     <row r="21" ht="22" customHeight="1">
@@ -2133,6 +2179,11 @@
       <c r="AA22" s="34" t="n">
         <v>1098.99</v>
       </c>
+      <c r="AB22" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="B23" s="6" t="n">
@@ -2239,6 +2290,9 @@
       <c r="AA23" s="34" t="n">
         <v>1199.99</v>
       </c>
+      <c r="AB23" s="34" t="n">
+        <v>1199.99</v>
+      </c>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="B24" s="15" t="n">
@@ -2345,6 +2399,9 @@
       <c r="AA24" s="34" t="n">
         <v>1199.99</v>
       </c>
+      <c r="AB24" s="34" t="n">
+        <v>1199.99</v>
+      </c>
     </row>
     <row r="25" ht="18" customHeight="1">
       <c r="B25" s="6" t="n">
@@ -2509,6 +2566,9 @@
       <c r="AA26" s="34" t="n">
         <v>1599.99</v>
       </c>
+      <c r="AB26" s="34" t="n">
+        <v>1599.99</v>
+      </c>
     </row>
     <row r="27" ht="18" customHeight="1">
       <c r="B27" s="6" t="n">
@@ -2611,6 +2671,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AB27" s="34" t="n">
+        <v>1799.99</v>
+      </c>
     </row>
     <row r="28" ht="18" customHeight="1">
       <c r="B28" s="15" t="n">
@@ -2709,6 +2772,11 @@
       <c r="AA28" s="34" t="n">
         <v>1479.99</v>
       </c>
+      <c r="AB28" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="18" customHeight="1">
       <c r="B29" s="6" t="n">
@@ -2811,6 +2879,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AB29" s="34" t="n">
+        <v>1799.99</v>
+      </c>
     </row>
     <row r="30" ht="18" customHeight="1">
       <c r="B30" s="15" t="n">
@@ -2913,6 +2984,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AB30" s="34" t="n">
+        <v>1799.99</v>
+      </c>
     </row>
     <row r="31" ht="5" customHeight="1"/>
     <row r="32" ht="22" customHeight="1">
@@ -3023,6 +3097,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AB33" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="18" customHeight="1">
       <c r="B34" s="15" t="n">
@@ -3125,6 +3204,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AB34" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="18" customHeight="1">
       <c r="B35" s="6" t="n">
@@ -3233,6 +3317,9 @@
       <c r="AA35" s="34" t="n">
         <v>1599.99</v>
       </c>
+      <c r="AB35" s="34" t="n">
+        <v>1599.99</v>
+      </c>
     </row>
     <row r="36" ht="18" customHeight="1">
       <c r="B36" s="15" t="n">
@@ -3337,6 +3424,9 @@
       <c r="AA36" s="34" t="n">
         <v>1699.99</v>
       </c>
+      <c r="AB36" s="34" t="n">
+        <v>1699.99</v>
+      </c>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="B37" s="6" t="n">
@@ -3439,6 +3529,9 @@
       <c r="AA37" s="34" t="n">
         <v>2499.99</v>
       </c>
+      <c r="AB37" s="34" t="n">
+        <v>2499.99</v>
+      </c>
     </row>
     <row r="38" ht="18" customHeight="1">
       <c r="B38" s="15" t="n">
@@ -3541,6 +3634,9 @@
       <c r="AA38" s="34" t="n">
         <v>2898.99</v>
       </c>
+      <c r="AB38" s="34" t="n">
+        <v>2898.99</v>
+      </c>
     </row>
     <row r="39" ht="18" customHeight="1">
       <c r="B39" s="6" t="n">
@@ -3643,6 +3739,9 @@
       <c r="AA39" s="34" t="n">
         <v>2499.99</v>
       </c>
+      <c r="AB39" s="34" t="n">
+        <v>2499.99</v>
+      </c>
     </row>
     <row r="40" ht="18" customHeight="1">
       <c r="B40" s="15" t="n">
@@ -3745,6 +3844,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AB40" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="18" customHeight="1">
       <c r="B41" s="6" t="n">
@@ -3845,6 +3949,11 @@
       <c r="AA41" s="34" t="n">
         <v>1749.99</v>
       </c>
+      <c r="AB41" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="18" customHeight="1">
       <c r="B42" s="15" t="n">
@@ -3955,6 +4064,9 @@
       <c r="AA42" s="34" t="n">
         <v>1899.99</v>
       </c>
+      <c r="AB42" s="34" t="n">
+        <v>1899.99</v>
+      </c>
     </row>
     <row r="43" ht="18" customHeight="1">
       <c r="B43" s="6" t="n">
@@ -4111,6 +4223,9 @@
       <c r="AA44" s="34" t="n">
         <v>3599.99</v>
       </c>
+      <c r="AB44" s="34" t="n">
+        <v>3599.99</v>
+      </c>
     </row>
     <row r="45" ht="5" customHeight="1"/>
     <row r="46" ht="22" customHeight="1">
@@ -4229,6 +4344,9 @@
       <c r="AA47" s="34" t="n">
         <v>1899.99</v>
       </c>
+      <c r="AB47" s="34" t="n">
+        <v>1899.99</v>
+      </c>
     </row>
     <row r="48" ht="18" customHeight="1">
       <c r="B48" s="15" t="n">
@@ -4337,6 +4455,9 @@
       <c r="AA48" s="34" t="n">
         <v>1599.99</v>
       </c>
+      <c r="AB48" s="34" t="n">
+        <v>1599.99</v>
+      </c>
     </row>
     <row r="49" ht="18" customHeight="1">
       <c r="B49" s="6" t="n">
@@ -4441,6 +4562,9 @@
       <c r="AA49" s="34" t="n">
         <v>1849.99</v>
       </c>
+      <c r="AB49" s="34" t="n">
+        <v>1849.99</v>
+      </c>
     </row>
     <row r="50" ht="18" customHeight="1">
       <c r="B50" s="15" t="n">
@@ -4541,6 +4665,9 @@
       <c r="AA50" s="34" t="n">
         <v>2599.99</v>
       </c>
+      <c r="AB50" s="34" t="n">
+        <v>2599.99</v>
+      </c>
     </row>
     <row r="51" ht="18" customHeight="1">
       <c r="B51" s="6" t="n">
@@ -4697,6 +4824,9 @@
       <c r="AA52" s="34" t="n">
         <v>2599.99</v>
       </c>
+      <c r="AB52" s="34" t="n">
+        <v>2599.99</v>
+      </c>
     </row>
     <row r="53" ht="18" customHeight="1">
       <c r="B53" s="6" t="n">
@@ -4797,6 +4927,9 @@
       <c r="AA53" s="34" t="n">
         <v>3499.99</v>
       </c>
+      <c r="AB53" s="34" t="n">
+        <v>3499.99</v>
+      </c>
     </row>
     <row r="54" ht="5" customHeight="1"/>
     <row r="55" ht="22" customHeight="1">
@@ -4905,6 +5038,9 @@
       <c r="AA56" s="34" t="n">
         <v>3599.99</v>
       </c>
+      <c r="AB56" s="34" t="n">
+        <v>3599.99</v>
+      </c>
     </row>
     <row r="57" ht="18" customHeight="1">
       <c r="B57" s="26" t="n">
@@ -5185,6 +5321,9 @@
       <c r="AA62" s="34" t="n">
         <v>127.99</v>
       </c>
+      <c r="AB62" s="34" t="n">
+        <v>127.99</v>
+      </c>
     </row>
     <row r="63" ht="18" customHeight="1">
       <c r="B63" s="6" t="n">
@@ -5295,6 +5434,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AB63" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="64" ht="18" customHeight="1">
       <c r="B64" s="15" t="n">
@@ -5400,6 +5544,9 @@
       </c>
       <c r="AA64" s="36" t="n">
         <v>499.99</v>
+      </c>
+      <c r="AB64" s="36" t="n">
+        <v>479.99</v>
       </c>
     </row>
     <row r="65" ht="18" customHeight="1">
@@ -5633,7 +5780,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:AA70"/>
+  <dimension ref="B1:AB70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -5663,6 +5810,7 @@
     <col width="12" customWidth="1" min="25" max="25"/>
     <col width="12" customWidth="1" min="26" max="26"/>
     <col width="12" customWidth="1" min="27" max="27"/>
+    <col width="12" customWidth="1" min="28" max="28"/>
   </cols>
   <sheetData>
     <row r="1" ht="8" customHeight="1"/>
@@ -5812,6 +5960,11 @@
           <t>3/22</t>
         </is>
       </c>
+      <c r="AB5" s="33" t="inlineStr">
+        <is>
+          <t>3/23</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="22" customHeight="1">
       <c r="B6" s="5" t="inlineStr">
@@ -5923,6 +6076,9 @@
       <c r="AA7" s="34" t="n">
         <v>89.98999999999999</v>
       </c>
+      <c r="AB7" s="34" t="n">
+        <v>89.98999999999999</v>
+      </c>
     </row>
     <row r="8" ht="18" customHeight="1">
       <c r="B8" s="15" t="n">
@@ -6025,6 +6181,9 @@
       <c r="AA8" s="34" t="n">
         <v>194.99</v>
       </c>
+      <c r="AB8" s="34" t="n">
+        <v>194.99</v>
+      </c>
     </row>
     <row r="9" ht="18" customHeight="1">
       <c r="B9" s="6" t="n">
@@ -6139,6 +6298,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AB9" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="18" customHeight="1">
       <c r="B10" s="15" t="n">
@@ -6291,6 +6455,9 @@
       <c r="AA11" s="34" t="n">
         <v>219.99</v>
       </c>
+      <c r="AB11" s="34" t="n">
+        <v>219.99</v>
+      </c>
     </row>
     <row r="12" ht="18" customHeight="1">
       <c r="B12" s="15" t="n">
@@ -6397,6 +6564,9 @@
       <c r="AA12" s="34" t="n">
         <v>349.99</v>
       </c>
+      <c r="AB12" s="34" t="n">
+        <v>349.99</v>
+      </c>
     </row>
     <row r="13" ht="18" customHeight="1">
       <c r="B13" s="6" t="n">
@@ -6509,6 +6679,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AB13" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="5" customHeight="1"/>
     <row r="15" ht="22" customHeight="1">
@@ -6631,6 +6806,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AB16" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="B17" s="6" t="n">
@@ -6727,6 +6907,11 @@
       <c r="AA17" s="34" t="n">
         <v>279.99</v>
       </c>
+      <c r="AB17" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="B18" s="15" t="n">
@@ -6831,6 +7016,9 @@
       <c r="AA18" s="34" t="n">
         <v>399.99</v>
       </c>
+      <c r="AB18" s="34" t="n">
+        <v>399.99</v>
+      </c>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="B19" s="6" t="n">
@@ -6933,6 +7121,11 @@
       <c r="AA19" s="34" t="n">
         <v>249.99</v>
       </c>
+      <c r="AB19" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="B20" s="15" t="n">
@@ -7035,6 +7228,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AB20" s="34" t="n">
+        <v>427.99</v>
+      </c>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="B21" s="6" t="n">
@@ -7131,6 +7327,9 @@
       <c r="AA21" s="34" t="n">
         <v>478.99</v>
       </c>
+      <c r="AB21" s="34" t="n">
+        <v>478.99</v>
+      </c>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="B22" s="15" t="n">
@@ -7241,6 +7440,9 @@
       <c r="AA22" s="34" t="n">
         <v>599.99</v>
       </c>
+      <c r="AB22" s="34" t="n">
+        <v>599.99</v>
+      </c>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="B23" s="6" t="n">
@@ -7343,6 +7545,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AB23" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="B24" s="15" t="n">
@@ -7455,6 +7662,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AB24" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="18" customHeight="1">
       <c r="B25" s="6" t="n">
@@ -7561,6 +7773,9 @@
       <c r="AA25" s="34" t="n">
         <v>1199.99</v>
       </c>
+      <c r="AB25" s="34" t="n">
+        <v>1199.99</v>
+      </c>
     </row>
     <row r="26" ht="18" customHeight="1">
       <c r="B26" s="15" t="n">
@@ -7663,6 +7878,9 @@
       <c r="AA26" s="34" t="n">
         <v>1274.99</v>
       </c>
+      <c r="AB26" s="34" t="n">
+        <v>1274.99</v>
+      </c>
     </row>
     <row r="27" ht="5" customHeight="1"/>
     <row r="28" ht="22" customHeight="1">
@@ -7777,6 +7995,11 @@
       <c r="AA29" s="34" t="n">
         <v>369.99</v>
       </c>
+      <c r="AB29" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="18" customHeight="1">
       <c r="B30" s="15" t="n">
@@ -7879,6 +8102,9 @@
       <c r="AA30" s="34" t="n">
         <v>579.99</v>
       </c>
+      <c r="AB30" s="34" t="n">
+        <v>579.99</v>
+      </c>
     </row>
     <row r="31" ht="18" customHeight="1">
       <c r="B31" s="6" t="n">
@@ -7985,6 +8211,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AB31" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="18" customHeight="1">
       <c r="B32" s="15" t="n">
@@ -8087,6 +8318,9 @@
       <c r="AA32" s="34" t="n">
         <v>759.99</v>
       </c>
+      <c r="AB32" s="34" t="n">
+        <v>759.99</v>
+      </c>
     </row>
     <row r="33" ht="18" customHeight="1">
       <c r="B33" s="6" t="n">
@@ -8191,6 +8425,9 @@
       <c r="AA33" s="34" t="n">
         <v>799.99</v>
       </c>
+      <c r="AB33" s="34" t="n">
+        <v>799.99</v>
+      </c>
     </row>
     <row r="34" ht="18" customHeight="1">
       <c r="B34" s="15" t="n">
@@ -8293,6 +8530,9 @@
       <c r="AA34" s="34" t="n">
         <v>1274.99</v>
       </c>
+      <c r="AB34" s="34" t="n">
+        <v>1274.99</v>
+      </c>
     </row>
     <row r="35" ht="18" customHeight="1">
       <c r="B35" s="6" t="n">
@@ -8395,6 +8635,11 @@
       <c r="AA35" s="34" t="n">
         <v>1799.99</v>
       </c>
+      <c r="AB35" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="18" customHeight="1">
       <c r="B36" s="15" t="n">
@@ -8495,6 +8740,9 @@
       <c r="AA36" s="34" t="n">
         <v>1975.99</v>
       </c>
+      <c r="AB36" s="34" t="n">
+        <v>1975.99</v>
+      </c>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="B37" s="6" t="n">
@@ -8599,6 +8847,11 @@
       <c r="AA37" s="34" t="n">
         <v>2699.99</v>
       </c>
+      <c r="AB37" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="5" customHeight="1"/>
     <row r="39" ht="22" customHeight="1">
@@ -8709,6 +8962,9 @@
       <c r="AA40" s="34" t="n">
         <v>740.99</v>
       </c>
+      <c r="AB40" s="34" t="n">
+        <v>740.99</v>
+      </c>
     </row>
     <row r="41" ht="18" customHeight="1">
       <c r="B41" s="6" t="n">
@@ -8815,6 +9071,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AB41" s="13" t="n">
+        <v>599.99</v>
+      </c>
     </row>
     <row r="42" ht="18" customHeight="1">
       <c r="B42" s="15" t="n">
@@ -8919,6 +9178,9 @@
       <c r="AA42" s="34" t="n">
         <v>799.99</v>
       </c>
+      <c r="AB42" s="34" t="n">
+        <v>799.99</v>
+      </c>
     </row>
     <row r="43" ht="18" customHeight="1">
       <c r="B43" s="6" t="n">
@@ -9025,6 +9287,11 @@
       <c r="AA43" s="34" t="n">
         <v>949.99</v>
       </c>
+      <c r="AB43" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="44" ht="18" customHeight="1">
       <c r="B44" s="15" t="n">
@@ -9123,6 +9390,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AB44" s="34" t="n">
+        <v>1139.99</v>
+      </c>
     </row>
     <row r="45" ht="18" customHeight="1">
       <c r="B45" s="6" t="n">
@@ -9221,6 +9491,9 @@
       <c r="AA45" s="34" t="n">
         <v>1529.99</v>
       </c>
+      <c r="AB45" s="34" t="n">
+        <v>1529.99</v>
+      </c>
     </row>
     <row r="46" ht="18" customHeight="1">
       <c r="B46" s="15" t="n">
@@ -9333,6 +9606,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AB46" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="47" ht="18" customHeight="1">
       <c r="B47" s="6" t="n">
@@ -9435,6 +9713,9 @@
       <c r="AA47" s="34" t="n">
         <v>2999.99</v>
       </c>
+      <c r="AB47" s="34" t="n">
+        <v>2999.99</v>
+      </c>
     </row>
     <row r="48" ht="18" customHeight="1">
       <c r="B48" s="15" t="n">
@@ -9539,6 +9820,11 @@
       <c r="AA48" s="34" t="n">
         <v>3499.99</v>
       </c>
+      <c r="AB48" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="49" ht="5" customHeight="1"/>
     <row r="50" ht="22" customHeight="1">
@@ -9647,6 +9933,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AB51" s="34" t="n">
+        <v>798.99</v>
+      </c>
     </row>
     <row r="52" ht="18" customHeight="1">
       <c r="B52" s="15" t="n">
@@ -9747,6 +10036,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AB52" s="34" t="n">
+        <v>798.99</v>
+      </c>
     </row>
     <row r="53" ht="18" customHeight="1">
       <c r="B53" s="6" t="n">
@@ -9849,6 +10141,9 @@
       <c r="AA53" s="34" t="n">
         <v>1499.99</v>
       </c>
+      <c r="AB53" s="34" t="n">
+        <v>1499.99</v>
+      </c>
     </row>
     <row r="54" ht="18" customHeight="1">
       <c r="B54" s="15" t="n">
@@ -9947,6 +10242,9 @@
       <c r="AA54" s="34" t="n">
         <v>899.99</v>
       </c>
+      <c r="AB54" s="34" t="n">
+        <v>899.99</v>
+      </c>
     </row>
     <row r="55" ht="18" customHeight="1">
       <c r="B55" s="6" t="n">
@@ -10049,6 +10347,9 @@
       <c r="AA55" s="34" t="n">
         <v>1397.99</v>
       </c>
+      <c r="AB55" s="13" t="n">
+        <v>1299.99</v>
+      </c>
     </row>
     <row r="56" ht="18" customHeight="1">
       <c r="B56" s="15" t="n">
@@ -10151,6 +10452,9 @@
       <c r="AA56" s="34" t="n">
         <v>2799.99</v>
       </c>
+      <c r="AB56" s="34" t="n">
+        <v>2799.99</v>
+      </c>
     </row>
     <row r="57" ht="18" customHeight="1">
       <c r="B57" s="6" t="n">
@@ -10253,6 +10557,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AB57" s="34" t="n">
+        <v>3199.99</v>
+      </c>
     </row>
     <row r="58" ht="18" customHeight="1">
       <c r="B58" s="26" t="n">
@@ -10419,6 +10726,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AB61" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="62" ht="18" customHeight="1">
       <c r="B62" s="15" t="n">
@@ -10579,6 +10891,11 @@
       <c r="AA63" s="34" t="n">
         <v>1658.99</v>
       </c>
+      <c r="AB63" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="64" ht="18" customHeight="1">
       <c r="B64" s="15" t="n">
@@ -10679,6 +10996,9 @@
       <c r="AA64" s="34" t="n">
         <v>2549.99</v>
       </c>
+      <c r="AB64" s="34" t="n">
+        <v>2549.99</v>
+      </c>
     </row>
     <row r="65" ht="18" customHeight="1">
       <c r="B65" s="26" t="n">
@@ -10954,6 +11274,11 @@
       </c>
       <c r="AA70" s="34" t="n">
         <v>1899.99</v>
+      </c>
+      <c r="AB70" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Price check — 03/24/2026
</commit_message>
<xml_diff>
--- a/PriceBook_Combined_Final.xlsx
+++ b/PriceBook_Combined_Final.xlsx
@@ -709,7 +709,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:AB67"/>
+  <dimension ref="B1:AC67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -740,6 +740,7 @@
     <col width="12" customWidth="1" min="26" max="26"/>
     <col width="12" customWidth="1" min="27" max="27"/>
     <col width="12" customWidth="1" min="28" max="28"/>
+    <col width="12" customWidth="1" min="29" max="29"/>
   </cols>
   <sheetData>
     <row r="1" ht="8" customHeight="1"/>
@@ -894,6 +895,11 @@
           <t>3/23</t>
         </is>
       </c>
+      <c r="AC5" s="33" t="inlineStr">
+        <is>
+          <t>3/24</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="22" customHeight="1">
       <c r="B6" s="5" t="inlineStr">
@@ -1000,6 +1006,9 @@
       <c r="AB7" s="34" t="n">
         <v>449.99</v>
       </c>
+      <c r="AC7" s="34" t="n">
+        <v>449.99</v>
+      </c>
     </row>
     <row r="8" ht="18" customHeight="1">
       <c r="B8" s="15" t="n">
@@ -1121,6 +1130,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AC8" s="34" t="n">
+        <v>659.99</v>
+      </c>
     </row>
     <row r="9" ht="18" customHeight="1">
       <c r="B9" s="6" t="n">
@@ -1242,6 +1254,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AC9" s="34" t="n">
+        <v>659.99</v>
+      </c>
     </row>
     <row r="10" ht="18" customHeight="1">
       <c r="B10" s="15" t="n">
@@ -1341,6 +1356,9 @@
       <c r="AB10" s="34" t="n">
         <v>449.99</v>
       </c>
+      <c r="AC10" s="34" t="n">
+        <v>449.99</v>
+      </c>
     </row>
     <row r="11" ht="18" customHeight="1">
       <c r="B11" s="6" t="n">
@@ -1462,6 +1480,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AC11" s="34" t="n">
+        <v>659.99</v>
+      </c>
     </row>
     <row r="12" ht="18" customHeight="1">
       <c r="B12" s="15" t="n">
@@ -1565,6 +1586,9 @@
       <c r="AB12" s="34" t="n">
         <v>729.99</v>
       </c>
+      <c r="AC12" s="34" t="n">
+        <v>729.99</v>
+      </c>
     </row>
     <row r="13" ht="5" customHeight="1"/>
     <row r="14" ht="22" customHeight="1">
@@ -1682,6 +1706,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AC15" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="18" customHeight="1">
       <c r="B16" s="15" t="n">
@@ -1787,6 +1816,9 @@
       <c r="AB16" s="13" t="n">
         <v>659.99</v>
       </c>
+      <c r="AC16" s="13" t="n">
+        <v>659.99</v>
+      </c>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="B17" s="6" t="n">
@@ -1908,6 +1940,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AC17" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="B18" s="15" t="n">
@@ -2069,6 +2106,9 @@
       <c r="AB19" s="34" t="n">
         <v>2199.99</v>
       </c>
+      <c r="AC19" s="34" t="n">
+        <v>2199.99</v>
+      </c>
     </row>
     <row r="20" ht="5" customHeight="1"/>
     <row r="21" ht="22" customHeight="1">
@@ -2184,6 +2224,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AC22" s="34" t="n">
+        <v>1098.99</v>
+      </c>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="B23" s="6" t="n">
@@ -2293,6 +2336,9 @@
       <c r="AB23" s="34" t="n">
         <v>1199.99</v>
       </c>
+      <c r="AC23" s="34" t="n">
+        <v>1199.99</v>
+      </c>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="B24" s="15" t="n">
@@ -2402,6 +2448,9 @@
       <c r="AB24" s="34" t="n">
         <v>1199.99</v>
       </c>
+      <c r="AC24" s="34" t="n">
+        <v>1199.99</v>
+      </c>
     </row>
     <row r="25" ht="18" customHeight="1">
       <c r="B25" s="6" t="n">
@@ -2569,6 +2618,9 @@
       <c r="AB26" s="34" t="n">
         <v>1599.99</v>
       </c>
+      <c r="AC26" s="34" t="n">
+        <v>1599.99</v>
+      </c>
     </row>
     <row r="27" ht="18" customHeight="1">
       <c r="B27" s="6" t="n">
@@ -2674,6 +2726,11 @@
       <c r="AB27" s="34" t="n">
         <v>1799.99</v>
       </c>
+      <c r="AC27" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="18" customHeight="1">
       <c r="B28" s="15" t="n">
@@ -2777,6 +2834,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AC28" s="34" t="n">
+        <v>1479.99</v>
+      </c>
     </row>
     <row r="29" ht="18" customHeight="1">
       <c r="B29" s="6" t="n">
@@ -2882,6 +2942,11 @@
       <c r="AB29" s="34" t="n">
         <v>1799.99</v>
       </c>
+      <c r="AC29" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="18" customHeight="1">
       <c r="B30" s="15" t="n">
@@ -2987,6 +3052,11 @@
       <c r="AB30" s="34" t="n">
         <v>1799.99</v>
       </c>
+      <c r="AC30" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="5" customHeight="1"/>
     <row r="32" ht="22" customHeight="1">
@@ -3102,6 +3172,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AC33" s="34" t="n">
+        <v>1029.99</v>
+      </c>
     </row>
     <row r="34" ht="18" customHeight="1">
       <c r="B34" s="15" t="n">
@@ -3209,6 +3282,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AC34" s="34" t="n">
+        <v>1029.99</v>
+      </c>
     </row>
     <row r="35" ht="18" customHeight="1">
       <c r="B35" s="6" t="n">
@@ -3320,6 +3396,9 @@
       <c r="AB35" s="34" t="n">
         <v>1599.99</v>
       </c>
+      <c r="AC35" s="34" t="n">
+        <v>1599.99</v>
+      </c>
     </row>
     <row r="36" ht="18" customHeight="1">
       <c r="B36" s="15" t="n">
@@ -3427,6 +3506,11 @@
       <c r="AB36" s="34" t="n">
         <v>1699.99</v>
       </c>
+      <c r="AC36" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="B37" s="6" t="n">
@@ -3532,6 +3616,9 @@
       <c r="AB37" s="34" t="n">
         <v>2499.99</v>
       </c>
+      <c r="AC37" s="34" t="n">
+        <v>2499.99</v>
+      </c>
     </row>
     <row r="38" ht="18" customHeight="1">
       <c r="B38" s="15" t="n">
@@ -3637,6 +3724,11 @@
       <c r="AB38" s="34" t="n">
         <v>2898.99</v>
       </c>
+      <c r="AC38" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="18" customHeight="1">
       <c r="B39" s="6" t="n">
@@ -3742,6 +3834,9 @@
       <c r="AB39" s="34" t="n">
         <v>2499.99</v>
       </c>
+      <c r="AC39" s="34" t="n">
+        <v>2499.99</v>
+      </c>
     </row>
     <row r="40" ht="18" customHeight="1">
       <c r="B40" s="15" t="n">
@@ -3849,6 +3944,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AC40" s="34" t="n">
+        <v>1029.99</v>
+      </c>
     </row>
     <row r="41" ht="18" customHeight="1">
       <c r="B41" s="6" t="n">
@@ -3954,6 +4052,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AC41" s="34" t="n">
+        <v>1749.99</v>
+      </c>
     </row>
     <row r="42" ht="18" customHeight="1">
       <c r="B42" s="15" t="n">
@@ -4067,6 +4168,11 @@
       <c r="AB42" s="34" t="n">
         <v>1899.99</v>
       </c>
+      <c r="AC42" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="43" ht="18" customHeight="1">
       <c r="B43" s="6" t="n">
@@ -4226,6 +4332,11 @@
       <c r="AB44" s="34" t="n">
         <v>3599.99</v>
       </c>
+      <c r="AC44" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="45" ht="5" customHeight="1"/>
     <row r="46" ht="22" customHeight="1">
@@ -4347,6 +4458,11 @@
       <c r="AB47" s="34" t="n">
         <v>1899.99</v>
       </c>
+      <c r="AC47" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="48" ht="18" customHeight="1">
       <c r="B48" s="15" t="n">
@@ -4458,6 +4574,9 @@
       <c r="AB48" s="34" t="n">
         <v>1599.99</v>
       </c>
+      <c r="AC48" s="34" t="n">
+        <v>1599.99</v>
+      </c>
     </row>
     <row r="49" ht="18" customHeight="1">
       <c r="B49" s="6" t="n">
@@ -4565,6 +4684,11 @@
       <c r="AB49" s="34" t="n">
         <v>1849.99</v>
       </c>
+      <c r="AC49" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="50" ht="18" customHeight="1">
       <c r="B50" s="15" t="n">
@@ -4668,6 +4792,9 @@
       <c r="AB50" s="34" t="n">
         <v>2599.99</v>
       </c>
+      <c r="AC50" s="34" t="n">
+        <v>2599.99</v>
+      </c>
     </row>
     <row r="51" ht="18" customHeight="1">
       <c r="B51" s="6" t="n">
@@ -4827,6 +4954,9 @@
       <c r="AB52" s="34" t="n">
         <v>2599.99</v>
       </c>
+      <c r="AC52" s="34" t="n">
+        <v>2599.99</v>
+      </c>
     </row>
     <row r="53" ht="18" customHeight="1">
       <c r="B53" s="6" t="n">
@@ -4930,6 +5060,9 @@
       <c r="AB53" s="34" t="n">
         <v>3499.99</v>
       </c>
+      <c r="AC53" s="34" t="n">
+        <v>3499.99</v>
+      </c>
     </row>
     <row r="54" ht="5" customHeight="1"/>
     <row r="55" ht="22" customHeight="1">
@@ -5041,6 +5174,11 @@
       <c r="AB56" s="34" t="n">
         <v>3599.99</v>
       </c>
+      <c r="AC56" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="57" ht="18" customHeight="1">
       <c r="B57" s="26" t="n">
@@ -5324,6 +5462,9 @@
       <c r="AB62" s="34" t="n">
         <v>127.99</v>
       </c>
+      <c r="AC62" s="34" t="n">
+        <v>127.99</v>
+      </c>
     </row>
     <row r="63" ht="18" customHeight="1">
       <c r="B63" s="6" t="n">
@@ -5439,6 +5580,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AC63" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="64" ht="18" customHeight="1">
       <c r="B64" s="15" t="n">
@@ -5547,6 +5693,11 @@
       </c>
       <c r="AB64" s="36" t="n">
         <v>479.99</v>
+      </c>
+      <c r="AC64" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
     </row>
     <row r="65" ht="18" customHeight="1">
@@ -5780,7 +5931,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:AB70"/>
+  <dimension ref="B1:AC70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -5811,6 +5962,7 @@
     <col width="12" customWidth="1" min="26" max="26"/>
     <col width="12" customWidth="1" min="27" max="27"/>
     <col width="12" customWidth="1" min="28" max="28"/>
+    <col width="12" customWidth="1" min="29" max="29"/>
   </cols>
   <sheetData>
     <row r="1" ht="8" customHeight="1"/>
@@ -5965,6 +6117,11 @@
           <t>3/23</t>
         </is>
       </c>
+      <c r="AC5" s="33" t="inlineStr">
+        <is>
+          <t>3/24</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="22" customHeight="1">
       <c r="B6" s="5" t="inlineStr">
@@ -6079,6 +6236,9 @@
       <c r="AB7" s="34" t="n">
         <v>89.98999999999999</v>
       </c>
+      <c r="AC7" s="34" t="n">
+        <v>89.98999999999999</v>
+      </c>
     </row>
     <row r="8" ht="18" customHeight="1">
       <c r="B8" s="15" t="n">
@@ -6184,6 +6344,9 @@
       <c r="AB8" s="34" t="n">
         <v>194.99</v>
       </c>
+      <c r="AC8" s="34" t="n">
+        <v>194.99</v>
+      </c>
     </row>
     <row r="9" ht="18" customHeight="1">
       <c r="B9" s="6" t="n">
@@ -6303,6 +6466,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AC9" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="18" customHeight="1">
       <c r="B10" s="15" t="n">
@@ -6458,6 +6626,11 @@
       <c r="AB11" s="34" t="n">
         <v>219.99</v>
       </c>
+      <c r="AC11" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="18" customHeight="1">
       <c r="B12" s="15" t="n">
@@ -6567,6 +6740,9 @@
       <c r="AB12" s="34" t="n">
         <v>349.99</v>
       </c>
+      <c r="AC12" s="34" t="n">
+        <v>349.99</v>
+      </c>
     </row>
     <row r="13" ht="18" customHeight="1">
       <c r="B13" s="6" t="n">
@@ -6684,6 +6860,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AC13" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="5" customHeight="1"/>
     <row r="15" ht="22" customHeight="1">
@@ -6811,6 +6992,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AC16" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="B17" s="6" t="n">
@@ -6912,6 +7098,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AC17" s="34" t="n">
+        <v>279.99</v>
+      </c>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="B18" s="15" t="n">
@@ -7019,6 +7208,11 @@
       <c r="AB18" s="34" t="n">
         <v>399.99</v>
       </c>
+      <c r="AC18" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="B19" s="6" t="n">
@@ -7126,6 +7320,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AC19" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="B20" s="15" t="n">
@@ -7231,6 +7430,9 @@
       <c r="AB20" s="34" t="n">
         <v>427.99</v>
       </c>
+      <c r="AC20" s="34" t="n">
+        <v>427.99</v>
+      </c>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="B21" s="6" t="n">
@@ -7330,6 +7532,9 @@
       <c r="AB21" s="34" t="n">
         <v>478.99</v>
       </c>
+      <c r="AC21" s="34" t="n">
+        <v>478.99</v>
+      </c>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="B22" s="15" t="n">
@@ -7443,6 +7648,9 @@
       <c r="AB22" s="34" t="n">
         <v>599.99</v>
       </c>
+      <c r="AC22" s="34" t="n">
+        <v>599.99</v>
+      </c>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="B23" s="6" t="n">
@@ -7550,6 +7758,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AC23" s="34" t="n">
+        <v>999.99</v>
+      </c>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="B24" s="15" t="n">
@@ -7667,6 +7878,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AC24" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="18" customHeight="1">
       <c r="B25" s="6" t="n">
@@ -7776,6 +7992,11 @@
       <c r="AB25" s="34" t="n">
         <v>1199.99</v>
       </c>
+      <c r="AC25" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="18" customHeight="1">
       <c r="B26" s="15" t="n">
@@ -7881,6 +8102,9 @@
       <c r="AB26" s="34" t="n">
         <v>1274.99</v>
       </c>
+      <c r="AC26" s="34" t="n">
+        <v>1274.99</v>
+      </c>
     </row>
     <row r="27" ht="5" customHeight="1"/>
     <row r="28" ht="22" customHeight="1">
@@ -8000,6 +8224,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AC29" s="34" t="n">
+        <v>369.99</v>
+      </c>
     </row>
     <row r="30" ht="18" customHeight="1">
       <c r="B30" s="15" t="n">
@@ -8105,6 +8332,11 @@
       <c r="AB30" s="34" t="n">
         <v>579.99</v>
       </c>
+      <c r="AC30" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="18" customHeight="1">
       <c r="B31" s="6" t="n">
@@ -8216,6 +8448,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AC31" s="13" t="n">
+        <v>699.99</v>
+      </c>
     </row>
     <row r="32" ht="18" customHeight="1">
       <c r="B32" s="15" t="n">
@@ -8321,6 +8556,9 @@
       <c r="AB32" s="34" t="n">
         <v>759.99</v>
       </c>
+      <c r="AC32" s="34" t="n">
+        <v>759.99</v>
+      </c>
     </row>
     <row r="33" ht="18" customHeight="1">
       <c r="B33" s="6" t="n">
@@ -8428,6 +8666,11 @@
       <c r="AB33" s="34" t="n">
         <v>799.99</v>
       </c>
+      <c r="AC33" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="18" customHeight="1">
       <c r="B34" s="15" t="n">
@@ -8533,6 +8776,9 @@
       <c r="AB34" s="34" t="n">
         <v>1274.99</v>
       </c>
+      <c r="AC34" s="34" t="n">
+        <v>1274.99</v>
+      </c>
     </row>
     <row r="35" ht="18" customHeight="1">
       <c r="B35" s="6" t="n">
@@ -8640,6 +8886,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AC35" s="34" t="n">
+        <v>1799.99</v>
+      </c>
     </row>
     <row r="36" ht="18" customHeight="1">
       <c r="B36" s="15" t="n">
@@ -8743,6 +8992,9 @@
       <c r="AB36" s="34" t="n">
         <v>1975.99</v>
       </c>
+      <c r="AC36" s="34" t="n">
+        <v>1975.99</v>
+      </c>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="B37" s="6" t="n">
@@ -8852,6 +9104,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AC37" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="5" customHeight="1"/>
     <row r="39" ht="22" customHeight="1">
@@ -8965,6 +9222,9 @@
       <c r="AB40" s="34" t="n">
         <v>740.99</v>
       </c>
+      <c r="AC40" s="34" t="n">
+        <v>740.99</v>
+      </c>
     </row>
     <row r="41" ht="18" customHeight="1">
       <c r="B41" s="6" t="n">
@@ -9074,6 +9334,9 @@
       <c r="AB41" s="13" t="n">
         <v>599.99</v>
       </c>
+      <c r="AC41" s="13" t="n">
+        <v>599.99</v>
+      </c>
     </row>
     <row r="42" ht="18" customHeight="1">
       <c r="B42" s="15" t="n">
@@ -9181,6 +9444,11 @@
       <c r="AB42" s="34" t="n">
         <v>799.99</v>
       </c>
+      <c r="AC42" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="43" ht="18" customHeight="1">
       <c r="B43" s="6" t="n">
@@ -9292,6 +9560,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AC43" s="34" t="n">
+        <v>949.99</v>
+      </c>
     </row>
     <row r="44" ht="18" customHeight="1">
       <c r="B44" s="15" t="n">
@@ -9393,6 +9664,9 @@
       <c r="AB44" s="34" t="n">
         <v>1139.99</v>
       </c>
+      <c r="AC44" s="34" t="n">
+        <v>1139.99</v>
+      </c>
     </row>
     <row r="45" ht="18" customHeight="1">
       <c r="B45" s="6" t="n">
@@ -9494,6 +9768,11 @@
       <c r="AB45" s="34" t="n">
         <v>1529.99</v>
       </c>
+      <c r="AC45" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="46" ht="18" customHeight="1">
       <c r="B46" s="15" t="n">
@@ -9611,6 +9890,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AC46" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="47" ht="18" customHeight="1">
       <c r="B47" s="6" t="n">
@@ -9716,6 +10000,9 @@
       <c r="AB47" s="34" t="n">
         <v>2999.99</v>
       </c>
+      <c r="AC47" s="34" t="n">
+        <v>2999.99</v>
+      </c>
     </row>
     <row r="48" ht="18" customHeight="1">
       <c r="B48" s="15" t="n">
@@ -9825,6 +10112,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AC48" s="34" t="n">
+        <v>3499.99</v>
+      </c>
     </row>
     <row r="49" ht="5" customHeight="1"/>
     <row r="50" ht="22" customHeight="1">
@@ -9936,6 +10226,11 @@
       <c r="AB51" s="34" t="n">
         <v>798.99</v>
       </c>
+      <c r="AC51" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="52" ht="18" customHeight="1">
       <c r="B52" s="15" t="n">
@@ -10039,6 +10334,11 @@
       <c r="AB52" s="34" t="n">
         <v>798.99</v>
       </c>
+      <c r="AC52" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="53" ht="18" customHeight="1">
       <c r="B53" s="6" t="n">
@@ -10144,6 +10444,9 @@
       <c r="AB53" s="34" t="n">
         <v>1499.99</v>
       </c>
+      <c r="AC53" s="34" t="n">
+        <v>1499.99</v>
+      </c>
     </row>
     <row r="54" ht="18" customHeight="1">
       <c r="B54" s="15" t="n">
@@ -10245,6 +10548,9 @@
       <c r="AB54" s="34" t="n">
         <v>899.99</v>
       </c>
+      <c r="AC54" s="34" t="n">
+        <v>899.99</v>
+      </c>
     </row>
     <row r="55" ht="18" customHeight="1">
       <c r="B55" s="6" t="n">
@@ -10350,6 +10656,9 @@
       <c r="AB55" s="13" t="n">
         <v>1299.99</v>
       </c>
+      <c r="AC55" s="13" t="n">
+        <v>1299.99</v>
+      </c>
     </row>
     <row r="56" ht="18" customHeight="1">
       <c r="B56" s="15" t="n">
@@ -10455,6 +10764,11 @@
       <c r="AB56" s="34" t="n">
         <v>2799.99</v>
       </c>
+      <c r="AC56" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="57" ht="18" customHeight="1">
       <c r="B57" s="6" t="n">
@@ -10560,6 +10874,9 @@
       <c r="AB57" s="34" t="n">
         <v>3199.99</v>
       </c>
+      <c r="AC57" s="34" t="n">
+        <v>3199.99</v>
+      </c>
     </row>
     <row r="58" ht="18" customHeight="1">
       <c r="B58" s="26" t="n">
@@ -10731,6 +11048,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AC61" s="34" t="n">
+        <v>999.99</v>
+      </c>
     </row>
     <row r="62" ht="18" customHeight="1">
       <c r="B62" s="15" t="n">
@@ -10896,6 +11216,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AC63" s="34" t="n">
+        <v>1658.99</v>
+      </c>
     </row>
     <row r="64" ht="18" customHeight="1">
       <c r="B64" s="15" t="n">
@@ -10999,6 +11322,11 @@
       <c r="AB64" s="34" t="n">
         <v>2549.99</v>
       </c>
+      <c r="AC64" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="65" ht="18" customHeight="1">
       <c r="B65" s="26" t="n">
@@ -11279,6 +11607,9 @@
         <is>
           <t>—</t>
         </is>
+      </c>
+      <c r="AC70" s="34" t="n">
+        <v>1899.99</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Price check — 03/25/2026
</commit_message>
<xml_diff>
--- a/PriceBook_Combined_Final.xlsx
+++ b/PriceBook_Combined_Final.xlsx
@@ -709,7 +709,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:AC67"/>
+  <dimension ref="B1:AD67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -741,6 +741,7 @@
     <col width="12" customWidth="1" min="27" max="27"/>
     <col width="12" customWidth="1" min="28" max="28"/>
     <col width="12" customWidth="1" min="29" max="29"/>
+    <col width="12" customWidth="1" min="30" max="30"/>
   </cols>
   <sheetData>
     <row r="1" ht="8" customHeight="1"/>
@@ -900,6 +901,11 @@
           <t>3/24</t>
         </is>
       </c>
+      <c r="AD5" s="33" t="inlineStr">
+        <is>
+          <t>3/25</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="22" customHeight="1">
       <c r="B6" s="5" t="inlineStr">
@@ -1009,6 +1015,9 @@
       <c r="AC7" s="34" t="n">
         <v>449.99</v>
       </c>
+      <c r="AD7" s="34" t="n">
+        <v>449.99</v>
+      </c>
     </row>
     <row r="8" ht="18" customHeight="1">
       <c r="B8" s="15" t="n">
@@ -1133,6 +1142,11 @@
       <c r="AC8" s="34" t="n">
         <v>659.99</v>
       </c>
+      <c r="AD8" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="18" customHeight="1">
       <c r="B9" s="6" t="n">
@@ -1257,6 +1271,11 @@
       <c r="AC9" s="34" t="n">
         <v>659.99</v>
       </c>
+      <c r="AD9" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="18" customHeight="1">
       <c r="B10" s="15" t="n">
@@ -1359,6 +1378,9 @@
       <c r="AC10" s="34" t="n">
         <v>449.99</v>
       </c>
+      <c r="AD10" s="34" t="n">
+        <v>449.99</v>
+      </c>
     </row>
     <row r="11" ht="18" customHeight="1">
       <c r="B11" s="6" t="n">
@@ -1483,6 +1505,11 @@
       <c r="AC11" s="34" t="n">
         <v>659.99</v>
       </c>
+      <c r="AD11" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="18" customHeight="1">
       <c r="B12" s="15" t="n">
@@ -1589,6 +1616,9 @@
       <c r="AC12" s="34" t="n">
         <v>729.99</v>
       </c>
+      <c r="AD12" s="34" t="n">
+        <v>729.99</v>
+      </c>
     </row>
     <row r="13" ht="5" customHeight="1"/>
     <row r="14" ht="22" customHeight="1">
@@ -1711,6 +1741,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AD15" s="34" t="n">
+        <v>599.99</v>
+      </c>
     </row>
     <row r="16" ht="18" customHeight="1">
       <c r="B16" s="15" t="n">
@@ -1819,6 +1852,11 @@
       <c r="AC16" s="13" t="n">
         <v>659.99</v>
       </c>
+      <c r="AD16" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="B17" s="6" t="n">
@@ -1945,6 +1983,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AD17" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="B18" s="15" t="n">
@@ -2109,6 +2152,11 @@
       <c r="AC19" s="34" t="n">
         <v>2199.99</v>
       </c>
+      <c r="AD19" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="5" customHeight="1"/>
     <row r="21" ht="22" customHeight="1">
@@ -2227,6 +2275,9 @@
       <c r="AC22" s="34" t="n">
         <v>1098.99</v>
       </c>
+      <c r="AD22" s="34" t="n">
+        <v>1098.99</v>
+      </c>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="B23" s="6" t="n">
@@ -2339,6 +2390,9 @@
       <c r="AC23" s="34" t="n">
         <v>1199.99</v>
       </c>
+      <c r="AD23" s="34" t="n">
+        <v>1199.99</v>
+      </c>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="B24" s="15" t="n">
@@ -2451,6 +2505,9 @@
       <c r="AC24" s="34" t="n">
         <v>1199.99</v>
       </c>
+      <c r="AD24" s="34" t="n">
+        <v>1199.99</v>
+      </c>
     </row>
     <row r="25" ht="18" customHeight="1">
       <c r="B25" s="6" t="n">
@@ -2621,6 +2678,9 @@
       <c r="AC26" s="34" t="n">
         <v>1599.99</v>
       </c>
+      <c r="AD26" s="34" t="n">
+        <v>1599.99</v>
+      </c>
     </row>
     <row r="27" ht="18" customHeight="1">
       <c r="B27" s="6" t="n">
@@ -2731,6 +2791,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AD27" s="34" t="n">
+        <v>1799.99</v>
+      </c>
     </row>
     <row r="28" ht="18" customHeight="1">
       <c r="B28" s="15" t="n">
@@ -2837,6 +2900,9 @@
       <c r="AC28" s="34" t="n">
         <v>1479.99</v>
       </c>
+      <c r="AD28" s="34" t="n">
+        <v>1479.99</v>
+      </c>
     </row>
     <row r="29" ht="18" customHeight="1">
       <c r="B29" s="6" t="n">
@@ -2947,6 +3013,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AD29" s="34" t="n">
+        <v>1799.99</v>
+      </c>
     </row>
     <row r="30" ht="18" customHeight="1">
       <c r="B30" s="15" t="n">
@@ -3057,6 +3126,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AD30" s="34" t="n">
+        <v>1799.99</v>
+      </c>
     </row>
     <row r="31" ht="5" customHeight="1"/>
     <row r="32" ht="22" customHeight="1">
@@ -3175,6 +3247,9 @@
       <c r="AC33" s="34" t="n">
         <v>1029.99</v>
       </c>
+      <c r="AD33" s="34" t="n">
+        <v>1029.99</v>
+      </c>
     </row>
     <row r="34" ht="18" customHeight="1">
       <c r="B34" s="15" t="n">
@@ -3285,6 +3360,9 @@
       <c r="AC34" s="34" t="n">
         <v>1029.99</v>
       </c>
+      <c r="AD34" s="34" t="n">
+        <v>1029.99</v>
+      </c>
     </row>
     <row r="35" ht="18" customHeight="1">
       <c r="B35" s="6" t="n">
@@ -3399,6 +3477,9 @@
       <c r="AC35" s="34" t="n">
         <v>1599.99</v>
       </c>
+      <c r="AD35" s="34" t="n">
+        <v>1599.99</v>
+      </c>
     </row>
     <row r="36" ht="18" customHeight="1">
       <c r="B36" s="15" t="n">
@@ -3511,6 +3592,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AD36" s="34" t="n">
+        <v>1699.99</v>
+      </c>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="B37" s="6" t="n">
@@ -3619,6 +3703,9 @@
       <c r="AC37" s="34" t="n">
         <v>2499.99</v>
       </c>
+      <c r="AD37" s="34" t="n">
+        <v>2499.99</v>
+      </c>
     </row>
     <row r="38" ht="18" customHeight="1">
       <c r="B38" s="15" t="n">
@@ -3729,6 +3816,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AD38" s="34" t="n">
+        <v>2898.99</v>
+      </c>
     </row>
     <row r="39" ht="18" customHeight="1">
       <c r="B39" s="6" t="n">
@@ -3837,6 +3927,9 @@
       <c r="AC39" s="34" t="n">
         <v>2499.99</v>
       </c>
+      <c r="AD39" s="34" t="n">
+        <v>2499.99</v>
+      </c>
     </row>
     <row r="40" ht="18" customHeight="1">
       <c r="B40" s="15" t="n">
@@ -3947,6 +4040,9 @@
       <c r="AC40" s="34" t="n">
         <v>1029.99</v>
       </c>
+      <c r="AD40" s="34" t="n">
+        <v>1029.99</v>
+      </c>
     </row>
     <row r="41" ht="18" customHeight="1">
       <c r="B41" s="6" t="n">
@@ -4055,6 +4151,11 @@
       <c r="AC41" s="34" t="n">
         <v>1749.99</v>
       </c>
+      <c r="AD41" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="18" customHeight="1">
       <c r="B42" s="15" t="n">
@@ -4173,6 +4274,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AD42" s="34" t="n">
+        <v>1899.99</v>
+      </c>
     </row>
     <row r="43" ht="18" customHeight="1">
       <c r="B43" s="6" t="n">
@@ -4337,6 +4441,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AD44" s="34" t="n">
+        <v>3599.99</v>
+      </c>
     </row>
     <row r="45" ht="5" customHeight="1"/>
     <row r="46" ht="22" customHeight="1">
@@ -4463,6 +4570,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AD47" s="34" t="n">
+        <v>1899.99</v>
+      </c>
     </row>
     <row r="48" ht="18" customHeight="1">
       <c r="B48" s="15" t="n">
@@ -4577,6 +4687,9 @@
       <c r="AC48" s="34" t="n">
         <v>1599.99</v>
       </c>
+      <c r="AD48" s="34" t="n">
+        <v>1599.99</v>
+      </c>
     </row>
     <row r="49" ht="18" customHeight="1">
       <c r="B49" s="6" t="n">
@@ -4689,6 +4802,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AD49" s="34" t="n">
+        <v>1849.99</v>
+      </c>
     </row>
     <row r="50" ht="18" customHeight="1">
       <c r="B50" s="15" t="n">
@@ -4795,6 +4911,9 @@
       <c r="AC50" s="34" t="n">
         <v>2599.99</v>
       </c>
+      <c r="AD50" s="34" t="n">
+        <v>2599.99</v>
+      </c>
     </row>
     <row r="51" ht="18" customHeight="1">
       <c r="B51" s="6" t="n">
@@ -4957,6 +5076,9 @@
       <c r="AC52" s="34" t="n">
         <v>2599.99</v>
       </c>
+      <c r="AD52" s="34" t="n">
+        <v>2599.99</v>
+      </c>
     </row>
     <row r="53" ht="18" customHeight="1">
       <c r="B53" s="6" t="n">
@@ -5063,6 +5185,11 @@
       <c r="AC53" s="34" t="n">
         <v>3499.99</v>
       </c>
+      <c r="AD53" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="54" ht="5" customHeight="1"/>
     <row r="55" ht="22" customHeight="1">
@@ -5179,6 +5306,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AD56" s="34" t="n">
+        <v>3599.99</v>
+      </c>
     </row>
     <row r="57" ht="18" customHeight="1">
       <c r="B57" s="26" t="n">
@@ -5465,6 +5595,9 @@
       <c r="AC62" s="34" t="n">
         <v>127.99</v>
       </c>
+      <c r="AD62" s="34" t="n">
+        <v>127.99</v>
+      </c>
     </row>
     <row r="63" ht="18" customHeight="1">
       <c r="B63" s="6" t="n">
@@ -5585,6 +5718,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AD63" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="64" ht="18" customHeight="1">
       <c r="B64" s="15" t="n">
@@ -5695,6 +5833,11 @@
         <v>479.99</v>
       </c>
       <c r="AC64" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AD64" s="35" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -5931,7 +6074,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:AC70"/>
+  <dimension ref="B1:AD70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -5963,6 +6106,7 @@
     <col width="12" customWidth="1" min="27" max="27"/>
     <col width="12" customWidth="1" min="28" max="28"/>
     <col width="12" customWidth="1" min="29" max="29"/>
+    <col width="12" customWidth="1" min="30" max="30"/>
   </cols>
   <sheetData>
     <row r="1" ht="8" customHeight="1"/>
@@ -6122,6 +6266,11 @@
           <t>3/24</t>
         </is>
       </c>
+      <c r="AD5" s="33" t="inlineStr">
+        <is>
+          <t>3/25</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="22" customHeight="1">
       <c r="B6" s="5" t="inlineStr">
@@ -6239,6 +6388,9 @@
       <c r="AC7" s="34" t="n">
         <v>89.98999999999999</v>
       </c>
+      <c r="AD7" s="34" t="n">
+        <v>89.98999999999999</v>
+      </c>
     </row>
     <row r="8" ht="18" customHeight="1">
       <c r="B8" s="15" t="n">
@@ -6347,6 +6499,9 @@
       <c r="AC8" s="34" t="n">
         <v>194.99</v>
       </c>
+      <c r="AD8" s="34" t="n">
+        <v>194.99</v>
+      </c>
     </row>
     <row r="9" ht="18" customHeight="1">
       <c r="B9" s="6" t="n">
@@ -6471,6 +6626,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AD9" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="18" customHeight="1">
       <c r="B10" s="15" t="n">
@@ -6631,6 +6791,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AD11" s="34" t="n">
+        <v>219.99</v>
+      </c>
     </row>
     <row r="12" ht="18" customHeight="1">
       <c r="B12" s="15" t="n">
@@ -6743,6 +6906,9 @@
       <c r="AC12" s="34" t="n">
         <v>349.99</v>
       </c>
+      <c r="AD12" s="34" t="n">
+        <v>349.99</v>
+      </c>
     </row>
     <row r="13" ht="18" customHeight="1">
       <c r="B13" s="6" t="n">
@@ -6865,6 +7031,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AD13" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="5" customHeight="1"/>
     <row r="15" ht="22" customHeight="1">
@@ -6997,6 +7168,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AD16" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="B17" s="6" t="n">
@@ -7101,6 +7277,9 @@
       <c r="AC17" s="34" t="n">
         <v>279.99</v>
       </c>
+      <c r="AD17" s="34" t="n">
+        <v>279.99</v>
+      </c>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="B18" s="15" t="n">
@@ -7213,6 +7392,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AD18" s="34" t="n">
+        <v>399.99</v>
+      </c>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="B19" s="6" t="n">
@@ -7325,6 +7507,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AD19" s="34" t="n">
+        <v>249.99</v>
+      </c>
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="B20" s="15" t="n">
@@ -7433,6 +7618,9 @@
       <c r="AC20" s="34" t="n">
         <v>427.99</v>
       </c>
+      <c r="AD20" s="34" t="n">
+        <v>427.99</v>
+      </c>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="B21" s="6" t="n">
@@ -7535,6 +7723,9 @@
       <c r="AC21" s="34" t="n">
         <v>478.99</v>
       </c>
+      <c r="AD21" s="34" t="n">
+        <v>478.99</v>
+      </c>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="B22" s="15" t="n">
@@ -7651,6 +7842,9 @@
       <c r="AC22" s="34" t="n">
         <v>599.99</v>
       </c>
+      <c r="AD22" s="34" t="n">
+        <v>599.99</v>
+      </c>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="B23" s="6" t="n">
@@ -7761,6 +7955,9 @@
       <c r="AC23" s="34" t="n">
         <v>999.99</v>
       </c>
+      <c r="AD23" s="34" t="n">
+        <v>999.99</v>
+      </c>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="B24" s="15" t="n">
@@ -7883,6 +8080,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AD24" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="18" customHeight="1">
       <c r="B25" s="6" t="n">
@@ -7997,6 +8199,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AD25" s="34" t="n">
+        <v>1199.99</v>
+      </c>
     </row>
     <row r="26" ht="18" customHeight="1">
       <c r="B26" s="15" t="n">
@@ -8105,6 +8310,9 @@
       <c r="AC26" s="34" t="n">
         <v>1274.99</v>
       </c>
+      <c r="AD26" s="34" t="n">
+        <v>1274.99</v>
+      </c>
     </row>
     <row r="27" ht="5" customHeight="1"/>
     <row r="28" ht="22" customHeight="1">
@@ -8227,6 +8435,9 @@
       <c r="AC29" s="34" t="n">
         <v>369.99</v>
       </c>
+      <c r="AD29" s="34" t="n">
+        <v>369.99</v>
+      </c>
     </row>
     <row r="30" ht="18" customHeight="1">
       <c r="B30" s="15" t="n">
@@ -8337,6 +8548,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AD30" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="18" customHeight="1">
       <c r="B31" s="6" t="n">
@@ -8451,6 +8667,9 @@
       <c r="AC31" s="13" t="n">
         <v>699.99</v>
       </c>
+      <c r="AD31" s="13" t="n">
+        <v>699.99</v>
+      </c>
     </row>
     <row r="32" ht="18" customHeight="1">
       <c r="B32" s="15" t="n">
@@ -8559,6 +8778,9 @@
       <c r="AC32" s="34" t="n">
         <v>759.99</v>
       </c>
+      <c r="AD32" s="34" t="n">
+        <v>759.99</v>
+      </c>
     </row>
     <row r="33" ht="18" customHeight="1">
       <c r="B33" s="6" t="n">
@@ -8671,6 +8893,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AD33" s="34" t="n">
+        <v>799.99</v>
+      </c>
     </row>
     <row r="34" ht="18" customHeight="1">
       <c r="B34" s="15" t="n">
@@ -8779,6 +9004,9 @@
       <c r="AC34" s="34" t="n">
         <v>1274.99</v>
       </c>
+      <c r="AD34" s="34" t="n">
+        <v>1274.99</v>
+      </c>
     </row>
     <row r="35" ht="18" customHeight="1">
       <c r="B35" s="6" t="n">
@@ -8889,6 +9117,9 @@
       <c r="AC35" s="34" t="n">
         <v>1799.99</v>
       </c>
+      <c r="AD35" s="34" t="n">
+        <v>1799.99</v>
+      </c>
     </row>
     <row r="36" ht="18" customHeight="1">
       <c r="B36" s="15" t="n">
@@ -8995,6 +9226,9 @@
       <c r="AC36" s="34" t="n">
         <v>1975.99</v>
       </c>
+      <c r="AD36" s="34" t="n">
+        <v>1975.99</v>
+      </c>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="B37" s="6" t="n">
@@ -9109,6 +9343,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AD37" s="34" t="n">
+        <v>2699.99</v>
+      </c>
     </row>
     <row r="38" ht="5" customHeight="1"/>
     <row r="39" ht="22" customHeight="1">
@@ -9225,6 +9462,11 @@
       <c r="AC40" s="34" t="n">
         <v>740.99</v>
       </c>
+      <c r="AD40" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="18" customHeight="1">
       <c r="B41" s="6" t="n">
@@ -9337,6 +9579,9 @@
       <c r="AC41" s="13" t="n">
         <v>599.99</v>
       </c>
+      <c r="AD41" s="13" t="n">
+        <v>599.99</v>
+      </c>
     </row>
     <row r="42" ht="18" customHeight="1">
       <c r="B42" s="15" t="n">
@@ -9449,6 +9694,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AD42" s="34" t="n">
+        <v>799.99</v>
+      </c>
     </row>
     <row r="43" ht="18" customHeight="1">
       <c r="B43" s="6" t="n">
@@ -9563,6 +9811,9 @@
       <c r="AC43" s="34" t="n">
         <v>949.99</v>
       </c>
+      <c r="AD43" s="34" t="n">
+        <v>949.99</v>
+      </c>
     </row>
     <row r="44" ht="18" customHeight="1">
       <c r="B44" s="15" t="n">
@@ -9667,6 +9918,9 @@
       <c r="AC44" s="34" t="n">
         <v>1139.99</v>
       </c>
+      <c r="AD44" s="34" t="n">
+        <v>1139.99</v>
+      </c>
     </row>
     <row r="45" ht="18" customHeight="1">
       <c r="B45" s="6" t="n">
@@ -9773,6 +10027,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AD45" s="34" t="n">
+        <v>1529.99</v>
+      </c>
     </row>
     <row r="46" ht="18" customHeight="1">
       <c r="B46" s="15" t="n">
@@ -9895,6 +10152,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AD46" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="47" ht="18" customHeight="1">
       <c r="B47" s="6" t="n">
@@ -10003,6 +10265,11 @@
       <c r="AC47" s="34" t="n">
         <v>2999.99</v>
       </c>
+      <c r="AD47" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="48" ht="18" customHeight="1">
       <c r="B48" s="15" t="n">
@@ -10115,6 +10382,9 @@
       <c r="AC48" s="34" t="n">
         <v>3499.99</v>
       </c>
+      <c r="AD48" s="34" t="n">
+        <v>3499.99</v>
+      </c>
     </row>
     <row r="49" ht="5" customHeight="1"/>
     <row r="50" ht="22" customHeight="1">
@@ -10231,6 +10501,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AD51" s="34" t="n">
+        <v>798.99</v>
+      </c>
     </row>
     <row r="52" ht="18" customHeight="1">
       <c r="B52" s="15" t="n">
@@ -10339,6 +10612,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AD52" s="34" t="n">
+        <v>798.99</v>
+      </c>
     </row>
     <row r="53" ht="18" customHeight="1">
       <c r="B53" s="6" t="n">
@@ -10447,6 +10723,9 @@
       <c r="AC53" s="34" t="n">
         <v>1499.99</v>
       </c>
+      <c r="AD53" s="34" t="n">
+        <v>1499.99</v>
+      </c>
     </row>
     <row r="54" ht="18" customHeight="1">
       <c r="B54" s="15" t="n">
@@ -10551,6 +10830,9 @@
       <c r="AC54" s="34" t="n">
         <v>899.99</v>
       </c>
+      <c r="AD54" s="34" t="n">
+        <v>899.99</v>
+      </c>
     </row>
     <row r="55" ht="18" customHeight="1">
       <c r="B55" s="6" t="n">
@@ -10659,6 +10941,11 @@
       <c r="AC55" s="13" t="n">
         <v>1299.99</v>
       </c>
+      <c r="AD55" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="56" ht="18" customHeight="1">
       <c r="B56" s="15" t="n">
@@ -10769,6 +11056,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AD56" s="34" t="n">
+        <v>2799.99</v>
+      </c>
     </row>
     <row r="57" ht="18" customHeight="1">
       <c r="B57" s="6" t="n">
@@ -10877,6 +11167,9 @@
       <c r="AC57" s="34" t="n">
         <v>3199.99</v>
       </c>
+      <c r="AD57" s="34" t="n">
+        <v>3199.99</v>
+      </c>
     </row>
     <row r="58" ht="18" customHeight="1">
       <c r="B58" s="26" t="n">
@@ -11051,6 +11344,9 @@
       <c r="AC61" s="34" t="n">
         <v>999.99</v>
       </c>
+      <c r="AD61" s="34" t="n">
+        <v>999.99</v>
+      </c>
     </row>
     <row r="62" ht="18" customHeight="1">
       <c r="B62" s="15" t="n">
@@ -11219,6 +11515,9 @@
       <c r="AC63" s="34" t="n">
         <v>1658.99</v>
       </c>
+      <c r="AD63" s="34" t="n">
+        <v>1658.99</v>
+      </c>
     </row>
     <row r="64" ht="18" customHeight="1">
       <c r="B64" s="15" t="n">
@@ -11327,6 +11626,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AD64" s="34" t="n">
+        <v>2549.99</v>
+      </c>
     </row>
     <row r="65" ht="18" customHeight="1">
       <c r="B65" s="26" t="n">
@@ -11609,6 +11911,9 @@
         </is>
       </c>
       <c r="AC70" s="34" t="n">
+        <v>1899.99</v>
+      </c>
+      <c r="AD70" s="34" t="n">
         <v>1899.99</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Price check — 03/26/2026
</commit_message>
<xml_diff>
--- a/PriceBook_Combined_Final.xlsx
+++ b/PriceBook_Combined_Final.xlsx
@@ -709,7 +709,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:AD67"/>
+  <dimension ref="B1:AE67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -742,6 +742,7 @@
     <col width="12" customWidth="1" min="28" max="28"/>
     <col width="12" customWidth="1" min="29" max="29"/>
     <col width="12" customWidth="1" min="30" max="30"/>
+    <col width="12" customWidth="1" min="31" max="31"/>
   </cols>
   <sheetData>
     <row r="1" ht="8" customHeight="1"/>
@@ -906,6 +907,11 @@
           <t>3/25</t>
         </is>
       </c>
+      <c r="AE5" s="33" t="inlineStr">
+        <is>
+          <t>3/26</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="22" customHeight="1">
       <c r="B6" s="5" t="inlineStr">
@@ -1018,6 +1024,9 @@
       <c r="AD7" s="34" t="n">
         <v>449.99</v>
       </c>
+      <c r="AE7" s="34" t="n">
+        <v>449.99</v>
+      </c>
     </row>
     <row r="8" ht="18" customHeight="1">
       <c r="B8" s="15" t="n">
@@ -1147,6 +1156,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AE8" s="36" t="n">
+        <v>809.99</v>
+      </c>
     </row>
     <row r="9" ht="18" customHeight="1">
       <c r="B9" s="6" t="n">
@@ -1276,6 +1288,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AE9" s="36" t="n">
+        <v>809.99</v>
+      </c>
     </row>
     <row r="10" ht="18" customHeight="1">
       <c r="B10" s="15" t="n">
@@ -1381,6 +1396,9 @@
       <c r="AD10" s="34" t="n">
         <v>449.99</v>
       </c>
+      <c r="AE10" s="34" t="n">
+        <v>449.99</v>
+      </c>
     </row>
     <row r="11" ht="18" customHeight="1">
       <c r="B11" s="6" t="n">
@@ -1510,6 +1528,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AE11" s="36" t="n">
+        <v>809.99</v>
+      </c>
     </row>
     <row r="12" ht="18" customHeight="1">
       <c r="B12" s="15" t="n">
@@ -1619,6 +1640,9 @@
       <c r="AD12" s="34" t="n">
         <v>729.99</v>
       </c>
+      <c r="AE12" s="36" t="n">
+        <v>839.99</v>
+      </c>
     </row>
     <row r="13" ht="5" customHeight="1"/>
     <row r="14" ht="22" customHeight="1">
@@ -1744,6 +1768,9 @@
       <c r="AD15" s="34" t="n">
         <v>599.99</v>
       </c>
+      <c r="AE15" s="34" t="n">
+        <v>599.99</v>
+      </c>
     </row>
     <row r="16" ht="18" customHeight="1">
       <c r="B16" s="15" t="n">
@@ -1857,6 +1884,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AE16" s="36" t="n">
+        <v>809.99</v>
+      </c>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="B17" s="6" t="n">
@@ -1984,6 +2014,11 @@
         </is>
       </c>
       <c r="AD17" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AE17" s="35" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2157,6 +2192,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AE19" s="34" t="n">
+        <v>2199.99</v>
+      </c>
     </row>
     <row r="20" ht="5" customHeight="1"/>
     <row r="21" ht="22" customHeight="1">
@@ -2278,6 +2316,9 @@
       <c r="AD22" s="34" t="n">
         <v>1098.99</v>
       </c>
+      <c r="AE22" s="34" t="n">
+        <v>1098.99</v>
+      </c>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="B23" s="6" t="n">
@@ -2393,6 +2434,9 @@
       <c r="AD23" s="34" t="n">
         <v>1199.99</v>
       </c>
+      <c r="AE23" s="34" t="n">
+        <v>1199.99</v>
+      </c>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="B24" s="15" t="n">
@@ -2506,6 +2550,9 @@
         <v>1199.99</v>
       </c>
       <c r="AD24" s="34" t="n">
+        <v>1199.99</v>
+      </c>
+      <c r="AE24" s="34" t="n">
         <v>1199.99</v>
       </c>
     </row>
@@ -2681,6 +2728,11 @@
       <c r="AD26" s="34" t="n">
         <v>1599.99</v>
       </c>
+      <c r="AE26" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="18" customHeight="1">
       <c r="B27" s="6" t="n">
@@ -2794,6 +2846,9 @@
       <c r="AD27" s="34" t="n">
         <v>1799.99</v>
       </c>
+      <c r="AE27" s="34" t="n">
+        <v>1799.99</v>
+      </c>
     </row>
     <row r="28" ht="18" customHeight="1">
       <c r="B28" s="15" t="n">
@@ -2903,6 +2958,9 @@
       <c r="AD28" s="34" t="n">
         <v>1479.99</v>
       </c>
+      <c r="AE28" s="34" t="n">
+        <v>1479.99</v>
+      </c>
     </row>
     <row r="29" ht="18" customHeight="1">
       <c r="B29" s="6" t="n">
@@ -3016,6 +3074,9 @@
       <c r="AD29" s="34" t="n">
         <v>1799.99</v>
       </c>
+      <c r="AE29" s="34" t="n">
+        <v>1799.99</v>
+      </c>
     </row>
     <row r="30" ht="18" customHeight="1">
       <c r="B30" s="15" t="n">
@@ -3129,6 +3190,9 @@
       <c r="AD30" s="34" t="n">
         <v>1799.99</v>
       </c>
+      <c r="AE30" s="34" t="n">
+        <v>1799.99</v>
+      </c>
     </row>
     <row r="31" ht="5" customHeight="1"/>
     <row r="32" ht="22" customHeight="1">
@@ -3250,6 +3314,9 @@
       <c r="AD33" s="34" t="n">
         <v>1029.99</v>
       </c>
+      <c r="AE33" s="34" t="n">
+        <v>1029.99</v>
+      </c>
     </row>
     <row r="34" ht="18" customHeight="1">
       <c r="B34" s="15" t="n">
@@ -3363,6 +3430,9 @@
       <c r="AD34" s="34" t="n">
         <v>1029.99</v>
       </c>
+      <c r="AE34" s="34" t="n">
+        <v>1029.99</v>
+      </c>
     </row>
     <row r="35" ht="18" customHeight="1">
       <c r="B35" s="6" t="n">
@@ -3480,6 +3550,11 @@
       <c r="AD35" s="34" t="n">
         <v>1599.99</v>
       </c>
+      <c r="AE35" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="18" customHeight="1">
       <c r="B36" s="15" t="n">
@@ -3595,6 +3670,11 @@
       <c r="AD36" s="34" t="n">
         <v>1699.99</v>
       </c>
+      <c r="AE36" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="B37" s="6" t="n">
@@ -3706,6 +3786,9 @@
       <c r="AD37" s="34" t="n">
         <v>2499.99</v>
       </c>
+      <c r="AE37" s="36" t="n">
+        <v>3399.99</v>
+      </c>
     </row>
     <row r="38" ht="18" customHeight="1">
       <c r="B38" s="15" t="n">
@@ -3819,6 +3902,9 @@
       <c r="AD38" s="34" t="n">
         <v>2898.99</v>
       </c>
+      <c r="AE38" s="34" t="n">
+        <v>2898.99</v>
+      </c>
     </row>
     <row r="39" ht="18" customHeight="1">
       <c r="B39" s="6" t="n">
@@ -3930,6 +4016,9 @@
       <c r="AD39" s="34" t="n">
         <v>2499.99</v>
       </c>
+      <c r="AE39" s="36" t="n">
+        <v>3399.99</v>
+      </c>
     </row>
     <row r="40" ht="18" customHeight="1">
       <c r="B40" s="15" t="n">
@@ -4043,6 +4132,9 @@
       <c r="AD40" s="34" t="n">
         <v>1029.99</v>
       </c>
+      <c r="AE40" s="34" t="n">
+        <v>1029.99</v>
+      </c>
     </row>
     <row r="41" ht="18" customHeight="1">
       <c r="B41" s="6" t="n">
@@ -4156,6 +4248,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AE41" s="34" t="n">
+        <v>1749.99</v>
+      </c>
     </row>
     <row r="42" ht="18" customHeight="1">
       <c r="B42" s="15" t="n">
@@ -4276,6 +4371,9 @@
       </c>
       <c r="AD42" s="34" t="n">
         <v>1899.99</v>
+      </c>
+      <c r="AE42" s="36" t="n">
+        <v>1999.99</v>
       </c>
     </row>
     <row r="43" ht="18" customHeight="1">
@@ -4444,6 +4542,9 @@
       <c r="AD44" s="34" t="n">
         <v>3599.99</v>
       </c>
+      <c r="AE44" s="34" t="n">
+        <v>3599.99</v>
+      </c>
     </row>
     <row r="45" ht="5" customHeight="1"/>
     <row r="46" ht="22" customHeight="1">
@@ -4573,6 +4674,9 @@
       <c r="AD47" s="34" t="n">
         <v>1899.99</v>
       </c>
+      <c r="AE47" s="36" t="n">
+        <v>1999.99</v>
+      </c>
     </row>
     <row r="48" ht="18" customHeight="1">
       <c r="B48" s="15" t="n">
@@ -4690,6 +4794,11 @@
       <c r="AD48" s="34" t="n">
         <v>1599.99</v>
       </c>
+      <c r="AE48" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="49" ht="18" customHeight="1">
       <c r="B49" s="6" t="n">
@@ -4805,6 +4914,9 @@
       <c r="AD49" s="34" t="n">
         <v>1849.99</v>
       </c>
+      <c r="AE49" s="34" t="n">
+        <v>1849.99</v>
+      </c>
     </row>
     <row r="50" ht="18" customHeight="1">
       <c r="B50" s="15" t="n">
@@ -4912,6 +5024,9 @@
         <v>2599.99</v>
       </c>
       <c r="AD50" s="34" t="n">
+        <v>2599.99</v>
+      </c>
+      <c r="AE50" s="34" t="n">
         <v>2599.99</v>
       </c>
     </row>
@@ -5079,6 +5194,9 @@
       <c r="AD52" s="34" t="n">
         <v>2599.99</v>
       </c>
+      <c r="AE52" s="34" t="n">
+        <v>2599.99</v>
+      </c>
     </row>
     <row r="53" ht="18" customHeight="1">
       <c r="B53" s="6" t="n">
@@ -5190,6 +5308,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AE53" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="54" ht="5" customHeight="1"/>
     <row r="55" ht="22" customHeight="1">
@@ -5307,6 +5430,9 @@
         </is>
       </c>
       <c r="AD56" s="34" t="n">
+        <v>3599.99</v>
+      </c>
+      <c r="AE56" s="34" t="n">
         <v>3599.99</v>
       </c>
     </row>
@@ -5598,6 +5724,9 @@
       <c r="AD62" s="34" t="n">
         <v>127.99</v>
       </c>
+      <c r="AE62" s="34" t="n">
+        <v>127.99</v>
+      </c>
     </row>
     <row r="63" ht="18" customHeight="1">
       <c r="B63" s="6" t="n">
@@ -5723,6 +5852,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AE63" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="64" ht="18" customHeight="1">
       <c r="B64" s="15" t="n">
@@ -5838,6 +5972,11 @@
         </is>
       </c>
       <c r="AD64" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AE64" s="35" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -6074,7 +6213,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:AD70"/>
+  <dimension ref="B1:AE70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -6107,6 +6246,7 @@
     <col width="12" customWidth="1" min="28" max="28"/>
     <col width="12" customWidth="1" min="29" max="29"/>
     <col width="12" customWidth="1" min="30" max="30"/>
+    <col width="12" customWidth="1" min="31" max="31"/>
   </cols>
   <sheetData>
     <row r="1" ht="8" customHeight="1"/>
@@ -6271,6 +6411,11 @@
           <t>3/25</t>
         </is>
       </c>
+      <c r="AE5" s="33" t="inlineStr">
+        <is>
+          <t>3/26</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="22" customHeight="1">
       <c r="B6" s="5" t="inlineStr">
@@ -6391,6 +6536,11 @@
       <c r="AD7" s="34" t="n">
         <v>89.98999999999999</v>
       </c>
+      <c r="AE7" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="18" customHeight="1">
       <c r="B8" s="15" t="n">
@@ -6502,6 +6652,9 @@
       <c r="AD8" s="34" t="n">
         <v>194.99</v>
       </c>
+      <c r="AE8" s="34" t="n">
+        <v>194.99</v>
+      </c>
     </row>
     <row r="9" ht="18" customHeight="1">
       <c r="B9" s="6" t="n">
@@ -6627,6 +6780,11 @@
         </is>
       </c>
       <c r="AD9" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AE9" s="35" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -6794,6 +6952,9 @@
       <c r="AD11" s="34" t="n">
         <v>219.99</v>
       </c>
+      <c r="AE11" s="34" t="n">
+        <v>219.99</v>
+      </c>
     </row>
     <row r="12" ht="18" customHeight="1">
       <c r="B12" s="15" t="n">
@@ -6909,6 +7070,9 @@
       <c r="AD12" s="34" t="n">
         <v>349.99</v>
       </c>
+      <c r="AE12" s="34" t="n">
+        <v>349.99</v>
+      </c>
     </row>
     <row r="13" ht="18" customHeight="1">
       <c r="B13" s="6" t="n">
@@ -7036,6 +7200,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AE13" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="5" customHeight="1"/>
     <row r="15" ht="22" customHeight="1">
@@ -7173,6 +7342,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AE16" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="B17" s="6" t="n">
@@ -7280,6 +7454,11 @@
       <c r="AD17" s="34" t="n">
         <v>279.99</v>
       </c>
+      <c r="AE17" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="B18" s="15" t="n">
@@ -7395,6 +7574,9 @@
       <c r="AD18" s="34" t="n">
         <v>399.99</v>
       </c>
+      <c r="AE18" s="34" t="n">
+        <v>399.99</v>
+      </c>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="B19" s="6" t="n">
@@ -7510,6 +7692,9 @@
       <c r="AD19" s="34" t="n">
         <v>249.99</v>
       </c>
+      <c r="AE19" s="34" t="n">
+        <v>249.99</v>
+      </c>
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="B20" s="15" t="n">
@@ -7621,6 +7806,11 @@
       <c r="AD20" s="34" t="n">
         <v>427.99</v>
       </c>
+      <c r="AE20" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="B21" s="6" t="n">
@@ -7726,6 +7916,9 @@
       <c r="AD21" s="34" t="n">
         <v>478.99</v>
       </c>
+      <c r="AE21" s="34" t="n">
+        <v>478.99</v>
+      </c>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="B22" s="15" t="n">
@@ -7845,6 +8038,11 @@
       <c r="AD22" s="34" t="n">
         <v>599.99</v>
       </c>
+      <c r="AE22" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="B23" s="6" t="n">
@@ -7958,6 +8156,9 @@
       <c r="AD23" s="34" t="n">
         <v>999.99</v>
       </c>
+      <c r="AE23" s="34" t="n">
+        <v>999.99</v>
+      </c>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="B24" s="15" t="n">
@@ -8085,6 +8286,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AE24" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="18" customHeight="1">
       <c r="B25" s="6" t="n">
@@ -8202,6 +8408,11 @@
       <c r="AD25" s="34" t="n">
         <v>1199.99</v>
       </c>
+      <c r="AE25" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="18" customHeight="1">
       <c r="B26" s="15" t="n">
@@ -8313,6 +8524,9 @@
       <c r="AD26" s="34" t="n">
         <v>1274.99</v>
       </c>
+      <c r="AE26" s="34" t="n">
+        <v>1274.99</v>
+      </c>
     </row>
     <row r="27" ht="5" customHeight="1"/>
     <row r="28" ht="22" customHeight="1">
@@ -8438,6 +8652,9 @@
       <c r="AD29" s="34" t="n">
         <v>369.99</v>
       </c>
+      <c r="AE29" s="34" t="n">
+        <v>369.99</v>
+      </c>
     </row>
     <row r="30" ht="18" customHeight="1">
       <c r="B30" s="15" t="n">
@@ -8553,6 +8770,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AE30" s="34" t="n">
+        <v>579.99</v>
+      </c>
     </row>
     <row r="31" ht="18" customHeight="1">
       <c r="B31" s="6" t="n">
@@ -8670,6 +8890,9 @@
       <c r="AD31" s="13" t="n">
         <v>699.99</v>
       </c>
+      <c r="AE31" s="13" t="n">
+        <v>699.99</v>
+      </c>
     </row>
     <row r="32" ht="18" customHeight="1">
       <c r="B32" s="15" t="n">
@@ -8781,6 +9004,11 @@
       <c r="AD32" s="34" t="n">
         <v>759.99</v>
       </c>
+      <c r="AE32" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="18" customHeight="1">
       <c r="B33" s="6" t="n">
@@ -8896,6 +9124,11 @@
       <c r="AD33" s="34" t="n">
         <v>799.99</v>
       </c>
+      <c r="AE33" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="18" customHeight="1">
       <c r="B34" s="15" t="n">
@@ -9007,6 +9240,9 @@
       <c r="AD34" s="34" t="n">
         <v>1274.99</v>
       </c>
+      <c r="AE34" s="34" t="n">
+        <v>1274.99</v>
+      </c>
     </row>
     <row r="35" ht="18" customHeight="1">
       <c r="B35" s="6" t="n">
@@ -9120,6 +9356,9 @@
       <c r="AD35" s="34" t="n">
         <v>1799.99</v>
       </c>
+      <c r="AE35" s="34" t="n">
+        <v>1799.99</v>
+      </c>
     </row>
     <row r="36" ht="18" customHeight="1">
       <c r="B36" s="15" t="n">
@@ -9229,6 +9468,9 @@
       <c r="AD36" s="34" t="n">
         <v>1975.99</v>
       </c>
+      <c r="AE36" s="34" t="n">
+        <v>1975.99</v>
+      </c>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="B37" s="6" t="n">
@@ -9346,6 +9588,9 @@
       <c r="AD37" s="34" t="n">
         <v>2699.99</v>
       </c>
+      <c r="AE37" s="34" t="n">
+        <v>2699.99</v>
+      </c>
     </row>
     <row r="38" ht="5" customHeight="1"/>
     <row r="39" ht="22" customHeight="1">
@@ -9467,6 +9712,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AE40" s="34" t="n">
+        <v>740.99</v>
+      </c>
     </row>
     <row r="41" ht="18" customHeight="1">
       <c r="B41" s="6" t="n">
@@ -9582,6 +9830,11 @@
       <c r="AD41" s="13" t="n">
         <v>599.99</v>
       </c>
+      <c r="AE41" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="18" customHeight="1">
       <c r="B42" s="15" t="n">
@@ -9697,6 +9950,11 @@
       <c r="AD42" s="34" t="n">
         <v>799.99</v>
       </c>
+      <c r="AE42" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="43" ht="18" customHeight="1">
       <c r="B43" s="6" t="n">
@@ -9814,6 +10072,11 @@
       <c r="AD43" s="34" t="n">
         <v>949.99</v>
       </c>
+      <c r="AE43" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="44" ht="18" customHeight="1">
       <c r="B44" s="15" t="n">
@@ -9921,6 +10184,9 @@
       <c r="AD44" s="34" t="n">
         <v>1139.99</v>
       </c>
+      <c r="AE44" s="34" t="n">
+        <v>1139.99</v>
+      </c>
     </row>
     <row r="45" ht="18" customHeight="1">
       <c r="B45" s="6" t="n">
@@ -10030,6 +10296,9 @@
       <c r="AD45" s="34" t="n">
         <v>1529.99</v>
       </c>
+      <c r="AE45" s="34" t="n">
+        <v>1529.99</v>
+      </c>
     </row>
     <row r="46" ht="18" customHeight="1">
       <c r="B46" s="15" t="n">
@@ -10157,6 +10426,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AE46" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="47" ht="18" customHeight="1">
       <c r="B47" s="6" t="n">
@@ -10270,6 +10544,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AE47" s="34" t="n">
+        <v>2999.99</v>
+      </c>
     </row>
     <row r="48" ht="18" customHeight="1">
       <c r="B48" s="15" t="n">
@@ -10385,6 +10662,11 @@
       <c r="AD48" s="34" t="n">
         <v>3499.99</v>
       </c>
+      <c r="AE48" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="49" ht="5" customHeight="1"/>
     <row r="50" ht="22" customHeight="1">
@@ -10504,6 +10786,9 @@
       <c r="AD51" s="34" t="n">
         <v>798.99</v>
       </c>
+      <c r="AE51" s="34" t="n">
+        <v>798.99</v>
+      </c>
     </row>
     <row r="52" ht="18" customHeight="1">
       <c r="B52" s="15" t="n">
@@ -10615,6 +10900,9 @@
       <c r="AD52" s="34" t="n">
         <v>798.99</v>
       </c>
+      <c r="AE52" s="34" t="n">
+        <v>798.99</v>
+      </c>
     </row>
     <row r="53" ht="18" customHeight="1">
       <c r="B53" s="6" t="n">
@@ -10726,6 +11014,11 @@
       <c r="AD53" s="34" t="n">
         <v>1499.99</v>
       </c>
+      <c r="AE53" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="54" ht="18" customHeight="1">
       <c r="B54" s="15" t="n">
@@ -10833,6 +11126,9 @@
       <c r="AD54" s="34" t="n">
         <v>899.99</v>
       </c>
+      <c r="AE54" s="34" t="n">
+        <v>899.99</v>
+      </c>
     </row>
     <row r="55" ht="18" customHeight="1">
       <c r="B55" s="6" t="n">
@@ -10946,6 +11242,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AE55" s="13" t="n">
+        <v>1299.99</v>
+      </c>
     </row>
     <row r="56" ht="18" customHeight="1">
       <c r="B56" s="15" t="n">
@@ -11059,6 +11358,11 @@
       <c r="AD56" s="34" t="n">
         <v>2799.99</v>
       </c>
+      <c r="AE56" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="57" ht="18" customHeight="1">
       <c r="B57" s="6" t="n">
@@ -11168,6 +11472,9 @@
         <v>3199.99</v>
       </c>
       <c r="AD57" s="34" t="n">
+        <v>3199.99</v>
+      </c>
+      <c r="AE57" s="34" t="n">
         <v>3199.99</v>
       </c>
     </row>
@@ -11347,6 +11654,9 @@
       <c r="AD61" s="34" t="n">
         <v>999.99</v>
       </c>
+      <c r="AE61" s="34" t="n">
+        <v>999.99</v>
+      </c>
     </row>
     <row r="62" ht="18" customHeight="1">
       <c r="B62" s="15" t="n">
@@ -11518,6 +11828,9 @@
       <c r="AD63" s="34" t="n">
         <v>1658.99</v>
       </c>
+      <c r="AE63" s="34" t="n">
+        <v>1658.99</v>
+      </c>
     </row>
     <row r="64" ht="18" customHeight="1">
       <c r="B64" s="15" t="n">
@@ -11627,6 +11940,9 @@
         </is>
       </c>
       <c r="AD64" s="34" t="n">
+        <v>2549.99</v>
+      </c>
+      <c r="AE64" s="34" t="n">
         <v>2549.99</v>
       </c>
     </row>
@@ -11915,6 +12231,11 @@
       </c>
       <c r="AD70" s="34" t="n">
         <v>1899.99</v>
+      </c>
+      <c r="AE70" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Price check — 03/27/2026
</commit_message>
<xml_diff>
--- a/PriceBook_Combined_Final.xlsx
+++ b/PriceBook_Combined_Final.xlsx
@@ -709,7 +709,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:AE67"/>
+  <dimension ref="B1:AF67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -743,6 +743,7 @@
     <col width="12" customWidth="1" min="29" max="29"/>
     <col width="12" customWidth="1" min="30" max="30"/>
     <col width="12" customWidth="1" min="31" max="31"/>
+    <col width="12" customWidth="1" min="32" max="32"/>
   </cols>
   <sheetData>
     <row r="1" ht="8" customHeight="1"/>
@@ -912,6 +913,11 @@
           <t>3/26</t>
         </is>
       </c>
+      <c r="AF5" s="33" t="inlineStr">
+        <is>
+          <t>3/27</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="22" customHeight="1">
       <c r="B6" s="5" t="inlineStr">
@@ -1027,6 +1033,9 @@
       <c r="AE7" s="34" t="n">
         <v>449.99</v>
       </c>
+      <c r="AF7" s="34" t="n">
+        <v>449.99</v>
+      </c>
     </row>
     <row r="8" ht="18" customHeight="1">
       <c r="B8" s="15" t="n">
@@ -1159,6 +1168,11 @@
       <c r="AE8" s="36" t="n">
         <v>809.99</v>
       </c>
+      <c r="AF8" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="18" customHeight="1">
       <c r="B9" s="6" t="n">
@@ -1291,6 +1305,11 @@
       <c r="AE9" s="36" t="n">
         <v>809.99</v>
       </c>
+      <c r="AF9" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="18" customHeight="1">
       <c r="B10" s="15" t="n">
@@ -1399,6 +1418,9 @@
       <c r="AE10" s="34" t="n">
         <v>449.99</v>
       </c>
+      <c r="AF10" s="34" t="n">
+        <v>449.99</v>
+      </c>
     </row>
     <row r="11" ht="18" customHeight="1">
       <c r="B11" s="6" t="n">
@@ -1531,6 +1553,11 @@
       <c r="AE11" s="36" t="n">
         <v>809.99</v>
       </c>
+      <c r="AF11" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="18" customHeight="1">
       <c r="B12" s="15" t="n">
@@ -1643,6 +1670,9 @@
       <c r="AE12" s="36" t="n">
         <v>839.99</v>
       </c>
+      <c r="AF12" s="36" t="n">
+        <v>839.99</v>
+      </c>
     </row>
     <row r="13" ht="5" customHeight="1"/>
     <row r="14" ht="22" customHeight="1">
@@ -1771,6 +1801,11 @@
       <c r="AE15" s="34" t="n">
         <v>599.99</v>
       </c>
+      <c r="AF15" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="18" customHeight="1">
       <c r="B16" s="15" t="n">
@@ -1887,6 +1922,9 @@
       <c r="AE16" s="36" t="n">
         <v>809.99</v>
       </c>
+      <c r="AF16" s="36" t="n">
+        <v>809.99</v>
+      </c>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="B17" s="6" t="n">
@@ -2019,6 +2057,11 @@
         </is>
       </c>
       <c r="AE17" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AF17" s="35" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2195,6 +2238,9 @@
       <c r="AE19" s="34" t="n">
         <v>2199.99</v>
       </c>
+      <c r="AF19" s="34" t="n">
+        <v>2199.99</v>
+      </c>
     </row>
     <row r="20" ht="5" customHeight="1"/>
     <row r="21" ht="22" customHeight="1">
@@ -2319,6 +2365,9 @@
       <c r="AE22" s="34" t="n">
         <v>1098.99</v>
       </c>
+      <c r="AF22" s="34" t="n">
+        <v>1098.99</v>
+      </c>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="B23" s="6" t="n">
@@ -2437,6 +2486,9 @@
       <c r="AE23" s="34" t="n">
         <v>1199.99</v>
       </c>
+      <c r="AF23" s="34" t="n">
+        <v>1198.99</v>
+      </c>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="B24" s="15" t="n">
@@ -2554,6 +2606,9 @@
       </c>
       <c r="AE24" s="34" t="n">
         <v>1199.99</v>
+      </c>
+      <c r="AF24" s="34" t="n">
+        <v>1198.99</v>
       </c>
     </row>
     <row r="25" ht="18" customHeight="1">
@@ -2733,6 +2788,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AF26" s="34" t="n">
+        <v>1599.99</v>
+      </c>
     </row>
     <row r="27" ht="18" customHeight="1">
       <c r="B27" s="6" t="n">
@@ -2849,6 +2907,9 @@
       <c r="AE27" s="34" t="n">
         <v>1799.99</v>
       </c>
+      <c r="AF27" s="34" t="n">
+        <v>1799.99</v>
+      </c>
     </row>
     <row r="28" ht="18" customHeight="1">
       <c r="B28" s="15" t="n">
@@ -2961,6 +3022,9 @@
       <c r="AE28" s="34" t="n">
         <v>1479.99</v>
       </c>
+      <c r="AF28" s="34" t="n">
+        <v>1479.99</v>
+      </c>
     </row>
     <row r="29" ht="18" customHeight="1">
       <c r="B29" s="6" t="n">
@@ -3077,6 +3141,9 @@
       <c r="AE29" s="34" t="n">
         <v>1799.99</v>
       </c>
+      <c r="AF29" s="34" t="n">
+        <v>1799.99</v>
+      </c>
     </row>
     <row r="30" ht="18" customHeight="1">
       <c r="B30" s="15" t="n">
@@ -3193,6 +3260,9 @@
       <c r="AE30" s="34" t="n">
         <v>1799.99</v>
       </c>
+      <c r="AF30" s="34" t="n">
+        <v>1799.99</v>
+      </c>
     </row>
     <row r="31" ht="5" customHeight="1"/>
     <row r="32" ht="22" customHeight="1">
@@ -3317,6 +3387,9 @@
       <c r="AE33" s="34" t="n">
         <v>1029.99</v>
       </c>
+      <c r="AF33" s="34" t="n">
+        <v>1029.99</v>
+      </c>
     </row>
     <row r="34" ht="18" customHeight="1">
       <c r="B34" s="15" t="n">
@@ -3433,6 +3506,9 @@
       <c r="AE34" s="34" t="n">
         <v>1029.99</v>
       </c>
+      <c r="AF34" s="34" t="n">
+        <v>1029.99</v>
+      </c>
     </row>
     <row r="35" ht="18" customHeight="1">
       <c r="B35" s="6" t="n">
@@ -3555,6 +3631,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AF35" s="34" t="n">
+        <v>1599.99</v>
+      </c>
     </row>
     <row r="36" ht="18" customHeight="1">
       <c r="B36" s="15" t="n">
@@ -3675,6 +3754,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AF36" s="34" t="n">
+        <v>1699.99</v>
+      </c>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="B37" s="6" t="n">
@@ -3789,6 +3871,9 @@
       <c r="AE37" s="36" t="n">
         <v>3399.99</v>
       </c>
+      <c r="AF37" s="36" t="n">
+        <v>3399.99</v>
+      </c>
     </row>
     <row r="38" ht="18" customHeight="1">
       <c r="B38" s="15" t="n">
@@ -3905,6 +3990,9 @@
       <c r="AE38" s="34" t="n">
         <v>2898.99</v>
       </c>
+      <c r="AF38" s="34" t="n">
+        <v>2898.99</v>
+      </c>
     </row>
     <row r="39" ht="18" customHeight="1">
       <c r="B39" s="6" t="n">
@@ -4019,6 +4107,9 @@
       <c r="AE39" s="36" t="n">
         <v>3399.99</v>
       </c>
+      <c r="AF39" s="36" t="n">
+        <v>3399.99</v>
+      </c>
     </row>
     <row r="40" ht="18" customHeight="1">
       <c r="B40" s="15" t="n">
@@ -4135,6 +4226,9 @@
       <c r="AE40" s="34" t="n">
         <v>1029.99</v>
       </c>
+      <c r="AF40" s="34" t="n">
+        <v>1029.99</v>
+      </c>
     </row>
     <row r="41" ht="18" customHeight="1">
       <c r="B41" s="6" t="n">
@@ -4251,6 +4345,9 @@
       <c r="AE41" s="34" t="n">
         <v>1749.99</v>
       </c>
+      <c r="AF41" s="36" t="n">
+        <v>2159.99</v>
+      </c>
     </row>
     <row r="42" ht="18" customHeight="1">
       <c r="B42" s="15" t="n">
@@ -4373,6 +4470,9 @@
         <v>1899.99</v>
       </c>
       <c r="AE42" s="36" t="n">
+        <v>1999.99</v>
+      </c>
+      <c r="AF42" s="36" t="n">
         <v>1999.99</v>
       </c>
     </row>
@@ -4545,6 +4645,9 @@
       <c r="AE44" s="34" t="n">
         <v>3599.99</v>
       </c>
+      <c r="AF44" s="34" t="n">
+        <v>3599.99</v>
+      </c>
     </row>
     <row r="45" ht="5" customHeight="1"/>
     <row r="46" ht="22" customHeight="1">
@@ -4677,6 +4780,9 @@
       <c r="AE47" s="36" t="n">
         <v>1999.99</v>
       </c>
+      <c r="AF47" s="36" t="n">
+        <v>1999.99</v>
+      </c>
     </row>
     <row r="48" ht="18" customHeight="1">
       <c r="B48" s="15" t="n">
@@ -4799,6 +4905,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AF48" s="34" t="n">
+        <v>1599.99</v>
+      </c>
     </row>
     <row r="49" ht="18" customHeight="1">
       <c r="B49" s="6" t="n">
@@ -4917,6 +5026,9 @@
       <c r="AE49" s="34" t="n">
         <v>1849.99</v>
       </c>
+      <c r="AF49" s="34" t="n">
+        <v>1849.99</v>
+      </c>
     </row>
     <row r="50" ht="18" customHeight="1">
       <c r="B50" s="15" t="n">
@@ -5027,6 +5139,9 @@
         <v>2599.99</v>
       </c>
       <c r="AE50" s="34" t="n">
+        <v>2599.99</v>
+      </c>
+      <c r="AF50" s="34" t="n">
         <v>2599.99</v>
       </c>
     </row>
@@ -5197,6 +5312,9 @@
       <c r="AE52" s="34" t="n">
         <v>2599.99</v>
       </c>
+      <c r="AF52" s="34" t="n">
+        <v>2599.99</v>
+      </c>
     </row>
     <row r="53" ht="18" customHeight="1">
       <c r="B53" s="6" t="n">
@@ -5313,6 +5431,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AF53" s="13" t="n">
+        <v>1899.99</v>
+      </c>
     </row>
     <row r="54" ht="5" customHeight="1"/>
     <row r="55" ht="22" customHeight="1">
@@ -5433,6 +5554,9 @@
         <v>3599.99</v>
       </c>
       <c r="AE56" s="34" t="n">
+        <v>3599.99</v>
+      </c>
+      <c r="AF56" s="34" t="n">
         <v>3599.99</v>
       </c>
     </row>
@@ -5727,6 +5851,9 @@
       <c r="AE62" s="34" t="n">
         <v>127.99</v>
       </c>
+      <c r="AF62" s="34" t="n">
+        <v>127.99</v>
+      </c>
     </row>
     <row r="63" ht="18" customHeight="1">
       <c r="B63" s="6" t="n">
@@ -5857,6 +5984,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AF63" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="64" ht="18" customHeight="1">
       <c r="B64" s="15" t="n">
@@ -5980,6 +6112,9 @@
         <is>
           <t>—</t>
         </is>
+      </c>
+      <c r="AF64" s="36" t="n">
+        <v>479.99</v>
       </c>
     </row>
     <row r="65" ht="18" customHeight="1">
@@ -6213,7 +6348,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:AE70"/>
+  <dimension ref="B1:AF70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -6247,6 +6382,7 @@
     <col width="12" customWidth="1" min="29" max="29"/>
     <col width="12" customWidth="1" min="30" max="30"/>
     <col width="12" customWidth="1" min="31" max="31"/>
+    <col width="12" customWidth="1" min="32" max="32"/>
   </cols>
   <sheetData>
     <row r="1" ht="8" customHeight="1"/>
@@ -6416,6 +6552,11 @@
           <t>3/26</t>
         </is>
       </c>
+      <c r="AF5" s="33" t="inlineStr">
+        <is>
+          <t>3/27</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="22" customHeight="1">
       <c r="B6" s="5" t="inlineStr">
@@ -6541,6 +6682,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AF7" s="34" t="n">
+        <v>89.98999999999999</v>
+      </c>
     </row>
     <row r="8" ht="18" customHeight="1">
       <c r="B8" s="15" t="n">
@@ -6655,6 +6799,9 @@
       <c r="AE8" s="34" t="n">
         <v>194.99</v>
       </c>
+      <c r="AF8" s="34" t="n">
+        <v>194.99</v>
+      </c>
     </row>
     <row r="9" ht="18" customHeight="1">
       <c r="B9" s="6" t="n">
@@ -6785,6 +6932,11 @@
         </is>
       </c>
       <c r="AE9" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AF9" s="35" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -6955,6 +7107,9 @@
       <c r="AE11" s="34" t="n">
         <v>219.99</v>
       </c>
+      <c r="AF11" s="34" t="n">
+        <v>219.99</v>
+      </c>
     </row>
     <row r="12" ht="18" customHeight="1">
       <c r="B12" s="15" t="n">
@@ -7073,6 +7228,9 @@
       <c r="AE12" s="34" t="n">
         <v>349.99</v>
       </c>
+      <c r="AF12" s="34" t="n">
+        <v>349.99</v>
+      </c>
     </row>
     <row r="13" ht="18" customHeight="1">
       <c r="B13" s="6" t="n">
@@ -7205,6 +7363,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AF13" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="5" customHeight="1"/>
     <row r="15" ht="22" customHeight="1">
@@ -7347,6 +7510,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AF16" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="B17" s="6" t="n">
@@ -7459,6 +7627,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AF17" s="34" t="n">
+        <v>279.99</v>
+      </c>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="B18" s="15" t="n">
@@ -7577,6 +7748,9 @@
       <c r="AE18" s="34" t="n">
         <v>399.99</v>
       </c>
+      <c r="AF18" s="34" t="n">
+        <v>399.99</v>
+      </c>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="B19" s="6" t="n">
@@ -7695,6 +7869,9 @@
       <c r="AE19" s="34" t="n">
         <v>249.99</v>
       </c>
+      <c r="AF19" s="34" t="n">
+        <v>249.99</v>
+      </c>
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="B20" s="15" t="n">
@@ -7811,6 +7988,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AF20" s="34" t="n">
+        <v>427.99</v>
+      </c>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="B21" s="6" t="n">
@@ -7919,6 +8099,9 @@
       <c r="AE21" s="34" t="n">
         <v>478.99</v>
       </c>
+      <c r="AF21" s="13" t="n">
+        <v>449.99</v>
+      </c>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="B22" s="15" t="n">
@@ -8043,6 +8226,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AF22" s="34" t="n">
+        <v>599.99</v>
+      </c>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="B23" s="6" t="n">
@@ -8159,6 +8345,9 @@
       <c r="AE23" s="34" t="n">
         <v>999.99</v>
       </c>
+      <c r="AF23" s="34" t="n">
+        <v>999.99</v>
+      </c>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="B24" s="15" t="n">
@@ -8291,6 +8480,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AF24" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="18" customHeight="1">
       <c r="B25" s="6" t="n">
@@ -8413,6 +8607,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AF25" s="34" t="n">
+        <v>1199.99</v>
+      </c>
     </row>
     <row r="26" ht="18" customHeight="1">
       <c r="B26" s="15" t="n">
@@ -8527,6 +8724,9 @@
       <c r="AE26" s="34" t="n">
         <v>1274.99</v>
       </c>
+      <c r="AF26" s="34" t="n">
+        <v>1274.99</v>
+      </c>
     </row>
     <row r="27" ht="5" customHeight="1"/>
     <row r="28" ht="22" customHeight="1">
@@ -8655,6 +8855,9 @@
       <c r="AE29" s="34" t="n">
         <v>369.99</v>
       </c>
+      <c r="AF29" s="34" t="n">
+        <v>369.99</v>
+      </c>
     </row>
     <row r="30" ht="18" customHeight="1">
       <c r="B30" s="15" t="n">
@@ -8773,6 +8976,9 @@
       <c r="AE30" s="34" t="n">
         <v>579.99</v>
       </c>
+      <c r="AF30" s="34" t="n">
+        <v>579.99</v>
+      </c>
     </row>
     <row r="31" ht="18" customHeight="1">
       <c r="B31" s="6" t="n">
@@ -8893,6 +9099,9 @@
       <c r="AE31" s="13" t="n">
         <v>699.99</v>
       </c>
+      <c r="AF31" s="13" t="n">
+        <v>699.99</v>
+      </c>
     </row>
     <row r="32" ht="18" customHeight="1">
       <c r="B32" s="15" t="n">
@@ -9009,6 +9218,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AF32" s="34" t="n">
+        <v>759.99</v>
+      </c>
     </row>
     <row r="33" ht="18" customHeight="1">
       <c r="B33" s="6" t="n">
@@ -9129,6 +9341,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AF33" s="34" t="n">
+        <v>799.99</v>
+      </c>
     </row>
     <row r="34" ht="18" customHeight="1">
       <c r="B34" s="15" t="n">
@@ -9243,6 +9458,9 @@
       <c r="AE34" s="34" t="n">
         <v>1274.99</v>
       </c>
+      <c r="AF34" s="34" t="n">
+        <v>1274.99</v>
+      </c>
     </row>
     <row r="35" ht="18" customHeight="1">
       <c r="B35" s="6" t="n">
@@ -9359,6 +9577,9 @@
       <c r="AE35" s="34" t="n">
         <v>1799.99</v>
       </c>
+      <c r="AF35" s="34" t="n">
+        <v>1799.99</v>
+      </c>
     </row>
     <row r="36" ht="18" customHeight="1">
       <c r="B36" s="15" t="n">
@@ -9471,6 +9692,9 @@
       <c r="AE36" s="34" t="n">
         <v>1975.99</v>
       </c>
+      <c r="AF36" s="34" t="n">
+        <v>1975.99</v>
+      </c>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="B37" s="6" t="n">
@@ -9591,6 +9815,9 @@
       <c r="AE37" s="34" t="n">
         <v>2699.99</v>
       </c>
+      <c r="AF37" s="34" t="n">
+        <v>2699.99</v>
+      </c>
     </row>
     <row r="38" ht="5" customHeight="1"/>
     <row r="39" ht="22" customHeight="1">
@@ -9715,6 +9942,11 @@
       <c r="AE40" s="34" t="n">
         <v>740.99</v>
       </c>
+      <c r="AF40" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="18" customHeight="1">
       <c r="B41" s="6" t="n">
@@ -9835,6 +10067,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AF41" s="13" t="n">
+        <v>599.99</v>
+      </c>
     </row>
     <row r="42" ht="18" customHeight="1">
       <c r="B42" s="15" t="n">
@@ -9955,6 +10190,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AF42" s="34" t="n">
+        <v>799.99</v>
+      </c>
     </row>
     <row r="43" ht="18" customHeight="1">
       <c r="B43" s="6" t="n">
@@ -10077,6 +10315,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AF43" s="34" t="n">
+        <v>949.99</v>
+      </c>
     </row>
     <row r="44" ht="18" customHeight="1">
       <c r="B44" s="15" t="n">
@@ -10187,6 +10428,9 @@
       <c r="AE44" s="34" t="n">
         <v>1139.99</v>
       </c>
+      <c r="AF44" s="34" t="n">
+        <v>1139.99</v>
+      </c>
     </row>
     <row r="45" ht="18" customHeight="1">
       <c r="B45" s="6" t="n">
@@ -10299,6 +10543,9 @@
       <c r="AE45" s="34" t="n">
         <v>1529.99</v>
       </c>
+      <c r="AF45" s="34" t="n">
+        <v>1529.99</v>
+      </c>
     </row>
     <row r="46" ht="18" customHeight="1">
       <c r="B46" s="15" t="n">
@@ -10431,6 +10678,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AF46" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="47" ht="18" customHeight="1">
       <c r="B47" s="6" t="n">
@@ -10547,6 +10799,9 @@
       <c r="AE47" s="34" t="n">
         <v>2999.99</v>
       </c>
+      <c r="AF47" s="34" t="n">
+        <v>2999.99</v>
+      </c>
     </row>
     <row r="48" ht="18" customHeight="1">
       <c r="B48" s="15" t="n">
@@ -10667,6 +10922,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AF48" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="49" ht="5" customHeight="1"/>
     <row r="50" ht="22" customHeight="1">
@@ -10789,6 +11049,9 @@
       <c r="AE51" s="34" t="n">
         <v>798.99</v>
       </c>
+      <c r="AF51" s="34" t="n">
+        <v>798.99</v>
+      </c>
     </row>
     <row r="52" ht="18" customHeight="1">
       <c r="B52" s="15" t="n">
@@ -10903,6 +11166,9 @@
       <c r="AE52" s="34" t="n">
         <v>798.99</v>
       </c>
+      <c r="AF52" s="34" t="n">
+        <v>798.99</v>
+      </c>
     </row>
     <row r="53" ht="18" customHeight="1">
       <c r="B53" s="6" t="n">
@@ -11019,6 +11285,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AF53" s="34" t="n">
+        <v>1499.99</v>
+      </c>
     </row>
     <row r="54" ht="18" customHeight="1">
       <c r="B54" s="15" t="n">
@@ -11129,6 +11398,11 @@
       <c r="AE54" s="34" t="n">
         <v>899.99</v>
       </c>
+      <c r="AF54" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="55" ht="18" customHeight="1">
       <c r="B55" s="6" t="n">
@@ -11245,6 +11519,9 @@
       <c r="AE55" s="13" t="n">
         <v>1299.99</v>
       </c>
+      <c r="AF55" s="13" t="n">
+        <v>1299.99</v>
+      </c>
     </row>
     <row r="56" ht="18" customHeight="1">
       <c r="B56" s="15" t="n">
@@ -11363,6 +11640,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AF56" s="34" t="n">
+        <v>2799.99</v>
+      </c>
     </row>
     <row r="57" ht="18" customHeight="1">
       <c r="B57" s="6" t="n">
@@ -11475,6 +11755,9 @@
         <v>3199.99</v>
       </c>
       <c r="AE57" s="34" t="n">
+        <v>3199.99</v>
+      </c>
+      <c r="AF57" s="34" t="n">
         <v>3199.99</v>
       </c>
     </row>
@@ -11657,6 +11940,9 @@
       <c r="AE61" s="34" t="n">
         <v>999.99</v>
       </c>
+      <c r="AF61" s="34" t="n">
+        <v>999.99</v>
+      </c>
     </row>
     <row r="62" ht="18" customHeight="1">
       <c r="B62" s="15" t="n">
@@ -11831,6 +12117,9 @@
       <c r="AE63" s="34" t="n">
         <v>1658.99</v>
       </c>
+      <c r="AF63" s="34" t="n">
+        <v>1658.99</v>
+      </c>
     </row>
     <row r="64" ht="18" customHeight="1">
       <c r="B64" s="15" t="n">
@@ -11943,6 +12232,9 @@
         <v>2549.99</v>
       </c>
       <c r="AE64" s="34" t="n">
+        <v>2549.99</v>
+      </c>
+      <c r="AF64" s="34" t="n">
         <v>2549.99</v>
       </c>
     </row>
@@ -12236,6 +12528,9 @@
         <is>
           <t>—</t>
         </is>
+      </c>
+      <c r="AF70" s="34" t="n">
+        <v>1899.99</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Price check — 03/28/2026
</commit_message>
<xml_diff>
--- a/PriceBook_Combined_Final.xlsx
+++ b/PriceBook_Combined_Final.xlsx
@@ -709,7 +709,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:AF67"/>
+  <dimension ref="B1:AG67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -744,6 +744,7 @@
     <col width="12" customWidth="1" min="30" max="30"/>
     <col width="12" customWidth="1" min="31" max="31"/>
     <col width="12" customWidth="1" min="32" max="32"/>
+    <col width="12" customWidth="1" min="33" max="33"/>
   </cols>
   <sheetData>
     <row r="1" ht="8" customHeight="1"/>
@@ -918,6 +919,11 @@
           <t>3/27</t>
         </is>
       </c>
+      <c r="AG5" s="33" t="inlineStr">
+        <is>
+          <t>3/28</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="22" customHeight="1">
       <c r="B6" s="5" t="inlineStr">
@@ -1036,6 +1042,9 @@
       <c r="AF7" s="34" t="n">
         <v>449.99</v>
       </c>
+      <c r="AG7" s="34" t="n">
+        <v>449.99</v>
+      </c>
     </row>
     <row r="8" ht="18" customHeight="1">
       <c r="B8" s="15" t="n">
@@ -1173,6 +1182,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AG8" s="36" t="n">
+        <v>809.99</v>
+      </c>
     </row>
     <row r="9" ht="18" customHeight="1">
       <c r="B9" s="6" t="n">
@@ -1310,6 +1322,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AG9" s="36" t="n">
+        <v>809.99</v>
+      </c>
     </row>
     <row r="10" ht="18" customHeight="1">
       <c r="B10" s="15" t="n">
@@ -1421,6 +1436,9 @@
       <c r="AF10" s="34" t="n">
         <v>449.99</v>
       </c>
+      <c r="AG10" s="34" t="n">
+        <v>449.99</v>
+      </c>
     </row>
     <row r="11" ht="18" customHeight="1">
       <c r="B11" s="6" t="n">
@@ -1558,6 +1576,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AG11" s="36" t="n">
+        <v>809.99</v>
+      </c>
     </row>
     <row r="12" ht="18" customHeight="1">
       <c r="B12" s="15" t="n">
@@ -1673,6 +1694,9 @@
       <c r="AF12" s="36" t="n">
         <v>839.99</v>
       </c>
+      <c r="AG12" s="36" t="n">
+        <v>839.99</v>
+      </c>
     </row>
     <row r="13" ht="5" customHeight="1"/>
     <row r="14" ht="22" customHeight="1">
@@ -1806,6 +1830,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AG15" s="34" t="n">
+        <v>599.99</v>
+      </c>
     </row>
     <row r="16" ht="18" customHeight="1">
       <c r="B16" s="15" t="n">
@@ -1925,6 +1952,11 @@
       <c r="AF16" s="36" t="n">
         <v>809.99</v>
       </c>
+      <c r="AG16" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="B17" s="6" t="n">
@@ -2062,6 +2094,11 @@
         </is>
       </c>
       <c r="AF17" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AG17" s="35" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2241,6 +2278,9 @@
       <c r="AF19" s="34" t="n">
         <v>2199.99</v>
       </c>
+      <c r="AG19" s="34" t="n">
+        <v>2199.99</v>
+      </c>
     </row>
     <row r="20" ht="5" customHeight="1"/>
     <row r="21" ht="22" customHeight="1">
@@ -2368,6 +2408,9 @@
       <c r="AF22" s="34" t="n">
         <v>1098.99</v>
       </c>
+      <c r="AG22" s="34" t="n">
+        <v>1098.99</v>
+      </c>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="B23" s="6" t="n">
@@ -2489,6 +2532,9 @@
       <c r="AF23" s="34" t="n">
         <v>1198.99</v>
       </c>
+      <c r="AG23" s="34" t="n">
+        <v>1198.99</v>
+      </c>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="B24" s="15" t="n">
@@ -2608,6 +2654,9 @@
         <v>1199.99</v>
       </c>
       <c r="AF24" s="34" t="n">
+        <v>1198.99</v>
+      </c>
+      <c r="AG24" s="34" t="n">
         <v>1198.99</v>
       </c>
     </row>
@@ -2791,6 +2840,9 @@
       <c r="AF26" s="34" t="n">
         <v>1599.99</v>
       </c>
+      <c r="AG26" s="34" t="n">
+        <v>1599.99</v>
+      </c>
     </row>
     <row r="27" ht="18" customHeight="1">
       <c r="B27" s="6" t="n">
@@ -2910,6 +2962,9 @@
       <c r="AF27" s="34" t="n">
         <v>1799.99</v>
       </c>
+      <c r="AG27" s="34" t="n">
+        <v>1799.99</v>
+      </c>
     </row>
     <row r="28" ht="18" customHeight="1">
       <c r="B28" s="15" t="n">
@@ -3025,6 +3080,9 @@
       <c r="AF28" s="34" t="n">
         <v>1479.99</v>
       </c>
+      <c r="AG28" s="34" t="n">
+        <v>1479.99</v>
+      </c>
     </row>
     <row r="29" ht="18" customHeight="1">
       <c r="B29" s="6" t="n">
@@ -3144,6 +3202,9 @@
       <c r="AF29" s="34" t="n">
         <v>1799.99</v>
       </c>
+      <c r="AG29" s="34" t="n">
+        <v>1799.99</v>
+      </c>
     </row>
     <row r="30" ht="18" customHeight="1">
       <c r="B30" s="15" t="n">
@@ -3263,6 +3324,9 @@
       <c r="AF30" s="34" t="n">
         <v>1799.99</v>
       </c>
+      <c r="AG30" s="34" t="n">
+        <v>1799.99</v>
+      </c>
     </row>
     <row r="31" ht="5" customHeight="1"/>
     <row r="32" ht="22" customHeight="1">
@@ -3390,6 +3454,9 @@
       <c r="AF33" s="34" t="n">
         <v>1029.99</v>
       </c>
+      <c r="AG33" s="34" t="n">
+        <v>1029.99</v>
+      </c>
     </row>
     <row r="34" ht="18" customHeight="1">
       <c r="B34" s="15" t="n">
@@ -3509,6 +3576,9 @@
       <c r="AF34" s="34" t="n">
         <v>1029.99</v>
       </c>
+      <c r="AG34" s="34" t="n">
+        <v>1029.99</v>
+      </c>
     </row>
     <row r="35" ht="18" customHeight="1">
       <c r="B35" s="6" t="n">
@@ -3634,6 +3704,9 @@
       <c r="AF35" s="34" t="n">
         <v>1599.99</v>
       </c>
+      <c r="AG35" s="34" t="n">
+        <v>1599.99</v>
+      </c>
     </row>
     <row r="36" ht="18" customHeight="1">
       <c r="B36" s="15" t="n">
@@ -3757,6 +3830,9 @@
       <c r="AF36" s="34" t="n">
         <v>1699.99</v>
       </c>
+      <c r="AG36" s="34" t="n">
+        <v>1699.99</v>
+      </c>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="B37" s="6" t="n">
@@ -3874,6 +3950,9 @@
       <c r="AF37" s="36" t="n">
         <v>3399.99</v>
       </c>
+      <c r="AG37" s="36" t="n">
+        <v>3399.99</v>
+      </c>
     </row>
     <row r="38" ht="18" customHeight="1">
       <c r="B38" s="15" t="n">
@@ -3993,6 +4072,9 @@
       <c r="AF38" s="34" t="n">
         <v>2898.99</v>
       </c>
+      <c r="AG38" s="34" t="n">
+        <v>2898.99</v>
+      </c>
     </row>
     <row r="39" ht="18" customHeight="1">
       <c r="B39" s="6" t="n">
@@ -4110,6 +4192,9 @@
       <c r="AF39" s="36" t="n">
         <v>3399.99</v>
       </c>
+      <c r="AG39" s="36" t="n">
+        <v>3399.99</v>
+      </c>
     </row>
     <row r="40" ht="18" customHeight="1">
       <c r="B40" s="15" t="n">
@@ -4229,6 +4314,9 @@
       <c r="AF40" s="34" t="n">
         <v>1029.99</v>
       </c>
+      <c r="AG40" s="34" t="n">
+        <v>1029.99</v>
+      </c>
     </row>
     <row r="41" ht="18" customHeight="1">
       <c r="B41" s="6" t="n">
@@ -4348,6 +4436,9 @@
       <c r="AF41" s="36" t="n">
         <v>2159.99</v>
       </c>
+      <c r="AG41" s="36" t="n">
+        <v>2159.99</v>
+      </c>
     </row>
     <row r="42" ht="18" customHeight="1">
       <c r="B42" s="15" t="n">
@@ -4474,6 +4565,11 @@
       </c>
       <c r="AF42" s="36" t="n">
         <v>1999.99</v>
+      </c>
+      <c r="AG42" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
     </row>
     <row r="43" ht="18" customHeight="1">
@@ -4648,6 +4744,9 @@
       <c r="AF44" s="34" t="n">
         <v>3599.99</v>
       </c>
+      <c r="AG44" s="34" t="n">
+        <v>3599.99</v>
+      </c>
     </row>
     <row r="45" ht="5" customHeight="1"/>
     <row r="46" ht="22" customHeight="1">
@@ -4783,6 +4882,11 @@
       <c r="AF47" s="36" t="n">
         <v>1999.99</v>
       </c>
+      <c r="AG47" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="48" ht="18" customHeight="1">
       <c r="B48" s="15" t="n">
@@ -4908,6 +5012,9 @@
       <c r="AF48" s="34" t="n">
         <v>1599.99</v>
       </c>
+      <c r="AG48" s="34" t="n">
+        <v>1599.99</v>
+      </c>
     </row>
     <row r="49" ht="18" customHeight="1">
       <c r="B49" s="6" t="n">
@@ -5029,6 +5136,9 @@
       <c r="AF49" s="34" t="n">
         <v>1849.99</v>
       </c>
+      <c r="AG49" s="34" t="n">
+        <v>1849.99</v>
+      </c>
     </row>
     <row r="50" ht="18" customHeight="1">
       <c r="B50" s="15" t="n">
@@ -5143,6 +5253,11 @@
       </c>
       <c r="AF50" s="34" t="n">
         <v>2599.99</v>
+      </c>
+      <c r="AG50" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
     </row>
     <row r="51" ht="18" customHeight="1">
@@ -5315,6 +5430,11 @@
       <c r="AF52" s="34" t="n">
         <v>2599.99</v>
       </c>
+      <c r="AG52" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="53" ht="18" customHeight="1">
       <c r="B53" s="6" t="n">
@@ -5434,6 +5554,9 @@
       <c r="AF53" s="13" t="n">
         <v>1899.99</v>
       </c>
+      <c r="AG53" s="13" t="n">
+        <v>1899.99</v>
+      </c>
     </row>
     <row r="54" ht="5" customHeight="1"/>
     <row r="55" ht="22" customHeight="1">
@@ -5557,6 +5680,9 @@
         <v>3599.99</v>
       </c>
       <c r="AF56" s="34" t="n">
+        <v>3599.99</v>
+      </c>
+      <c r="AG56" s="34" t="n">
         <v>3599.99</v>
       </c>
     </row>
@@ -5854,6 +5980,9 @@
       <c r="AF62" s="34" t="n">
         <v>127.99</v>
       </c>
+      <c r="AG62" s="34" t="n">
+        <v>127.99</v>
+      </c>
     </row>
     <row r="63" ht="18" customHeight="1">
       <c r="B63" s="6" t="n">
@@ -5989,6 +6118,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AG63" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="64" ht="18" customHeight="1">
       <c r="B64" s="15" t="n">
@@ -6114,6 +6248,9 @@
         </is>
       </c>
       <c r="AF64" s="36" t="n">
+        <v>479.99</v>
+      </c>
+      <c r="AG64" s="36" t="n">
         <v>479.99</v>
       </c>
     </row>
@@ -6348,7 +6485,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:AF70"/>
+  <dimension ref="B1:AG70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -6383,6 +6520,7 @@
     <col width="12" customWidth="1" min="30" max="30"/>
     <col width="12" customWidth="1" min="31" max="31"/>
     <col width="12" customWidth="1" min="32" max="32"/>
+    <col width="12" customWidth="1" min="33" max="33"/>
   </cols>
   <sheetData>
     <row r="1" ht="8" customHeight="1"/>
@@ -6557,6 +6695,11 @@
           <t>3/27</t>
         </is>
       </c>
+      <c r="AG5" s="33" t="inlineStr">
+        <is>
+          <t>3/28</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="22" customHeight="1">
       <c r="B6" s="5" t="inlineStr">
@@ -6685,6 +6828,9 @@
       <c r="AF7" s="34" t="n">
         <v>89.98999999999999</v>
       </c>
+      <c r="AG7" s="34" t="n">
+        <v>89.98999999999999</v>
+      </c>
     </row>
     <row r="8" ht="18" customHeight="1">
       <c r="B8" s="15" t="n">
@@ -6802,6 +6948,9 @@
       <c r="AF8" s="34" t="n">
         <v>194.99</v>
       </c>
+      <c r="AG8" s="34" t="n">
+        <v>194.99</v>
+      </c>
     </row>
     <row r="9" ht="18" customHeight="1">
       <c r="B9" s="6" t="n">
@@ -6937,6 +7086,11 @@
         </is>
       </c>
       <c r="AF9" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AG9" s="35" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -7110,6 +7264,9 @@
       <c r="AF11" s="34" t="n">
         <v>219.99</v>
       </c>
+      <c r="AG11" s="34" t="n">
+        <v>219.99</v>
+      </c>
     </row>
     <row r="12" ht="18" customHeight="1">
       <c r="B12" s="15" t="n">
@@ -7231,6 +7388,9 @@
       <c r="AF12" s="34" t="n">
         <v>349.99</v>
       </c>
+      <c r="AG12" s="34" t="n">
+        <v>349.99</v>
+      </c>
     </row>
     <row r="13" ht="18" customHeight="1">
       <c r="B13" s="6" t="n">
@@ -7368,6 +7528,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AG13" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="5" customHeight="1"/>
     <row r="15" ht="22" customHeight="1">
@@ -7515,6 +7680,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AG16" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="B17" s="6" t="n">
@@ -7630,6 +7800,9 @@
       <c r="AF17" s="34" t="n">
         <v>279.99</v>
       </c>
+      <c r="AG17" s="34" t="n">
+        <v>279.99</v>
+      </c>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="B18" s="15" t="n">
@@ -7751,6 +7924,9 @@
       <c r="AF18" s="34" t="n">
         <v>399.99</v>
       </c>
+      <c r="AG18" s="34" t="n">
+        <v>399.99</v>
+      </c>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="B19" s="6" t="n">
@@ -7872,6 +8048,11 @@
       <c r="AF19" s="34" t="n">
         <v>249.99</v>
       </c>
+      <c r="AG19" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="B20" s="15" t="n">
@@ -7991,6 +8172,9 @@
       <c r="AF20" s="34" t="n">
         <v>427.99</v>
       </c>
+      <c r="AG20" s="34" t="n">
+        <v>427.99</v>
+      </c>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="B21" s="6" t="n">
@@ -8102,6 +8286,9 @@
       <c r="AF21" s="13" t="n">
         <v>449.99</v>
       </c>
+      <c r="AG21" s="13" t="n">
+        <v>449.99</v>
+      </c>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="B22" s="15" t="n">
@@ -8229,6 +8416,9 @@
       <c r="AF22" s="34" t="n">
         <v>599.99</v>
       </c>
+      <c r="AG22" s="34" t="n">
+        <v>599.99</v>
+      </c>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="B23" s="6" t="n">
@@ -8348,6 +8538,9 @@
       <c r="AF23" s="34" t="n">
         <v>999.99</v>
       </c>
+      <c r="AG23" s="34" t="n">
+        <v>999.99</v>
+      </c>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="B24" s="15" t="n">
@@ -8485,6 +8678,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AG24" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="18" customHeight="1">
       <c r="B25" s="6" t="n">
@@ -8610,6 +8808,9 @@
       <c r="AF25" s="34" t="n">
         <v>1199.99</v>
       </c>
+      <c r="AG25" s="34" t="n">
+        <v>1199.99</v>
+      </c>
     </row>
     <row r="26" ht="18" customHeight="1">
       <c r="B26" s="15" t="n">
@@ -8727,6 +8928,9 @@
       <c r="AF26" s="34" t="n">
         <v>1274.99</v>
       </c>
+      <c r="AG26" s="34" t="n">
+        <v>1274.99</v>
+      </c>
     </row>
     <row r="27" ht="5" customHeight="1"/>
     <row r="28" ht="22" customHeight="1">
@@ -8858,6 +9062,9 @@
       <c r="AF29" s="34" t="n">
         <v>369.99</v>
       </c>
+      <c r="AG29" s="34" t="n">
+        <v>369.99</v>
+      </c>
     </row>
     <row r="30" ht="18" customHeight="1">
       <c r="B30" s="15" t="n">
@@ -8979,6 +9186,9 @@
       <c r="AF30" s="34" t="n">
         <v>579.99</v>
       </c>
+      <c r="AG30" s="34" t="n">
+        <v>579.99</v>
+      </c>
     </row>
     <row r="31" ht="18" customHeight="1">
       <c r="B31" s="6" t="n">
@@ -9102,6 +9312,9 @@
       <c r="AF31" s="13" t="n">
         <v>699.99</v>
       </c>
+      <c r="AG31" s="13" t="n">
+        <v>699.99</v>
+      </c>
     </row>
     <row r="32" ht="18" customHeight="1">
       <c r="B32" s="15" t="n">
@@ -9221,6 +9434,11 @@
       <c r="AF32" s="34" t="n">
         <v>759.99</v>
       </c>
+      <c r="AG32" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="18" customHeight="1">
       <c r="B33" s="6" t="n">
@@ -9344,6 +9562,9 @@
       <c r="AF33" s="34" t="n">
         <v>799.99</v>
       </c>
+      <c r="AG33" s="34" t="n">
+        <v>799.99</v>
+      </c>
     </row>
     <row r="34" ht="18" customHeight="1">
       <c r="B34" s="15" t="n">
@@ -9461,6 +9682,9 @@
       <c r="AF34" s="34" t="n">
         <v>1274.99</v>
       </c>
+      <c r="AG34" s="34" t="n">
+        <v>1274.99</v>
+      </c>
     </row>
     <row r="35" ht="18" customHeight="1">
       <c r="B35" s="6" t="n">
@@ -9580,6 +9804,9 @@
       <c r="AF35" s="34" t="n">
         <v>1799.99</v>
       </c>
+      <c r="AG35" s="34" t="n">
+        <v>1799.99</v>
+      </c>
     </row>
     <row r="36" ht="18" customHeight="1">
       <c r="B36" s="15" t="n">
@@ -9695,6 +9922,9 @@
       <c r="AF36" s="34" t="n">
         <v>1975.99</v>
       </c>
+      <c r="AG36" s="34" t="n">
+        <v>1975.99</v>
+      </c>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="B37" s="6" t="n">
@@ -9818,6 +10048,11 @@
       <c r="AF37" s="34" t="n">
         <v>2699.99</v>
       </c>
+      <c r="AG37" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="5" customHeight="1"/>
     <row r="39" ht="22" customHeight="1">
@@ -9947,6 +10182,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AG40" s="34" t="n">
+        <v>740.99</v>
+      </c>
     </row>
     <row r="41" ht="18" customHeight="1">
       <c r="B41" s="6" t="n">
@@ -10070,6 +10308,11 @@
       <c r="AF41" s="13" t="n">
         <v>599.99</v>
       </c>
+      <c r="AG41" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="18" customHeight="1">
       <c r="B42" s="15" t="n">
@@ -10193,6 +10436,9 @@
       <c r="AF42" s="34" t="n">
         <v>799.99</v>
       </c>
+      <c r="AG42" s="34" t="n">
+        <v>799.99</v>
+      </c>
     </row>
     <row r="43" ht="18" customHeight="1">
       <c r="B43" s="6" t="n">
@@ -10318,6 +10564,9 @@
       <c r="AF43" s="34" t="n">
         <v>949.99</v>
       </c>
+      <c r="AG43" s="34" t="n">
+        <v>949.99</v>
+      </c>
     </row>
     <row r="44" ht="18" customHeight="1">
       <c r="B44" s="15" t="n">
@@ -10431,6 +10680,11 @@
       <c r="AF44" s="34" t="n">
         <v>1139.99</v>
       </c>
+      <c r="AG44" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="45" ht="18" customHeight="1">
       <c r="B45" s="6" t="n">
@@ -10546,6 +10800,9 @@
       <c r="AF45" s="34" t="n">
         <v>1529.99</v>
       </c>
+      <c r="AG45" s="34" t="n">
+        <v>1529.99</v>
+      </c>
     </row>
     <row r="46" ht="18" customHeight="1">
       <c r="B46" s="15" t="n">
@@ -10683,6 +10940,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AG46" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="47" ht="18" customHeight="1">
       <c r="B47" s="6" t="n">
@@ -10802,6 +11064,9 @@
       <c r="AF47" s="34" t="n">
         <v>2999.99</v>
       </c>
+      <c r="AG47" s="34" t="n">
+        <v>2999.99</v>
+      </c>
     </row>
     <row r="48" ht="18" customHeight="1">
       <c r="B48" s="15" t="n">
@@ -10927,6 +11192,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AG48" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="49" ht="5" customHeight="1"/>
     <row r="50" ht="22" customHeight="1">
@@ -11052,6 +11322,9 @@
       <c r="AF51" s="34" t="n">
         <v>798.99</v>
       </c>
+      <c r="AG51" s="34" t="n">
+        <v>798.99</v>
+      </c>
     </row>
     <row r="52" ht="18" customHeight="1">
       <c r="B52" s="15" t="n">
@@ -11169,6 +11442,9 @@
       <c r="AF52" s="34" t="n">
         <v>798.99</v>
       </c>
+      <c r="AG52" s="34" t="n">
+        <v>798.99</v>
+      </c>
     </row>
     <row r="53" ht="18" customHeight="1">
       <c r="B53" s="6" t="n">
@@ -11288,6 +11564,9 @@
       <c r="AF53" s="34" t="n">
         <v>1499.99</v>
       </c>
+      <c r="AG53" s="34" t="n">
+        <v>1499.99</v>
+      </c>
     </row>
     <row r="54" ht="18" customHeight="1">
       <c r="B54" s="15" t="n">
@@ -11403,6 +11682,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AG54" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="55" ht="18" customHeight="1">
       <c r="B55" s="6" t="n">
@@ -11522,6 +11806,9 @@
       <c r="AF55" s="13" t="n">
         <v>1299.99</v>
       </c>
+      <c r="AG55" s="13" t="n">
+        <v>1299.99</v>
+      </c>
     </row>
     <row r="56" ht="18" customHeight="1">
       <c r="B56" s="15" t="n">
@@ -11643,6 +11930,9 @@
       <c r="AF56" s="34" t="n">
         <v>2799.99</v>
       </c>
+      <c r="AG56" s="34" t="n">
+        <v>2799.99</v>
+      </c>
     </row>
     <row r="57" ht="18" customHeight="1">
       <c r="B57" s="6" t="n">
@@ -11758,6 +12048,9 @@
         <v>3199.99</v>
       </c>
       <c r="AF57" s="34" t="n">
+        <v>3199.99</v>
+      </c>
+      <c r="AG57" s="34" t="n">
         <v>3199.99</v>
       </c>
     </row>
@@ -11943,6 +12236,9 @@
       <c r="AF61" s="34" t="n">
         <v>999.99</v>
       </c>
+      <c r="AG61" s="34" t="n">
+        <v>999.99</v>
+      </c>
     </row>
     <row r="62" ht="18" customHeight="1">
       <c r="B62" s="15" t="n">
@@ -12120,6 +12416,9 @@
       <c r="AF63" s="34" t="n">
         <v>1658.99</v>
       </c>
+      <c r="AG63" s="34" t="n">
+        <v>1658.99</v>
+      </c>
     </row>
     <row r="64" ht="18" customHeight="1">
       <c r="B64" s="15" t="n">
@@ -12235,6 +12534,9 @@
         <v>2549.99</v>
       </c>
       <c r="AF64" s="34" t="n">
+        <v>2549.99</v>
+      </c>
+      <c r="AG64" s="34" t="n">
         <v>2549.99</v>
       </c>
     </row>
@@ -12530,6 +12832,9 @@
         </is>
       </c>
       <c r="AF70" s="34" t="n">
+        <v>1899.99</v>
+      </c>
+      <c r="AG70" s="34" t="n">
         <v>1899.99</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Price check — 03/29/2026
</commit_message>
<xml_diff>
--- a/PriceBook_Combined_Final.xlsx
+++ b/PriceBook_Combined_Final.xlsx
@@ -709,7 +709,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:AG67"/>
+  <dimension ref="B1:AH67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -745,6 +745,7 @@
     <col width="12" customWidth="1" min="31" max="31"/>
     <col width="12" customWidth="1" min="32" max="32"/>
     <col width="12" customWidth="1" min="33" max="33"/>
+    <col width="12" customWidth="1" min="34" max="34"/>
   </cols>
   <sheetData>
     <row r="1" ht="8" customHeight="1"/>
@@ -924,6 +925,11 @@
           <t>3/28</t>
         </is>
       </c>
+      <c r="AH5" s="33" t="inlineStr">
+        <is>
+          <t>3/29</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="22" customHeight="1">
       <c r="B6" s="5" t="inlineStr">
@@ -1045,6 +1051,9 @@
       <c r="AG7" s="34" t="n">
         <v>449.99</v>
       </c>
+      <c r="AH7" s="34" t="n">
+        <v>449.99</v>
+      </c>
     </row>
     <row r="8" ht="18" customHeight="1">
       <c r="B8" s="15" t="n">
@@ -1185,6 +1194,11 @@
       <c r="AG8" s="36" t="n">
         <v>809.99</v>
       </c>
+      <c r="AH8" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="18" customHeight="1">
       <c r="B9" s="6" t="n">
@@ -1325,6 +1339,11 @@
       <c r="AG9" s="36" t="n">
         <v>809.99</v>
       </c>
+      <c r="AH9" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="18" customHeight="1">
       <c r="B10" s="15" t="n">
@@ -1439,6 +1458,9 @@
       <c r="AG10" s="34" t="n">
         <v>449.99</v>
       </c>
+      <c r="AH10" s="34" t="n">
+        <v>449.99</v>
+      </c>
     </row>
     <row r="11" ht="18" customHeight="1">
       <c r="B11" s="6" t="n">
@@ -1579,6 +1601,11 @@
       <c r="AG11" s="36" t="n">
         <v>809.99</v>
       </c>
+      <c r="AH11" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="18" customHeight="1">
       <c r="B12" s="15" t="n">
@@ -1697,6 +1724,9 @@
       <c r="AG12" s="36" t="n">
         <v>839.99</v>
       </c>
+      <c r="AH12" s="36" t="n">
+        <v>839.99</v>
+      </c>
     </row>
     <row r="13" ht="5" customHeight="1"/>
     <row r="14" ht="22" customHeight="1">
@@ -1833,6 +1863,11 @@
       <c r="AG15" s="34" t="n">
         <v>599.99</v>
       </c>
+      <c r="AH15" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="18" customHeight="1">
       <c r="B16" s="15" t="n">
@@ -1957,6 +1992,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AH16" s="36" t="n">
+        <v>809.99</v>
+      </c>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="B17" s="6" t="n">
@@ -2099,6 +2137,11 @@
         </is>
       </c>
       <c r="AG17" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AH17" s="35" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2281,6 +2324,9 @@
       <c r="AG19" s="34" t="n">
         <v>2199.99</v>
       </c>
+      <c r="AH19" s="34" t="n">
+        <v>2199.99</v>
+      </c>
     </row>
     <row r="20" ht="5" customHeight="1"/>
     <row r="21" ht="22" customHeight="1">
@@ -2411,6 +2457,11 @@
       <c r="AG22" s="34" t="n">
         <v>1098.99</v>
       </c>
+      <c r="AH22" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="B23" s="6" t="n">
@@ -2535,6 +2586,9 @@
       <c r="AG23" s="34" t="n">
         <v>1198.99</v>
       </c>
+      <c r="AH23" s="34" t="n">
+        <v>1198.99</v>
+      </c>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="B24" s="15" t="n">
@@ -2657,6 +2711,9 @@
         <v>1198.99</v>
       </c>
       <c r="AG24" s="34" t="n">
+        <v>1198.99</v>
+      </c>
+      <c r="AH24" s="34" t="n">
         <v>1198.99</v>
       </c>
     </row>
@@ -2843,6 +2900,9 @@
       <c r="AG26" s="34" t="n">
         <v>1599.99</v>
       </c>
+      <c r="AH26" s="34" t="n">
+        <v>1599.99</v>
+      </c>
     </row>
     <row r="27" ht="18" customHeight="1">
       <c r="B27" s="6" t="n">
@@ -2965,6 +3025,11 @@
       <c r="AG27" s="34" t="n">
         <v>1799.99</v>
       </c>
+      <c r="AH27" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="18" customHeight="1">
       <c r="B28" s="15" t="n">
@@ -3083,6 +3148,9 @@
       <c r="AG28" s="34" t="n">
         <v>1479.99</v>
       </c>
+      <c r="AH28" s="34" t="n">
+        <v>1479.99</v>
+      </c>
     </row>
     <row r="29" ht="18" customHeight="1">
       <c r="B29" s="6" t="n">
@@ -3205,6 +3273,11 @@
       <c r="AG29" s="34" t="n">
         <v>1799.99</v>
       </c>
+      <c r="AH29" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="18" customHeight="1">
       <c r="B30" s="15" t="n">
@@ -3327,6 +3400,11 @@
       <c r="AG30" s="34" t="n">
         <v>1799.99</v>
       </c>
+      <c r="AH30" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="5" customHeight="1"/>
     <row r="32" ht="22" customHeight="1">
@@ -3457,6 +3535,9 @@
       <c r="AG33" s="34" t="n">
         <v>1029.99</v>
       </c>
+      <c r="AH33" s="34" t="n">
+        <v>1029.99</v>
+      </c>
     </row>
     <row r="34" ht="18" customHeight="1">
       <c r="B34" s="15" t="n">
@@ -3579,6 +3660,9 @@
       <c r="AG34" s="34" t="n">
         <v>1029.99</v>
       </c>
+      <c r="AH34" s="34" t="n">
+        <v>1029.99</v>
+      </c>
     </row>
     <row r="35" ht="18" customHeight="1">
       <c r="B35" s="6" t="n">
@@ -3707,6 +3791,9 @@
       <c r="AG35" s="34" t="n">
         <v>1599.99</v>
       </c>
+      <c r="AH35" s="34" t="n">
+        <v>1599.99</v>
+      </c>
     </row>
     <row r="36" ht="18" customHeight="1">
       <c r="B36" s="15" t="n">
@@ -3833,6 +3920,9 @@
       <c r="AG36" s="34" t="n">
         <v>1699.99</v>
       </c>
+      <c r="AH36" s="34" t="n">
+        <v>1699.99</v>
+      </c>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="B37" s="6" t="n">
@@ -3953,6 +4043,11 @@
       <c r="AG37" s="36" t="n">
         <v>3399.99</v>
       </c>
+      <c r="AH37" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="18" customHeight="1">
       <c r="B38" s="15" t="n">
@@ -4075,6 +4170,9 @@
       <c r="AG38" s="34" t="n">
         <v>2898.99</v>
       </c>
+      <c r="AH38" s="34" t="n">
+        <v>2898.99</v>
+      </c>
     </row>
     <row r="39" ht="18" customHeight="1">
       <c r="B39" s="6" t="n">
@@ -4195,6 +4293,11 @@
       <c r="AG39" s="36" t="n">
         <v>3399.99</v>
       </c>
+      <c r="AH39" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="40" ht="18" customHeight="1">
       <c r="B40" s="15" t="n">
@@ -4317,6 +4420,9 @@
       <c r="AG40" s="34" t="n">
         <v>1029.99</v>
       </c>
+      <c r="AH40" s="34" t="n">
+        <v>1029.99</v>
+      </c>
     </row>
     <row r="41" ht="18" customHeight="1">
       <c r="B41" s="6" t="n">
@@ -4439,6 +4545,9 @@
       <c r="AG41" s="36" t="n">
         <v>2159.99</v>
       </c>
+      <c r="AH41" s="36" t="n">
+        <v>2159.99</v>
+      </c>
     </row>
     <row r="42" ht="18" customHeight="1">
       <c r="B42" s="15" t="n">
@@ -4570,6 +4679,9 @@
         <is>
           <t>—</t>
         </is>
+      </c>
+      <c r="AH42" s="36" t="n">
+        <v>1999.99</v>
       </c>
     </row>
     <row r="43" ht="18" customHeight="1">
@@ -4747,6 +4859,9 @@
       <c r="AG44" s="34" t="n">
         <v>3599.99</v>
       </c>
+      <c r="AH44" s="34" t="n">
+        <v>3599.99</v>
+      </c>
     </row>
     <row r="45" ht="5" customHeight="1"/>
     <row r="46" ht="22" customHeight="1">
@@ -4887,6 +5002,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AH47" s="36" t="n">
+        <v>1999.99</v>
+      </c>
     </row>
     <row r="48" ht="18" customHeight="1">
       <c r="B48" s="15" t="n">
@@ -5015,6 +5133,9 @@
       <c r="AG48" s="34" t="n">
         <v>1599.99</v>
       </c>
+      <c r="AH48" s="34" t="n">
+        <v>1599.99</v>
+      </c>
     </row>
     <row r="49" ht="18" customHeight="1">
       <c r="B49" s="6" t="n">
@@ -5139,6 +5260,11 @@
       <c r="AG49" s="34" t="n">
         <v>1849.99</v>
       </c>
+      <c r="AH49" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="50" ht="18" customHeight="1">
       <c r="B50" s="15" t="n">
@@ -5258,6 +5384,9 @@
         <is>
           <t>—</t>
         </is>
+      </c>
+      <c r="AH50" s="34" t="n">
+        <v>2599.99</v>
       </c>
     </row>
     <row r="51" ht="18" customHeight="1">
@@ -5435,6 +5564,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AH52" s="34" t="n">
+        <v>2599.99</v>
+      </c>
     </row>
     <row r="53" ht="18" customHeight="1">
       <c r="B53" s="6" t="n">
@@ -5557,6 +5689,9 @@
       <c r="AG53" s="13" t="n">
         <v>1899.99</v>
       </c>
+      <c r="AH53" s="13" t="n">
+        <v>1899.99</v>
+      </c>
     </row>
     <row r="54" ht="5" customHeight="1"/>
     <row r="55" ht="22" customHeight="1">
@@ -5683,6 +5818,9 @@
         <v>3599.99</v>
       </c>
       <c r="AG56" s="34" t="n">
+        <v>3599.99</v>
+      </c>
+      <c r="AH56" s="34" t="n">
         <v>3599.99</v>
       </c>
     </row>
@@ -5983,6 +6121,9 @@
       <c r="AG62" s="34" t="n">
         <v>127.99</v>
       </c>
+      <c r="AH62" s="34" t="n">
+        <v>127.99</v>
+      </c>
     </row>
     <row r="63" ht="18" customHeight="1">
       <c r="B63" s="6" t="n">
@@ -6123,6 +6264,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AH63" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="64" ht="18" customHeight="1">
       <c r="B64" s="15" t="n">
@@ -6251,6 +6397,9 @@
         <v>479.99</v>
       </c>
       <c r="AG64" s="36" t="n">
+        <v>479.99</v>
+      </c>
+      <c r="AH64" s="36" t="n">
         <v>479.99</v>
       </c>
     </row>
@@ -6485,7 +6634,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:AG70"/>
+  <dimension ref="B1:AH70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -6521,6 +6670,7 @@
     <col width="12" customWidth="1" min="31" max="31"/>
     <col width="12" customWidth="1" min="32" max="32"/>
     <col width="12" customWidth="1" min="33" max="33"/>
+    <col width="12" customWidth="1" min="34" max="34"/>
   </cols>
   <sheetData>
     <row r="1" ht="8" customHeight="1"/>
@@ -6700,6 +6850,11 @@
           <t>3/28</t>
         </is>
       </c>
+      <c r="AH5" s="33" t="inlineStr">
+        <is>
+          <t>3/29</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="22" customHeight="1">
       <c r="B6" s="5" t="inlineStr">
@@ -6831,6 +6986,9 @@
       <c r="AG7" s="34" t="n">
         <v>89.98999999999999</v>
       </c>
+      <c r="AH7" s="34" t="n">
+        <v>89.98999999999999</v>
+      </c>
     </row>
     <row r="8" ht="18" customHeight="1">
       <c r="B8" s="15" t="n">
@@ -6951,6 +7109,9 @@
       <c r="AG8" s="34" t="n">
         <v>194.99</v>
       </c>
+      <c r="AH8" s="34" t="n">
+        <v>194.99</v>
+      </c>
     </row>
     <row r="9" ht="18" customHeight="1">
       <c r="B9" s="6" t="n">
@@ -7091,6 +7252,11 @@
         </is>
       </c>
       <c r="AG9" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AH9" s="35" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -7267,6 +7433,9 @@
       <c r="AG11" s="34" t="n">
         <v>219.99</v>
       </c>
+      <c r="AH11" s="34" t="n">
+        <v>219.99</v>
+      </c>
     </row>
     <row r="12" ht="18" customHeight="1">
       <c r="B12" s="15" t="n">
@@ -7391,6 +7560,9 @@
       <c r="AG12" s="34" t="n">
         <v>349.99</v>
       </c>
+      <c r="AH12" s="34" t="n">
+        <v>349.99</v>
+      </c>
     </row>
     <row r="13" ht="18" customHeight="1">
       <c r="B13" s="6" t="n">
@@ -7533,6 +7705,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AH13" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="5" customHeight="1"/>
     <row r="15" ht="22" customHeight="1">
@@ -7685,6 +7862,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AH16" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="B17" s="6" t="n">
@@ -7803,6 +7985,11 @@
       <c r="AG17" s="34" t="n">
         <v>279.99</v>
       </c>
+      <c r="AH17" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="B18" s="15" t="n">
@@ -7927,6 +8114,9 @@
       <c r="AG18" s="34" t="n">
         <v>399.99</v>
       </c>
+      <c r="AH18" s="34" t="n">
+        <v>399.99</v>
+      </c>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="B19" s="6" t="n">
@@ -8053,6 +8243,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AH19" s="13" t="n">
+        <v>229.99</v>
+      </c>
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="B20" s="15" t="n">
@@ -8175,6 +8368,11 @@
       <c r="AG20" s="34" t="n">
         <v>427.99</v>
       </c>
+      <c r="AH20" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="B21" s="6" t="n">
@@ -8289,6 +8487,9 @@
       <c r="AG21" s="13" t="n">
         <v>449.99</v>
       </c>
+      <c r="AH21" s="13" t="n">
+        <v>449.99</v>
+      </c>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="B22" s="15" t="n">
@@ -8419,6 +8620,9 @@
       <c r="AG22" s="34" t="n">
         <v>599.99</v>
       </c>
+      <c r="AH22" s="34" t="n">
+        <v>599.99</v>
+      </c>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="B23" s="6" t="n">
@@ -8541,6 +8745,9 @@
       <c r="AG23" s="34" t="n">
         <v>999.99</v>
       </c>
+      <c r="AH23" s="34" t="n">
+        <v>999.99</v>
+      </c>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="B24" s="15" t="n">
@@ -8683,6 +8890,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AH24" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="18" customHeight="1">
       <c r="B25" s="6" t="n">
@@ -8811,6 +9023,11 @@
       <c r="AG25" s="34" t="n">
         <v>1199.99</v>
       </c>
+      <c r="AH25" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="18" customHeight="1">
       <c r="B26" s="15" t="n">
@@ -8931,6 +9148,9 @@
       <c r="AG26" s="34" t="n">
         <v>1274.99</v>
       </c>
+      <c r="AH26" s="34" t="n">
+        <v>1274.99</v>
+      </c>
     </row>
     <row r="27" ht="5" customHeight="1"/>
     <row r="28" ht="22" customHeight="1">
@@ -9065,6 +9285,9 @@
       <c r="AG29" s="34" t="n">
         <v>369.99</v>
       </c>
+      <c r="AH29" s="34" t="n">
+        <v>369.99</v>
+      </c>
     </row>
     <row r="30" ht="18" customHeight="1">
       <c r="B30" s="15" t="n">
@@ -9189,6 +9412,9 @@
       <c r="AG30" s="34" t="n">
         <v>579.99</v>
       </c>
+      <c r="AH30" s="34" t="n">
+        <v>579.99</v>
+      </c>
     </row>
     <row r="31" ht="18" customHeight="1">
       <c r="B31" s="6" t="n">
@@ -9315,6 +9541,9 @@
       <c r="AG31" s="13" t="n">
         <v>699.99</v>
       </c>
+      <c r="AH31" s="13" t="n">
+        <v>699.99</v>
+      </c>
     </row>
     <row r="32" ht="18" customHeight="1">
       <c r="B32" s="15" t="n">
@@ -9439,6 +9668,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AH32" s="34" t="n">
+        <v>759.99</v>
+      </c>
     </row>
     <row r="33" ht="18" customHeight="1">
       <c r="B33" s="6" t="n">
@@ -9565,6 +9797,9 @@
       <c r="AG33" s="34" t="n">
         <v>799.99</v>
       </c>
+      <c r="AH33" s="34" t="n">
+        <v>799.99</v>
+      </c>
     </row>
     <row r="34" ht="18" customHeight="1">
       <c r="B34" s="15" t="n">
@@ -9685,6 +9920,9 @@
       <c r="AG34" s="34" t="n">
         <v>1274.99</v>
       </c>
+      <c r="AH34" s="34" t="n">
+        <v>1274.99</v>
+      </c>
     </row>
     <row r="35" ht="18" customHeight="1">
       <c r="B35" s="6" t="n">
@@ -9807,6 +10045,9 @@
       <c r="AG35" s="34" t="n">
         <v>1799.99</v>
       </c>
+      <c r="AH35" s="34" t="n">
+        <v>1799.99</v>
+      </c>
     </row>
     <row r="36" ht="18" customHeight="1">
       <c r="B36" s="15" t="n">
@@ -9925,6 +10166,9 @@
       <c r="AG36" s="34" t="n">
         <v>1975.99</v>
       </c>
+      <c r="AH36" s="34" t="n">
+        <v>1975.99</v>
+      </c>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="B37" s="6" t="n">
@@ -10053,6 +10297,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AH37" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="5" customHeight="1"/>
     <row r="39" ht="22" customHeight="1">
@@ -10185,6 +10434,9 @@
       <c r="AG40" s="34" t="n">
         <v>740.99</v>
       </c>
+      <c r="AH40" s="34" t="n">
+        <v>740.99</v>
+      </c>
     </row>
     <row r="41" ht="18" customHeight="1">
       <c r="B41" s="6" t="n">
@@ -10313,6 +10565,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AH41" s="13" t="n">
+        <v>599.99</v>
+      </c>
     </row>
     <row r="42" ht="18" customHeight="1">
       <c r="B42" s="15" t="n">
@@ -10439,6 +10694,9 @@
       <c r="AG42" s="34" t="n">
         <v>799.99</v>
       </c>
+      <c r="AH42" s="34" t="n">
+        <v>799.99</v>
+      </c>
     </row>
     <row r="43" ht="18" customHeight="1">
       <c r="B43" s="6" t="n">
@@ -10567,6 +10825,9 @@
       <c r="AG43" s="34" t="n">
         <v>949.99</v>
       </c>
+      <c r="AH43" s="34" t="n">
+        <v>949.99</v>
+      </c>
     </row>
     <row r="44" ht="18" customHeight="1">
       <c r="B44" s="15" t="n">
@@ -10685,6 +10946,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AH44" s="34" t="n">
+        <v>1139.99</v>
+      </c>
     </row>
     <row r="45" ht="18" customHeight="1">
       <c r="B45" s="6" t="n">
@@ -10803,6 +11067,9 @@
       <c r="AG45" s="34" t="n">
         <v>1529.99</v>
       </c>
+      <c r="AH45" s="34" t="n">
+        <v>1529.99</v>
+      </c>
     </row>
     <row r="46" ht="18" customHeight="1">
       <c r="B46" s="15" t="n">
@@ -10945,6 +11212,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AH46" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="47" ht="18" customHeight="1">
       <c r="B47" s="6" t="n">
@@ -11067,6 +11339,9 @@
       <c r="AG47" s="34" t="n">
         <v>2999.99</v>
       </c>
+      <c r="AH47" s="34" t="n">
+        <v>2999.99</v>
+      </c>
     </row>
     <row r="48" ht="18" customHeight="1">
       <c r="B48" s="15" t="n">
@@ -11197,6 +11472,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AH48" s="34" t="n">
+        <v>3499.99</v>
+      </c>
     </row>
     <row r="49" ht="5" customHeight="1"/>
     <row r="50" ht="22" customHeight="1">
@@ -11325,6 +11603,9 @@
       <c r="AG51" s="34" t="n">
         <v>798.99</v>
       </c>
+      <c r="AH51" s="34" t="n">
+        <v>798.99</v>
+      </c>
     </row>
     <row r="52" ht="18" customHeight="1">
       <c r="B52" s="15" t="n">
@@ -11445,6 +11726,9 @@
       <c r="AG52" s="34" t="n">
         <v>798.99</v>
       </c>
+      <c r="AH52" s="34" t="n">
+        <v>798.99</v>
+      </c>
     </row>
     <row r="53" ht="18" customHeight="1">
       <c r="B53" s="6" t="n">
@@ -11567,6 +11851,11 @@
       <c r="AG53" s="34" t="n">
         <v>1499.99</v>
       </c>
+      <c r="AH53" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="54" ht="18" customHeight="1">
       <c r="B54" s="15" t="n">
@@ -11687,6 +11976,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AH54" s="34" t="n">
+        <v>899.99</v>
+      </c>
     </row>
     <row r="55" ht="18" customHeight="1">
       <c r="B55" s="6" t="n">
@@ -11809,6 +12101,9 @@
       <c r="AG55" s="13" t="n">
         <v>1299.99</v>
       </c>
+      <c r="AH55" s="13" t="n">
+        <v>1299.99</v>
+      </c>
     </row>
     <row r="56" ht="18" customHeight="1">
       <c r="B56" s="15" t="n">
@@ -11933,6 +12228,9 @@
       <c r="AG56" s="34" t="n">
         <v>2799.99</v>
       </c>
+      <c r="AH56" s="34" t="n">
+        <v>2799.99</v>
+      </c>
     </row>
     <row r="57" ht="18" customHeight="1">
       <c r="B57" s="6" t="n">
@@ -12051,6 +12349,9 @@
         <v>3199.99</v>
       </c>
       <c r="AG57" s="34" t="n">
+        <v>3199.99</v>
+      </c>
+      <c r="AH57" s="34" t="n">
         <v>3199.99</v>
       </c>
     </row>
@@ -12239,6 +12540,9 @@
       <c r="AG61" s="34" t="n">
         <v>999.99</v>
       </c>
+      <c r="AH61" s="34" t="n">
+        <v>999.99</v>
+      </c>
     </row>
     <row r="62" ht="18" customHeight="1">
       <c r="B62" s="15" t="n">
@@ -12419,6 +12723,9 @@
       <c r="AG63" s="34" t="n">
         <v>1658.99</v>
       </c>
+      <c r="AH63" s="34" t="n">
+        <v>1658.99</v>
+      </c>
     </row>
     <row r="64" ht="18" customHeight="1">
       <c r="B64" s="15" t="n">
@@ -12537,6 +12844,9 @@
         <v>2549.99</v>
       </c>
       <c r="AG64" s="34" t="n">
+        <v>2549.99</v>
+      </c>
+      <c r="AH64" s="34" t="n">
         <v>2549.99</v>
       </c>
     </row>
@@ -12835,6 +13145,9 @@
         <v>1899.99</v>
       </c>
       <c r="AG70" s="34" t="n">
+        <v>1899.99</v>
+      </c>
+      <c r="AH70" s="34" t="n">
         <v>1899.99</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Price check — 03/30/2026
</commit_message>
<xml_diff>
--- a/PriceBook_Combined_Final.xlsx
+++ b/PriceBook_Combined_Final.xlsx
@@ -709,7 +709,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:AH67"/>
+  <dimension ref="B1:AI67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -746,6 +746,7 @@
     <col width="12" customWidth="1" min="32" max="32"/>
     <col width="12" customWidth="1" min="33" max="33"/>
     <col width="12" customWidth="1" min="34" max="34"/>
+    <col width="12" customWidth="1" min="35" max="35"/>
   </cols>
   <sheetData>
     <row r="1" ht="8" customHeight="1"/>
@@ -930,6 +931,11 @@
           <t>3/29</t>
         </is>
       </c>
+      <c r="AI5" s="33" t="inlineStr">
+        <is>
+          <t>3/30</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="22" customHeight="1">
       <c r="B6" s="5" t="inlineStr">
@@ -1054,6 +1060,9 @@
       <c r="AH7" s="34" t="n">
         <v>449.99</v>
       </c>
+      <c r="AI7" s="34" t="n">
+        <v>449.99</v>
+      </c>
     </row>
     <row r="8" ht="18" customHeight="1">
       <c r="B8" s="15" t="n">
@@ -1199,6 +1208,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AI8" s="36" t="n">
+        <v>809.99</v>
+      </c>
     </row>
     <row r="9" ht="18" customHeight="1">
       <c r="B9" s="6" t="n">
@@ -1344,6 +1356,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AI9" s="36" t="n">
+        <v>809.99</v>
+      </c>
     </row>
     <row r="10" ht="18" customHeight="1">
       <c r="B10" s="15" t="n">
@@ -1461,6 +1476,9 @@
       <c r="AH10" s="34" t="n">
         <v>449.99</v>
       </c>
+      <c r="AI10" s="34" t="n">
+        <v>449.99</v>
+      </c>
     </row>
     <row r="11" ht="18" customHeight="1">
       <c r="B11" s="6" t="n">
@@ -1606,6 +1624,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AI11" s="36" t="n">
+        <v>809.99</v>
+      </c>
     </row>
     <row r="12" ht="18" customHeight="1">
       <c r="B12" s="15" t="n">
@@ -1727,6 +1748,9 @@
       <c r="AH12" s="36" t="n">
         <v>839.99</v>
       </c>
+      <c r="AI12" s="36" t="n">
+        <v>839.99</v>
+      </c>
     </row>
     <row r="13" ht="5" customHeight="1"/>
     <row r="14" ht="22" customHeight="1">
@@ -1868,6 +1892,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AI15" s="34" t="n">
+        <v>599.99</v>
+      </c>
     </row>
     <row r="16" ht="18" customHeight="1">
       <c r="B16" s="15" t="n">
@@ -1995,6 +2022,9 @@
       <c r="AH16" s="36" t="n">
         <v>809.99</v>
       </c>
+      <c r="AI16" s="36" t="n">
+        <v>809.99</v>
+      </c>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="B17" s="6" t="n">
@@ -2142,6 +2172,11 @@
         </is>
       </c>
       <c r="AH17" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AI17" s="35" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2327,6 +2362,9 @@
       <c r="AH19" s="34" t="n">
         <v>2199.99</v>
       </c>
+      <c r="AI19" s="34" t="n">
+        <v>2199.99</v>
+      </c>
     </row>
     <row r="20" ht="5" customHeight="1"/>
     <row r="21" ht="22" customHeight="1">
@@ -2462,6 +2500,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AI22" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="B23" s="6" t="n">
@@ -2589,6 +2632,9 @@
       <c r="AH23" s="34" t="n">
         <v>1198.99</v>
       </c>
+      <c r="AI23" s="34" t="n">
+        <v>1198.99</v>
+      </c>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="B24" s="15" t="n">
@@ -2714,6 +2760,9 @@
         <v>1198.99</v>
       </c>
       <c r="AH24" s="34" t="n">
+        <v>1198.99</v>
+      </c>
+      <c r="AI24" s="34" t="n">
         <v>1198.99</v>
       </c>
     </row>
@@ -2903,6 +2952,9 @@
       <c r="AH26" s="34" t="n">
         <v>1599.99</v>
       </c>
+      <c r="AI26" s="34" t="n">
+        <v>1599.99</v>
+      </c>
     </row>
     <row r="27" ht="18" customHeight="1">
       <c r="B27" s="6" t="n">
@@ -3030,6 +3082,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AI27" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="18" customHeight="1">
       <c r="B28" s="15" t="n">
@@ -3151,6 +3208,9 @@
       <c r="AH28" s="34" t="n">
         <v>1479.99</v>
       </c>
+      <c r="AI28" s="34" t="n">
+        <v>1479.99</v>
+      </c>
     </row>
     <row r="29" ht="18" customHeight="1">
       <c r="B29" s="6" t="n">
@@ -3278,6 +3338,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AI29" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="18" customHeight="1">
       <c r="B30" s="15" t="n">
@@ -3405,6 +3470,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AI30" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="5" customHeight="1"/>
     <row r="32" ht="22" customHeight="1">
@@ -3538,6 +3608,11 @@
       <c r="AH33" s="34" t="n">
         <v>1029.99</v>
       </c>
+      <c r="AI33" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="18" customHeight="1">
       <c r="B34" s="15" t="n">
@@ -3663,6 +3738,11 @@
       <c r="AH34" s="34" t="n">
         <v>1029.99</v>
       </c>
+      <c r="AI34" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="18" customHeight="1">
       <c r="B35" s="6" t="n">
@@ -3794,6 +3874,9 @@
       <c r="AH35" s="34" t="n">
         <v>1599.99</v>
       </c>
+      <c r="AI35" s="34" t="n">
+        <v>1599.99</v>
+      </c>
     </row>
     <row r="36" ht="18" customHeight="1">
       <c r="B36" s="15" t="n">
@@ -3923,6 +4006,11 @@
       <c r="AH36" s="34" t="n">
         <v>1699.99</v>
       </c>
+      <c r="AI36" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="B37" s="6" t="n">
@@ -4048,6 +4136,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AI37" s="36" t="n">
+        <v>3399.99</v>
+      </c>
     </row>
     <row r="38" ht="18" customHeight="1">
       <c r="B38" s="15" t="n">
@@ -4173,6 +4264,9 @@
       <c r="AH38" s="34" t="n">
         <v>2898.99</v>
       </c>
+      <c r="AI38" s="34" t="n">
+        <v>2898.99</v>
+      </c>
     </row>
     <row r="39" ht="18" customHeight="1">
       <c r="B39" s="6" t="n">
@@ -4298,6 +4392,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AI39" s="36" t="n">
+        <v>3399.99</v>
+      </c>
     </row>
     <row r="40" ht="18" customHeight="1">
       <c r="B40" s="15" t="n">
@@ -4423,6 +4520,11 @@
       <c r="AH40" s="34" t="n">
         <v>1029.99</v>
       </c>
+      <c r="AI40" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="18" customHeight="1">
       <c r="B41" s="6" t="n">
@@ -4548,6 +4650,9 @@
       <c r="AH41" s="36" t="n">
         <v>2159.99</v>
       </c>
+      <c r="AI41" s="36" t="n">
+        <v>2159.99</v>
+      </c>
     </row>
     <row r="42" ht="18" customHeight="1">
       <c r="B42" s="15" t="n">
@@ -4682,6 +4787,11 @@
       </c>
       <c r="AH42" s="36" t="n">
         <v>1999.99</v>
+      </c>
+      <c r="AI42" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
     </row>
     <row r="43" ht="18" customHeight="1">
@@ -4862,6 +4972,9 @@
       <c r="AH44" s="34" t="n">
         <v>3599.99</v>
       </c>
+      <c r="AI44" s="34" t="n">
+        <v>3599.99</v>
+      </c>
     </row>
     <row r="45" ht="5" customHeight="1"/>
     <row r="46" ht="22" customHeight="1">
@@ -5005,6 +5118,11 @@
       <c r="AH47" s="36" t="n">
         <v>1999.99</v>
       </c>
+      <c r="AI47" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="48" ht="18" customHeight="1">
       <c r="B48" s="15" t="n">
@@ -5136,6 +5254,9 @@
       <c r="AH48" s="34" t="n">
         <v>1599.99</v>
       </c>
+      <c r="AI48" s="34" t="n">
+        <v>1599.99</v>
+      </c>
     </row>
     <row r="49" ht="18" customHeight="1">
       <c r="B49" s="6" t="n">
@@ -5265,6 +5386,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AI49" s="34" t="n">
+        <v>1849.99</v>
+      </c>
     </row>
     <row r="50" ht="18" customHeight="1">
       <c r="B50" s="15" t="n">
@@ -5386,6 +5510,9 @@
         </is>
       </c>
       <c r="AH50" s="34" t="n">
+        <v>2599.99</v>
+      </c>
+      <c r="AI50" s="34" t="n">
         <v>2599.99</v>
       </c>
     </row>
@@ -5567,6 +5694,9 @@
       <c r="AH52" s="34" t="n">
         <v>2599.99</v>
       </c>
+      <c r="AI52" s="34" t="n">
+        <v>2599.99</v>
+      </c>
     </row>
     <row r="53" ht="18" customHeight="1">
       <c r="B53" s="6" t="n">
@@ -5692,6 +5822,9 @@
       <c r="AH53" s="13" t="n">
         <v>1899.99</v>
       </c>
+      <c r="AI53" s="13" t="n">
+        <v>1899.99</v>
+      </c>
     </row>
     <row r="54" ht="5" customHeight="1"/>
     <row r="55" ht="22" customHeight="1">
@@ -5821,6 +5954,9 @@
         <v>3599.99</v>
       </c>
       <c r="AH56" s="34" t="n">
+        <v>3599.99</v>
+      </c>
+      <c r="AI56" s="34" t="n">
         <v>3599.99</v>
       </c>
     </row>
@@ -6124,6 +6260,11 @@
       <c r="AH62" s="34" t="n">
         <v>127.99</v>
       </c>
+      <c r="AI62" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="63" ht="18" customHeight="1">
       <c r="B63" s="6" t="n">
@@ -6269,6 +6410,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AI63" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="64" ht="18" customHeight="1">
       <c r="B64" s="15" t="n">
@@ -6401,6 +6547,9 @@
       </c>
       <c r="AH64" s="36" t="n">
         <v>479.99</v>
+      </c>
+      <c r="AI64" s="36" t="n">
+        <v>599.99</v>
       </c>
     </row>
     <row r="65" ht="18" customHeight="1">
@@ -6634,7 +6783,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:AH70"/>
+  <dimension ref="B1:AI70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -6671,6 +6820,7 @@
     <col width="12" customWidth="1" min="32" max="32"/>
     <col width="12" customWidth="1" min="33" max="33"/>
     <col width="12" customWidth="1" min="34" max="34"/>
+    <col width="12" customWidth="1" min="35" max="35"/>
   </cols>
   <sheetData>
     <row r="1" ht="8" customHeight="1"/>
@@ -6855,6 +7005,11 @@
           <t>3/29</t>
         </is>
       </c>
+      <c r="AI5" s="33" t="inlineStr">
+        <is>
+          <t>3/30</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="22" customHeight="1">
       <c r="B6" s="5" t="inlineStr">
@@ -6989,6 +7144,9 @@
       <c r="AH7" s="34" t="n">
         <v>89.98999999999999</v>
       </c>
+      <c r="AI7" s="34" t="n">
+        <v>89.98999999999999</v>
+      </c>
     </row>
     <row r="8" ht="18" customHeight="1">
       <c r="B8" s="15" t="n">
@@ -7112,6 +7270,11 @@
       <c r="AH8" s="34" t="n">
         <v>194.99</v>
       </c>
+      <c r="AI8" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="18" customHeight="1">
       <c r="B9" s="6" t="n">
@@ -7257,6 +7420,11 @@
         </is>
       </c>
       <c r="AH9" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AI9" s="35" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -7436,6 +7604,9 @@
       <c r="AH11" s="34" t="n">
         <v>219.99</v>
       </c>
+      <c r="AI11" s="34" t="n">
+        <v>219.99</v>
+      </c>
     </row>
     <row r="12" ht="18" customHeight="1">
       <c r="B12" s="15" t="n">
@@ -7563,6 +7734,9 @@
       <c r="AH12" s="34" t="n">
         <v>349.99</v>
       </c>
+      <c r="AI12" s="36" t="n">
+        <v>379.99</v>
+      </c>
     </row>
     <row r="13" ht="18" customHeight="1">
       <c r="B13" s="6" t="n">
@@ -7710,6 +7884,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AI13" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="5" customHeight="1"/>
     <row r="15" ht="22" customHeight="1">
@@ -7867,6 +8046,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AI16" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="B17" s="6" t="n">
@@ -7990,6 +8174,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AI17" s="36" t="n">
+        <v>299.99</v>
+      </c>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="B18" s="15" t="n">
@@ -8117,6 +8304,11 @@
       <c r="AH18" s="34" t="n">
         <v>399.99</v>
       </c>
+      <c r="AI18" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="B19" s="6" t="n">
@@ -8246,6 +8438,9 @@
       <c r="AH19" s="13" t="n">
         <v>229.99</v>
       </c>
+      <c r="AI19" s="34" t="n">
+        <v>249.99</v>
+      </c>
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="B20" s="15" t="n">
@@ -8373,6 +8568,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AI20" s="34" t="n">
+        <v>427.99</v>
+      </c>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="B21" s="6" t="n">
@@ -8490,6 +8688,9 @@
       <c r="AH21" s="13" t="n">
         <v>449.99</v>
       </c>
+      <c r="AI21" s="13" t="n">
+        <v>449.99</v>
+      </c>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="B22" s="15" t="n">
@@ -8623,6 +8824,9 @@
       <c r="AH22" s="34" t="n">
         <v>599.99</v>
       </c>
+      <c r="AI22" s="34" t="n">
+        <v>599.99</v>
+      </c>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="B23" s="6" t="n">
@@ -8748,6 +8952,11 @@
       <c r="AH23" s="34" t="n">
         <v>999.99</v>
       </c>
+      <c r="AI23" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="B24" s="15" t="n">
@@ -8895,6 +9104,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AI24" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="18" customHeight="1">
       <c r="B25" s="6" t="n">
@@ -9028,6 +9242,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AI25" s="34" t="n">
+        <v>1199.99</v>
+      </c>
     </row>
     <row r="26" ht="18" customHeight="1">
       <c r="B26" s="15" t="n">
@@ -9151,6 +9368,9 @@
       <c r="AH26" s="34" t="n">
         <v>1274.99</v>
       </c>
+      <c r="AI26" s="34" t="n">
+        <v>1274.99</v>
+      </c>
     </row>
     <row r="27" ht="5" customHeight="1"/>
     <row r="28" ht="22" customHeight="1">
@@ -9288,6 +9508,9 @@
       <c r="AH29" s="34" t="n">
         <v>369.99</v>
       </c>
+      <c r="AI29" s="34" t="n">
+        <v>369.99</v>
+      </c>
     </row>
     <row r="30" ht="18" customHeight="1">
       <c r="B30" s="15" t="n">
@@ -9415,6 +9638,9 @@
       <c r="AH30" s="34" t="n">
         <v>579.99</v>
       </c>
+      <c r="AI30" s="34" t="n">
+        <v>579.99</v>
+      </c>
     </row>
     <row r="31" ht="18" customHeight="1">
       <c r="B31" s="6" t="n">
@@ -9544,6 +9770,9 @@
       <c r="AH31" s="13" t="n">
         <v>699.99</v>
       </c>
+      <c r="AI31" s="13" t="n">
+        <v>699.99</v>
+      </c>
     </row>
     <row r="32" ht="18" customHeight="1">
       <c r="B32" s="15" t="n">
@@ -9671,6 +9900,9 @@
       <c r="AH32" s="34" t="n">
         <v>759.99</v>
       </c>
+      <c r="AI32" s="34" t="n">
+        <v>759.99</v>
+      </c>
     </row>
     <row r="33" ht="18" customHeight="1">
       <c r="B33" s="6" t="n">
@@ -9800,6 +10032,11 @@
       <c r="AH33" s="34" t="n">
         <v>799.99</v>
       </c>
+      <c r="AI33" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="18" customHeight="1">
       <c r="B34" s="15" t="n">
@@ -9923,6 +10160,9 @@
       <c r="AH34" s="34" t="n">
         <v>1274.99</v>
       </c>
+      <c r="AI34" s="34" t="n">
+        <v>1274.99</v>
+      </c>
     </row>
     <row r="35" ht="18" customHeight="1">
       <c r="B35" s="6" t="n">
@@ -10048,6 +10288,9 @@
       <c r="AH35" s="34" t="n">
         <v>1799.99</v>
       </c>
+      <c r="AI35" s="34" t="n">
+        <v>1799.99</v>
+      </c>
     </row>
     <row r="36" ht="18" customHeight="1">
       <c r="B36" s="15" t="n">
@@ -10169,6 +10412,11 @@
       <c r="AH36" s="34" t="n">
         <v>1975.99</v>
       </c>
+      <c r="AI36" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="B37" s="6" t="n">
@@ -10302,6 +10550,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AI37" s="34" t="n">
+        <v>2699.99</v>
+      </c>
     </row>
     <row r="38" ht="5" customHeight="1"/>
     <row r="39" ht="22" customHeight="1">
@@ -10437,6 +10688,9 @@
       <c r="AH40" s="34" t="n">
         <v>740.99</v>
       </c>
+      <c r="AI40" s="34" t="n">
+        <v>740.99</v>
+      </c>
     </row>
     <row r="41" ht="18" customHeight="1">
       <c r="B41" s="6" t="n">
@@ -10568,6 +10822,9 @@
       <c r="AH41" s="13" t="n">
         <v>599.99</v>
       </c>
+      <c r="AI41" s="13" t="n">
+        <v>549.99</v>
+      </c>
     </row>
     <row r="42" ht="18" customHeight="1">
       <c r="B42" s="15" t="n">
@@ -10697,6 +10954,11 @@
       <c r="AH42" s="34" t="n">
         <v>799.99</v>
       </c>
+      <c r="AI42" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="43" ht="18" customHeight="1">
       <c r="B43" s="6" t="n">
@@ -10828,6 +11090,9 @@
       <c r="AH43" s="34" t="n">
         <v>949.99</v>
       </c>
+      <c r="AI43" s="34" t="n">
+        <v>949.99</v>
+      </c>
     </row>
     <row r="44" ht="18" customHeight="1">
       <c r="B44" s="15" t="n">
@@ -10949,6 +11214,9 @@
       <c r="AH44" s="34" t="n">
         <v>1139.99</v>
       </c>
+      <c r="AI44" s="34" t="n">
+        <v>1139.99</v>
+      </c>
     </row>
     <row r="45" ht="18" customHeight="1">
       <c r="B45" s="6" t="n">
@@ -11070,6 +11338,9 @@
       <c r="AH45" s="34" t="n">
         <v>1529.99</v>
       </c>
+      <c r="AI45" s="34" t="n">
+        <v>1529.99</v>
+      </c>
     </row>
     <row r="46" ht="18" customHeight="1">
       <c r="B46" s="15" t="n">
@@ -11217,6 +11488,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AI46" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="47" ht="18" customHeight="1">
       <c r="B47" s="6" t="n">
@@ -11342,6 +11618,11 @@
       <c r="AH47" s="34" t="n">
         <v>2999.99</v>
       </c>
+      <c r="AI47" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="48" ht="18" customHeight="1">
       <c r="B48" s="15" t="n">
@@ -11475,6 +11756,9 @@
       <c r="AH48" s="34" t="n">
         <v>3499.99</v>
       </c>
+      <c r="AI48" s="36" t="n">
+        <v>3799.99</v>
+      </c>
     </row>
     <row r="49" ht="5" customHeight="1"/>
     <row r="50" ht="22" customHeight="1">
@@ -11606,6 +11890,9 @@
       <c r="AH51" s="34" t="n">
         <v>798.99</v>
       </c>
+      <c r="AI51" s="34" t="n">
+        <v>798.99</v>
+      </c>
     </row>
     <row r="52" ht="18" customHeight="1">
       <c r="B52" s="15" t="n">
@@ -11729,6 +12016,9 @@
       <c r="AH52" s="34" t="n">
         <v>798.99</v>
       </c>
+      <c r="AI52" s="34" t="n">
+        <v>798.99</v>
+      </c>
     </row>
     <row r="53" ht="18" customHeight="1">
       <c r="B53" s="6" t="n">
@@ -11856,6 +12146,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AI53" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="54" ht="18" customHeight="1">
       <c r="B54" s="15" t="n">
@@ -11979,6 +12274,9 @@
       <c r="AH54" s="34" t="n">
         <v>899.99</v>
       </c>
+      <c r="AI54" s="34" t="n">
+        <v>899.99</v>
+      </c>
     </row>
     <row r="55" ht="18" customHeight="1">
       <c r="B55" s="6" t="n">
@@ -12104,6 +12402,9 @@
       <c r="AH55" s="13" t="n">
         <v>1299.99</v>
       </c>
+      <c r="AI55" s="13" t="n">
+        <v>1299.99</v>
+      </c>
     </row>
     <row r="56" ht="18" customHeight="1">
       <c r="B56" s="15" t="n">
@@ -12231,6 +12532,11 @@
       <c r="AH56" s="34" t="n">
         <v>2799.99</v>
       </c>
+      <c r="AI56" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="57" ht="18" customHeight="1">
       <c r="B57" s="6" t="n">
@@ -12353,6 +12659,11 @@
       </c>
       <c r="AH57" s="34" t="n">
         <v>3199.99</v>
+      </c>
+      <c r="AI57" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
     </row>
     <row r="58" ht="18" customHeight="1">
@@ -12543,6 +12854,11 @@
       <c r="AH61" s="34" t="n">
         <v>999.99</v>
       </c>
+      <c r="AI61" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="62" ht="18" customHeight="1">
       <c r="B62" s="15" t="n">
@@ -12726,6 +13042,11 @@
       <c r="AH63" s="34" t="n">
         <v>1658.99</v>
       </c>
+      <c r="AI63" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="64" ht="18" customHeight="1">
       <c r="B64" s="15" t="n">
@@ -12847,6 +13168,9 @@
         <v>2549.99</v>
       </c>
       <c r="AH64" s="34" t="n">
+        <v>2549.99</v>
+      </c>
+      <c r="AI64" s="34" t="n">
         <v>2549.99</v>
       </c>
     </row>
@@ -13148,6 +13472,9 @@
         <v>1899.99</v>
       </c>
       <c r="AH70" s="34" t="n">
+        <v>1899.99</v>
+      </c>
+      <c r="AI70" s="34" t="n">
         <v>1899.99</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Price check — 03/31/2026
</commit_message>
<xml_diff>
--- a/PriceBook_Combined_Final.xlsx
+++ b/PriceBook_Combined_Final.xlsx
@@ -709,7 +709,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:AI67"/>
+  <dimension ref="B1:AJ67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -747,6 +747,7 @@
     <col width="12" customWidth="1" min="33" max="33"/>
     <col width="12" customWidth="1" min="34" max="34"/>
     <col width="12" customWidth="1" min="35" max="35"/>
+    <col width="12" customWidth="1" min="36" max="36"/>
   </cols>
   <sheetData>
     <row r="1" ht="8" customHeight="1"/>
@@ -936,6 +937,11 @@
           <t>3/30</t>
         </is>
       </c>
+      <c r="AJ5" s="33" t="inlineStr">
+        <is>
+          <t>3/31</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="22" customHeight="1">
       <c r="B6" s="5" t="inlineStr">
@@ -1063,6 +1069,9 @@
       <c r="AI7" s="34" t="n">
         <v>449.99</v>
       </c>
+      <c r="AJ7" s="34" t="n">
+        <v>449.99</v>
+      </c>
     </row>
     <row r="8" ht="18" customHeight="1">
       <c r="B8" s="15" t="n">
@@ -1211,6 +1220,9 @@
       <c r="AI8" s="36" t="n">
         <v>809.99</v>
       </c>
+      <c r="AJ8" s="36" t="n">
+        <v>809.99</v>
+      </c>
     </row>
     <row r="9" ht="18" customHeight="1">
       <c r="B9" s="6" t="n">
@@ -1359,6 +1371,9 @@
       <c r="AI9" s="36" t="n">
         <v>809.99</v>
       </c>
+      <c r="AJ9" s="36" t="n">
+        <v>809.99</v>
+      </c>
     </row>
     <row r="10" ht="18" customHeight="1">
       <c r="B10" s="15" t="n">
@@ -1479,6 +1494,9 @@
       <c r="AI10" s="34" t="n">
         <v>449.99</v>
       </c>
+      <c r="AJ10" s="34" t="n">
+        <v>449.99</v>
+      </c>
     </row>
     <row r="11" ht="18" customHeight="1">
       <c r="B11" s="6" t="n">
@@ -1627,6 +1645,9 @@
       <c r="AI11" s="36" t="n">
         <v>809.99</v>
       </c>
+      <c r="AJ11" s="36" t="n">
+        <v>809.99</v>
+      </c>
     </row>
     <row r="12" ht="18" customHeight="1">
       <c r="B12" s="15" t="n">
@@ -1751,6 +1772,11 @@
       <c r="AI12" s="36" t="n">
         <v>839.99</v>
       </c>
+      <c r="AJ12" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="5" customHeight="1"/>
     <row r="14" ht="22" customHeight="1">
@@ -1895,6 +1921,9 @@
       <c r="AI15" s="34" t="n">
         <v>599.99</v>
       </c>
+      <c r="AJ15" s="34" t="n">
+        <v>599.99</v>
+      </c>
     </row>
     <row r="16" ht="18" customHeight="1">
       <c r="B16" s="15" t="n">
@@ -2025,6 +2054,9 @@
       <c r="AI16" s="36" t="n">
         <v>809.99</v>
       </c>
+      <c r="AJ16" s="36" t="n">
+        <v>809.99</v>
+      </c>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="B17" s="6" t="n">
@@ -2177,6 +2209,11 @@
         </is>
       </c>
       <c r="AI17" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AJ17" s="35" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2365,6 +2402,9 @@
       <c r="AI19" s="34" t="n">
         <v>2199.99</v>
       </c>
+      <c r="AJ19" s="34" t="n">
+        <v>2199.99</v>
+      </c>
     </row>
     <row r="20" ht="5" customHeight="1"/>
     <row r="21" ht="22" customHeight="1">
@@ -2505,6 +2545,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AJ22" s="34" t="n">
+        <v>1098.99</v>
+      </c>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="B23" s="6" t="n">
@@ -2635,6 +2678,11 @@
       <c r="AI23" s="34" t="n">
         <v>1198.99</v>
       </c>
+      <c r="AJ23" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="B24" s="15" t="n">
@@ -2764,6 +2812,11 @@
       </c>
       <c r="AI24" s="34" t="n">
         <v>1198.99</v>
+      </c>
+      <c r="AJ24" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
     </row>
     <row r="25" ht="18" customHeight="1">
@@ -2955,6 +3008,9 @@
       <c r="AI26" s="34" t="n">
         <v>1599.99</v>
       </c>
+      <c r="AJ26" s="34" t="n">
+        <v>1599.99</v>
+      </c>
     </row>
     <row r="27" ht="18" customHeight="1">
       <c r="B27" s="6" t="n">
@@ -3087,6 +3143,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AJ27" s="34" t="n">
+        <v>1799.99</v>
+      </c>
     </row>
     <row r="28" ht="18" customHeight="1">
       <c r="B28" s="15" t="n">
@@ -3211,6 +3270,11 @@
       <c r="AI28" s="34" t="n">
         <v>1479.99</v>
       </c>
+      <c r="AJ28" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="18" customHeight="1">
       <c r="B29" s="6" t="n">
@@ -3343,6 +3407,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AJ29" s="34" t="n">
+        <v>1799.99</v>
+      </c>
     </row>
     <row r="30" ht="18" customHeight="1">
       <c r="B30" s="15" t="n">
@@ -3475,6 +3542,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AJ30" s="34" t="n">
+        <v>1799.99</v>
+      </c>
     </row>
     <row r="31" ht="5" customHeight="1"/>
     <row r="32" ht="22" customHeight="1">
@@ -3613,6 +3683,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AJ33" s="34" t="n">
+        <v>1029.99</v>
+      </c>
     </row>
     <row r="34" ht="18" customHeight="1">
       <c r="B34" s="15" t="n">
@@ -3743,6 +3816,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AJ34" s="34" t="n">
+        <v>1029.99</v>
+      </c>
     </row>
     <row r="35" ht="18" customHeight="1">
       <c r="B35" s="6" t="n">
@@ -3877,6 +3953,9 @@
       <c r="AI35" s="34" t="n">
         <v>1599.99</v>
       </c>
+      <c r="AJ35" s="34" t="n">
+        <v>1599.99</v>
+      </c>
     </row>
     <row r="36" ht="18" customHeight="1">
       <c r="B36" s="15" t="n">
@@ -4011,6 +4090,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AJ36" s="34" t="n">
+        <v>1699.99</v>
+      </c>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="B37" s="6" t="n">
@@ -4139,6 +4221,9 @@
       <c r="AI37" s="36" t="n">
         <v>3399.99</v>
       </c>
+      <c r="AJ37" s="36" t="n">
+        <v>3399.99</v>
+      </c>
     </row>
     <row r="38" ht="18" customHeight="1">
       <c r="B38" s="15" t="n">
@@ -4267,6 +4352,9 @@
       <c r="AI38" s="34" t="n">
         <v>2898.99</v>
       </c>
+      <c r="AJ38" s="34" t="n">
+        <v>2898.99</v>
+      </c>
     </row>
     <row r="39" ht="18" customHeight="1">
       <c r="B39" s="6" t="n">
@@ -4395,6 +4483,9 @@
       <c r="AI39" s="36" t="n">
         <v>3399.99</v>
       </c>
+      <c r="AJ39" s="36" t="n">
+        <v>3399.99</v>
+      </c>
     </row>
     <row r="40" ht="18" customHeight="1">
       <c r="B40" s="15" t="n">
@@ -4525,6 +4616,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AJ40" s="34" t="n">
+        <v>1029.99</v>
+      </c>
     </row>
     <row r="41" ht="18" customHeight="1">
       <c r="B41" s="6" t="n">
@@ -4653,6 +4747,9 @@
       <c r="AI41" s="36" t="n">
         <v>2159.99</v>
       </c>
+      <c r="AJ41" s="36" t="n">
+        <v>2159.99</v>
+      </c>
     </row>
     <row r="42" ht="18" customHeight="1">
       <c r="B42" s="15" t="n">
@@ -4792,6 +4889,9 @@
         <is>
           <t>—</t>
         </is>
+      </c>
+      <c r="AJ42" s="36" t="n">
+        <v>1999.99</v>
       </c>
     </row>
     <row r="43" ht="18" customHeight="1">
@@ -4975,6 +5075,9 @@
       <c r="AI44" s="34" t="n">
         <v>3599.99</v>
       </c>
+      <c r="AJ44" s="34" t="n">
+        <v>3599.99</v>
+      </c>
     </row>
     <row r="45" ht="5" customHeight="1"/>
     <row r="46" ht="22" customHeight="1">
@@ -5123,6 +5226,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AJ47" s="36" t="n">
+        <v>1999.99</v>
+      </c>
     </row>
     <row r="48" ht="18" customHeight="1">
       <c r="B48" s="15" t="n">
@@ -5257,6 +5363,9 @@
       <c r="AI48" s="34" t="n">
         <v>1599.99</v>
       </c>
+      <c r="AJ48" s="34" t="n">
+        <v>1599.99</v>
+      </c>
     </row>
     <row r="49" ht="18" customHeight="1">
       <c r="B49" s="6" t="n">
@@ -5389,6 +5498,9 @@
       <c r="AI49" s="34" t="n">
         <v>1849.99</v>
       </c>
+      <c r="AJ49" s="34" t="n">
+        <v>1849.99</v>
+      </c>
     </row>
     <row r="50" ht="18" customHeight="1">
       <c r="B50" s="15" t="n">
@@ -5514,6 +5626,11 @@
       </c>
       <c r="AI50" s="34" t="n">
         <v>2599.99</v>
+      </c>
+      <c r="AJ50" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
     </row>
     <row r="51" ht="18" customHeight="1">
@@ -5697,6 +5814,11 @@
       <c r="AI52" s="34" t="n">
         <v>2599.99</v>
       </c>
+      <c r="AJ52" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="53" ht="18" customHeight="1">
       <c r="B53" s="6" t="n">
@@ -5825,6 +5947,11 @@
       <c r="AI53" s="13" t="n">
         <v>1899.99</v>
       </c>
+      <c r="AJ53" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="54" ht="5" customHeight="1"/>
     <row r="55" ht="22" customHeight="1">
@@ -5957,6 +6084,9 @@
         <v>3599.99</v>
       </c>
       <c r="AI56" s="34" t="n">
+        <v>3599.99</v>
+      </c>
+      <c r="AJ56" s="34" t="n">
         <v>3599.99</v>
       </c>
     </row>
@@ -6265,6 +6395,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AJ62" s="34" t="n">
+        <v>127.99</v>
+      </c>
     </row>
     <row r="63" ht="18" customHeight="1">
       <c r="B63" s="6" t="n">
@@ -6415,6 +6548,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AJ63" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="64" ht="18" customHeight="1">
       <c r="B64" s="15" t="n">
@@ -6550,6 +6688,11 @@
       </c>
       <c r="AI64" s="36" t="n">
         <v>599.99</v>
+      </c>
+      <c r="AJ64" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
     </row>
     <row r="65" ht="18" customHeight="1">
@@ -6783,7 +6926,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:AI70"/>
+  <dimension ref="B1:AJ70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -6821,6 +6964,7 @@
     <col width="12" customWidth="1" min="33" max="33"/>
     <col width="12" customWidth="1" min="34" max="34"/>
     <col width="12" customWidth="1" min="35" max="35"/>
+    <col width="12" customWidth="1" min="36" max="36"/>
   </cols>
   <sheetData>
     <row r="1" ht="8" customHeight="1"/>
@@ -7010,6 +7154,11 @@
           <t>3/30</t>
         </is>
       </c>
+      <c r="AJ5" s="33" t="inlineStr">
+        <is>
+          <t>3/31</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="22" customHeight="1">
       <c r="B6" s="5" t="inlineStr">
@@ -7147,6 +7296,9 @@
       <c r="AI7" s="34" t="n">
         <v>89.98999999999999</v>
       </c>
+      <c r="AJ7" s="34" t="n">
+        <v>89.98999999999999</v>
+      </c>
     </row>
     <row r="8" ht="18" customHeight="1">
       <c r="B8" s="15" t="n">
@@ -7275,6 +7427,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AJ8" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="18" customHeight="1">
       <c r="B9" s="6" t="n">
@@ -7425,6 +7582,11 @@
         </is>
       </c>
       <c r="AI9" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AJ9" s="35" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -7607,6 +7769,9 @@
       <c r="AI11" s="34" t="n">
         <v>219.99</v>
       </c>
+      <c r="AJ11" s="34" t="n">
+        <v>219.99</v>
+      </c>
     </row>
     <row r="12" ht="18" customHeight="1">
       <c r="B12" s="15" t="n">
@@ -7737,6 +7902,9 @@
       <c r="AI12" s="36" t="n">
         <v>379.99</v>
       </c>
+      <c r="AJ12" s="36" t="n">
+        <v>379.99</v>
+      </c>
     </row>
     <row r="13" ht="18" customHeight="1">
       <c r="B13" s="6" t="n">
@@ -7889,6 +8057,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AJ13" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="5" customHeight="1"/>
     <row r="15" ht="22" customHeight="1">
@@ -8051,6 +8224,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AJ16" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="B17" s="6" t="n">
@@ -8177,6 +8355,9 @@
       <c r="AI17" s="36" t="n">
         <v>299.99</v>
       </c>
+      <c r="AJ17" s="36" t="n">
+        <v>299.99</v>
+      </c>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="B18" s="15" t="n">
@@ -8309,6 +8490,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AJ18" s="34" t="n">
+        <v>399.99</v>
+      </c>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="B19" s="6" t="n">
@@ -8441,6 +8625,9 @@
       <c r="AI19" s="34" t="n">
         <v>249.99</v>
       </c>
+      <c r="AJ19" s="34" t="n">
+        <v>249.99</v>
+      </c>
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="B20" s="15" t="n">
@@ -8571,6 +8758,9 @@
       <c r="AI20" s="34" t="n">
         <v>427.99</v>
       </c>
+      <c r="AJ20" s="34" t="n">
+        <v>427.99</v>
+      </c>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="B21" s="6" t="n">
@@ -8691,6 +8881,9 @@
       <c r="AI21" s="13" t="n">
         <v>449.99</v>
       </c>
+      <c r="AJ21" s="13" t="n">
+        <v>449.99</v>
+      </c>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="B22" s="15" t="n">
@@ -8827,6 +9020,9 @@
       <c r="AI22" s="34" t="n">
         <v>599.99</v>
       </c>
+      <c r="AJ22" s="34" t="n">
+        <v>599.99</v>
+      </c>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="B23" s="6" t="n">
@@ -8957,6 +9153,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AJ23" s="34" t="n">
+        <v>999.99</v>
+      </c>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="B24" s="15" t="n">
@@ -9109,6 +9308,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AJ24" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="18" customHeight="1">
       <c r="B25" s="6" t="n">
@@ -9245,6 +9449,11 @@
       <c r="AI25" s="34" t="n">
         <v>1199.99</v>
       </c>
+      <c r="AJ25" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="18" customHeight="1">
       <c r="B26" s="15" t="n">
@@ -9371,6 +9580,9 @@
       <c r="AI26" s="34" t="n">
         <v>1274.99</v>
       </c>
+      <c r="AJ26" s="34" t="n">
+        <v>1274.99</v>
+      </c>
     </row>
     <row r="27" ht="5" customHeight="1"/>
     <row r="28" ht="22" customHeight="1">
@@ -9511,6 +9723,9 @@
       <c r="AI29" s="34" t="n">
         <v>369.99</v>
       </c>
+      <c r="AJ29" s="34" t="n">
+        <v>369.99</v>
+      </c>
     </row>
     <row r="30" ht="18" customHeight="1">
       <c r="B30" s="15" t="n">
@@ -9641,6 +9856,9 @@
       <c r="AI30" s="34" t="n">
         <v>579.99</v>
       </c>
+      <c r="AJ30" s="34" t="n">
+        <v>579.99</v>
+      </c>
     </row>
     <row r="31" ht="18" customHeight="1">
       <c r="B31" s="6" t="n">
@@ -9773,6 +9991,11 @@
       <c r="AI31" s="13" t="n">
         <v>699.99</v>
       </c>
+      <c r="AJ31" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="18" customHeight="1">
       <c r="B32" s="15" t="n">
@@ -9903,6 +10126,9 @@
       <c r="AI32" s="34" t="n">
         <v>759.99</v>
       </c>
+      <c r="AJ32" s="34" t="n">
+        <v>759.99</v>
+      </c>
     </row>
     <row r="33" ht="18" customHeight="1">
       <c r="B33" s="6" t="n">
@@ -10037,6 +10263,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AJ33" s="34" t="n">
+        <v>799.99</v>
+      </c>
     </row>
     <row r="34" ht="18" customHeight="1">
       <c r="B34" s="15" t="n">
@@ -10163,6 +10392,9 @@
       <c r="AI34" s="34" t="n">
         <v>1274.99</v>
       </c>
+      <c r="AJ34" s="34" t="n">
+        <v>1274.99</v>
+      </c>
     </row>
     <row r="35" ht="18" customHeight="1">
       <c r="B35" s="6" t="n">
@@ -10291,6 +10523,9 @@
       <c r="AI35" s="34" t="n">
         <v>1799.99</v>
       </c>
+      <c r="AJ35" s="13" t="n">
+        <v>1399.99</v>
+      </c>
     </row>
     <row r="36" ht="18" customHeight="1">
       <c r="B36" s="15" t="n">
@@ -10417,6 +10652,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AJ36" s="34" t="n">
+        <v>1975.99</v>
+      </c>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="B37" s="6" t="n">
@@ -10553,6 +10791,9 @@
       <c r="AI37" s="34" t="n">
         <v>2699.99</v>
       </c>
+      <c r="AJ37" s="34" t="n">
+        <v>2699.99</v>
+      </c>
     </row>
     <row r="38" ht="5" customHeight="1"/>
     <row r="39" ht="22" customHeight="1">
@@ -10691,6 +10932,9 @@
       <c r="AI40" s="34" t="n">
         <v>740.99</v>
       </c>
+      <c r="AJ40" s="34" t="n">
+        <v>740.99</v>
+      </c>
     </row>
     <row r="41" ht="18" customHeight="1">
       <c r="B41" s="6" t="n">
@@ -10825,6 +11069,9 @@
       <c r="AI41" s="13" t="n">
         <v>549.99</v>
       </c>
+      <c r="AJ41" s="13" t="n">
+        <v>549.99</v>
+      </c>
     </row>
     <row r="42" ht="18" customHeight="1">
       <c r="B42" s="15" t="n">
@@ -10959,6 +11206,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AJ42" s="34" t="n">
+        <v>799.99</v>
+      </c>
     </row>
     <row r="43" ht="18" customHeight="1">
       <c r="B43" s="6" t="n">
@@ -11093,6 +11343,9 @@
       <c r="AI43" s="34" t="n">
         <v>949.99</v>
       </c>
+      <c r="AJ43" s="34" t="n">
+        <v>949.99</v>
+      </c>
     </row>
     <row r="44" ht="18" customHeight="1">
       <c r="B44" s="15" t="n">
@@ -11217,6 +11470,9 @@
       <c r="AI44" s="34" t="n">
         <v>1139.99</v>
       </c>
+      <c r="AJ44" s="34" t="n">
+        <v>1139.99</v>
+      </c>
     </row>
     <row r="45" ht="18" customHeight="1">
       <c r="B45" s="6" t="n">
@@ -11341,6 +11597,9 @@
       <c r="AI45" s="34" t="n">
         <v>1529.99</v>
       </c>
+      <c r="AJ45" s="34" t="n">
+        <v>1529.99</v>
+      </c>
     </row>
     <row r="46" ht="18" customHeight="1">
       <c r="B46" s="15" t="n">
@@ -11493,6 +11752,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AJ46" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="47" ht="18" customHeight="1">
       <c r="B47" s="6" t="n">
@@ -11623,6 +11887,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AJ47" s="34" t="n">
+        <v>2999.99</v>
+      </c>
     </row>
     <row r="48" ht="18" customHeight="1">
       <c r="B48" s="15" t="n">
@@ -11759,6 +12026,9 @@
       <c r="AI48" s="36" t="n">
         <v>3799.99</v>
       </c>
+      <c r="AJ48" s="36" t="n">
+        <v>3799.99</v>
+      </c>
     </row>
     <row r="49" ht="5" customHeight="1"/>
     <row r="50" ht="22" customHeight="1">
@@ -11893,6 +12163,9 @@
       <c r="AI51" s="34" t="n">
         <v>798.99</v>
       </c>
+      <c r="AJ51" s="34" t="n">
+        <v>798.99</v>
+      </c>
     </row>
     <row r="52" ht="18" customHeight="1">
       <c r="B52" s="15" t="n">
@@ -12019,6 +12292,9 @@
       <c r="AI52" s="34" t="n">
         <v>798.99</v>
       </c>
+      <c r="AJ52" s="34" t="n">
+        <v>798.99</v>
+      </c>
     </row>
     <row r="53" ht="18" customHeight="1">
       <c r="B53" s="6" t="n">
@@ -12151,6 +12427,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AJ53" s="34" t="n">
+        <v>1499.99</v>
+      </c>
     </row>
     <row r="54" ht="18" customHeight="1">
       <c r="B54" s="15" t="n">
@@ -12277,6 +12556,9 @@
       <c r="AI54" s="34" t="n">
         <v>899.99</v>
       </c>
+      <c r="AJ54" s="34" t="n">
+        <v>899.99</v>
+      </c>
     </row>
     <row r="55" ht="18" customHeight="1">
       <c r="B55" s="6" t="n">
@@ -12405,6 +12687,9 @@
       <c r="AI55" s="13" t="n">
         <v>1299.99</v>
       </c>
+      <c r="AJ55" s="13" t="n">
+        <v>1299.99</v>
+      </c>
     </row>
     <row r="56" ht="18" customHeight="1">
       <c r="B56" s="15" t="n">
@@ -12537,6 +12822,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AJ56" s="34" t="n">
+        <v>2799.99</v>
+      </c>
     </row>
     <row r="57" ht="18" customHeight="1">
       <c r="B57" s="6" t="n">
@@ -12664,6 +12952,9 @@
         <is>
           <t>—</t>
         </is>
+      </c>
+      <c r="AJ57" s="13" t="n">
+        <v>1600.99</v>
       </c>
     </row>
     <row r="58" ht="18" customHeight="1">
@@ -12859,6 +13150,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AJ61" s="34" t="n">
+        <v>999.99</v>
+      </c>
     </row>
     <row r="62" ht="18" customHeight="1">
       <c r="B62" s="15" t="n">
@@ -13047,6 +13341,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AJ63" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="64" ht="18" customHeight="1">
       <c r="B64" s="15" t="n">
@@ -13171,6 +13470,9 @@
         <v>2549.99</v>
       </c>
       <c r="AI64" s="34" t="n">
+        <v>2549.99</v>
+      </c>
+      <c r="AJ64" s="34" t="n">
         <v>2549.99</v>
       </c>
     </row>
@@ -13475,6 +13777,9 @@
         <v>1899.99</v>
       </c>
       <c r="AI70" s="34" t="n">
+        <v>1899.99</v>
+      </c>
+      <c r="AJ70" s="34" t="n">
         <v>1899.99</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Price check — 04/01/2026
</commit_message>
<xml_diff>
--- a/PriceBook_Combined_Final.xlsx
+++ b/PriceBook_Combined_Final.xlsx
@@ -709,7 +709,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:AJ67"/>
+  <dimension ref="B1:AK67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -748,6 +748,7 @@
     <col width="12" customWidth="1" min="34" max="34"/>
     <col width="12" customWidth="1" min="35" max="35"/>
     <col width="12" customWidth="1" min="36" max="36"/>
+    <col width="12" customWidth="1" min="37" max="37"/>
   </cols>
   <sheetData>
     <row r="1" ht="8" customHeight="1"/>
@@ -942,6 +943,11 @@
           <t>3/31</t>
         </is>
       </c>
+      <c r="AK5" s="33" t="inlineStr">
+        <is>
+          <t>4/1</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="22" customHeight="1">
       <c r="B6" s="5" t="inlineStr">
@@ -1072,6 +1078,9 @@
       <c r="AJ7" s="34" t="n">
         <v>449.99</v>
       </c>
+      <c r="AK7" s="34" t="n">
+        <v>449.99</v>
+      </c>
     </row>
     <row r="8" ht="18" customHeight="1">
       <c r="B8" s="15" t="n">
@@ -1223,6 +1232,11 @@
       <c r="AJ8" s="36" t="n">
         <v>809.99</v>
       </c>
+      <c r="AK8" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="18" customHeight="1">
       <c r="B9" s="6" t="n">
@@ -1374,6 +1388,11 @@
       <c r="AJ9" s="36" t="n">
         <v>809.99</v>
       </c>
+      <c r="AK9" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="18" customHeight="1">
       <c r="B10" s="15" t="n">
@@ -1497,6 +1516,9 @@
       <c r="AJ10" s="34" t="n">
         <v>449.99</v>
       </c>
+      <c r="AK10" s="34" t="n">
+        <v>449.99</v>
+      </c>
     </row>
     <row r="11" ht="18" customHeight="1">
       <c r="B11" s="6" t="n">
@@ -1648,6 +1670,11 @@
       <c r="AJ11" s="36" t="n">
         <v>809.99</v>
       </c>
+      <c r="AK11" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="18" customHeight="1">
       <c r="B12" s="15" t="n">
@@ -1777,6 +1804,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AK12" s="36" t="n">
+        <v>839.99</v>
+      </c>
     </row>
     <row r="13" ht="5" customHeight="1"/>
     <row r="14" ht="22" customHeight="1">
@@ -1924,6 +1954,9 @@
       <c r="AJ15" s="34" t="n">
         <v>599.99</v>
       </c>
+      <c r="AK15" s="34" t="n">
+        <v>599.99</v>
+      </c>
     </row>
     <row r="16" ht="18" customHeight="1">
       <c r="B16" s="15" t="n">
@@ -2057,6 +2090,9 @@
       <c r="AJ16" s="36" t="n">
         <v>809.99</v>
       </c>
+      <c r="AK16" s="36" t="n">
+        <v>809.99</v>
+      </c>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="B17" s="6" t="n">
@@ -2214,6 +2250,11 @@
         </is>
       </c>
       <c r="AJ17" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AK17" s="35" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2405,6 +2446,9 @@
       <c r="AJ19" s="34" t="n">
         <v>2199.99</v>
       </c>
+      <c r="AK19" s="34" t="n">
+        <v>2199.99</v>
+      </c>
     </row>
     <row r="20" ht="5" customHeight="1"/>
     <row r="21" ht="22" customHeight="1">
@@ -2548,6 +2592,9 @@
       <c r="AJ22" s="34" t="n">
         <v>1098.99</v>
       </c>
+      <c r="AK22" s="34" t="n">
+        <v>1098.99</v>
+      </c>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="B23" s="6" t="n">
@@ -2683,6 +2730,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AK23" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="B24" s="15" t="n">
@@ -2814,6 +2866,11 @@
         <v>1198.99</v>
       </c>
       <c r="AJ24" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AK24" s="35" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -3011,6 +3068,11 @@
       <c r="AJ26" s="34" t="n">
         <v>1599.99</v>
       </c>
+      <c r="AK26" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="18" customHeight="1">
       <c r="B27" s="6" t="n">
@@ -3146,6 +3208,9 @@
       <c r="AJ27" s="34" t="n">
         <v>1799.99</v>
       </c>
+      <c r="AK27" s="34" t="n">
+        <v>1799.99</v>
+      </c>
     </row>
     <row r="28" ht="18" customHeight="1">
       <c r="B28" s="15" t="n">
@@ -3275,6 +3340,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AK28" s="34" t="n">
+        <v>1479.99</v>
+      </c>
     </row>
     <row r="29" ht="18" customHeight="1">
       <c r="B29" s="6" t="n">
@@ -3410,6 +3478,9 @@
       <c r="AJ29" s="34" t="n">
         <v>1799.99</v>
       </c>
+      <c r="AK29" s="34" t="n">
+        <v>1799.99</v>
+      </c>
     </row>
     <row r="30" ht="18" customHeight="1">
       <c r="B30" s="15" t="n">
@@ -3545,6 +3616,9 @@
       <c r="AJ30" s="34" t="n">
         <v>1799.99</v>
       </c>
+      <c r="AK30" s="34" t="n">
+        <v>1799.99</v>
+      </c>
     </row>
     <row r="31" ht="5" customHeight="1"/>
     <row r="32" ht="22" customHeight="1">
@@ -3686,6 +3760,9 @@
       <c r="AJ33" s="34" t="n">
         <v>1029.99</v>
       </c>
+      <c r="AK33" s="34" t="n">
+        <v>1029.99</v>
+      </c>
     </row>
     <row r="34" ht="18" customHeight="1">
       <c r="B34" s="15" t="n">
@@ -3819,6 +3896,9 @@
       <c r="AJ34" s="34" t="n">
         <v>1029.99</v>
       </c>
+      <c r="AK34" s="34" t="n">
+        <v>1029.99</v>
+      </c>
     </row>
     <row r="35" ht="18" customHeight="1">
       <c r="B35" s="6" t="n">
@@ -3956,6 +4036,11 @@
       <c r="AJ35" s="34" t="n">
         <v>1599.99</v>
       </c>
+      <c r="AK35" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="18" customHeight="1">
       <c r="B36" s="15" t="n">
@@ -4093,6 +4178,9 @@
       <c r="AJ36" s="34" t="n">
         <v>1699.99</v>
       </c>
+      <c r="AK36" s="34" t="n">
+        <v>1699.99</v>
+      </c>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="B37" s="6" t="n">
@@ -4224,6 +4312,9 @@
       <c r="AJ37" s="36" t="n">
         <v>3399.99</v>
       </c>
+      <c r="AK37" s="36" t="n">
+        <v>3399.99</v>
+      </c>
     </row>
     <row r="38" ht="18" customHeight="1">
       <c r="B38" s="15" t="n">
@@ -4355,6 +4446,11 @@
       <c r="AJ38" s="34" t="n">
         <v>2898.99</v>
       </c>
+      <c r="AK38" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="18" customHeight="1">
       <c r="B39" s="6" t="n">
@@ -4486,6 +4582,9 @@
       <c r="AJ39" s="36" t="n">
         <v>3399.99</v>
       </c>
+      <c r="AK39" s="36" t="n">
+        <v>3399.99</v>
+      </c>
     </row>
     <row r="40" ht="18" customHeight="1">
       <c r="B40" s="15" t="n">
@@ -4619,6 +4718,9 @@
       <c r="AJ40" s="34" t="n">
         <v>1029.99</v>
       </c>
+      <c r="AK40" s="34" t="n">
+        <v>1029.99</v>
+      </c>
     </row>
     <row r="41" ht="18" customHeight="1">
       <c r="B41" s="6" t="n">
@@ -4750,6 +4852,9 @@
       <c r="AJ41" s="36" t="n">
         <v>2159.99</v>
       </c>
+      <c r="AK41" s="36" t="n">
+        <v>2159.99</v>
+      </c>
     </row>
     <row r="42" ht="18" customHeight="1">
       <c r="B42" s="15" t="n">
@@ -4891,6 +4996,9 @@
         </is>
       </c>
       <c r="AJ42" s="36" t="n">
+        <v>1999.99</v>
+      </c>
+      <c r="AK42" s="36" t="n">
         <v>1999.99</v>
       </c>
     </row>
@@ -5078,6 +5186,11 @@
       <c r="AJ44" s="34" t="n">
         <v>3599.99</v>
       </c>
+      <c r="AK44" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="45" ht="5" customHeight="1"/>
     <row r="46" ht="22" customHeight="1">
@@ -5229,6 +5342,9 @@
       <c r="AJ47" s="36" t="n">
         <v>1999.99</v>
       </c>
+      <c r="AK47" s="36" t="n">
+        <v>1999.99</v>
+      </c>
     </row>
     <row r="48" ht="18" customHeight="1">
       <c r="B48" s="15" t="n">
@@ -5366,6 +5482,11 @@
       <c r="AJ48" s="34" t="n">
         <v>1599.99</v>
       </c>
+      <c r="AK48" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="49" ht="18" customHeight="1">
       <c r="B49" s="6" t="n">
@@ -5501,6 +5622,9 @@
       <c r="AJ49" s="34" t="n">
         <v>1849.99</v>
       </c>
+      <c r="AK49" s="34" t="n">
+        <v>1849.99</v>
+      </c>
     </row>
     <row r="50" ht="18" customHeight="1">
       <c r="B50" s="15" t="n">
@@ -5631,6 +5755,9 @@
         <is>
           <t>—</t>
         </is>
+      </c>
+      <c r="AK50" s="34" t="n">
+        <v>2599.99</v>
       </c>
     </row>
     <row r="51" ht="18" customHeight="1">
@@ -5819,6 +5946,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AK52" s="34" t="n">
+        <v>2599.99</v>
+      </c>
     </row>
     <row r="53" ht="18" customHeight="1">
       <c r="B53" s="6" t="n">
@@ -5952,6 +6082,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AK53" s="13" t="n">
+        <v>1899.99</v>
+      </c>
     </row>
     <row r="54" ht="5" customHeight="1"/>
     <row r="55" ht="22" customHeight="1">
@@ -6088,6 +6221,11 @@
       </c>
       <c r="AJ56" s="34" t="n">
         <v>3599.99</v>
+      </c>
+      <c r="AK56" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
     </row>
     <row r="57" ht="18" customHeight="1">
@@ -6398,6 +6536,9 @@
       <c r="AJ62" s="34" t="n">
         <v>127.99</v>
       </c>
+      <c r="AK62" s="34" t="n">
+        <v>127.99</v>
+      </c>
     </row>
     <row r="63" ht="18" customHeight="1">
       <c r="B63" s="6" t="n">
@@ -6553,6 +6694,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AK63" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="64" ht="18" customHeight="1">
       <c r="B64" s="15" t="n">
@@ -6693,6 +6839,9 @@
         <is>
           <t>—</t>
         </is>
+      </c>
+      <c r="AK64" s="36" t="n">
+        <v>599.99</v>
       </c>
     </row>
     <row r="65" ht="18" customHeight="1">
@@ -6926,7 +7075,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:AJ70"/>
+  <dimension ref="B1:AK70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -6965,6 +7114,7 @@
     <col width="12" customWidth="1" min="34" max="34"/>
     <col width="12" customWidth="1" min="35" max="35"/>
     <col width="12" customWidth="1" min="36" max="36"/>
+    <col width="12" customWidth="1" min="37" max="37"/>
   </cols>
   <sheetData>
     <row r="1" ht="8" customHeight="1"/>
@@ -7159,6 +7309,11 @@
           <t>3/31</t>
         </is>
       </c>
+      <c r="AK5" s="33" t="inlineStr">
+        <is>
+          <t>4/1</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="22" customHeight="1">
       <c r="B6" s="5" t="inlineStr">
@@ -7299,6 +7454,9 @@
       <c r="AJ7" s="34" t="n">
         <v>89.98999999999999</v>
       </c>
+      <c r="AK7" s="34" t="n">
+        <v>89.98999999999999</v>
+      </c>
     </row>
     <row r="8" ht="18" customHeight="1">
       <c r="B8" s="15" t="n">
@@ -7432,6 +7590,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AK8" s="34" t="n">
+        <v>194.99</v>
+      </c>
     </row>
     <row r="9" ht="18" customHeight="1">
       <c r="B9" s="6" t="n">
@@ -7587,6 +7748,11 @@
         </is>
       </c>
       <c r="AJ9" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AK9" s="35" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -7772,6 +7938,9 @@
       <c r="AJ11" s="34" t="n">
         <v>219.99</v>
       </c>
+      <c r="AK11" s="34" t="n">
+        <v>219.99</v>
+      </c>
     </row>
     <row r="12" ht="18" customHeight="1">
       <c r="B12" s="15" t="n">
@@ -7905,6 +8074,9 @@
       <c r="AJ12" s="36" t="n">
         <v>379.99</v>
       </c>
+      <c r="AK12" s="36" t="n">
+        <v>379.99</v>
+      </c>
     </row>
     <row r="13" ht="18" customHeight="1">
       <c r="B13" s="6" t="n">
@@ -8062,6 +8234,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AK13" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="5" customHeight="1"/>
     <row r="15" ht="22" customHeight="1">
@@ -8229,6 +8406,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AK16" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="B17" s="6" t="n">
@@ -8358,6 +8540,9 @@
       <c r="AJ17" s="36" t="n">
         <v>299.99</v>
       </c>
+      <c r="AK17" s="36" t="n">
+        <v>299.99</v>
+      </c>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="B18" s="15" t="n">
@@ -8493,6 +8678,11 @@
       <c r="AJ18" s="34" t="n">
         <v>399.99</v>
       </c>
+      <c r="AK18" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="B19" s="6" t="n">
@@ -8628,6 +8818,9 @@
       <c r="AJ19" s="34" t="n">
         <v>249.99</v>
       </c>
+      <c r="AK19" s="34" t="n">
+        <v>249.99</v>
+      </c>
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="B20" s="15" t="n">
@@ -8761,6 +8954,9 @@
       <c r="AJ20" s="34" t="n">
         <v>427.99</v>
       </c>
+      <c r="AK20" s="34" t="n">
+        <v>427.99</v>
+      </c>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="B21" s="6" t="n">
@@ -8884,6 +9080,9 @@
       <c r="AJ21" s="13" t="n">
         <v>449.99</v>
       </c>
+      <c r="AK21" s="13" t="n">
+        <v>449.99</v>
+      </c>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="B22" s="15" t="n">
@@ -9023,6 +9222,11 @@
       <c r="AJ22" s="34" t="n">
         <v>599.99</v>
       </c>
+      <c r="AK22" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="B23" s="6" t="n">
@@ -9156,6 +9360,9 @@
       <c r="AJ23" s="34" t="n">
         <v>999.99</v>
       </c>
+      <c r="AK23" s="34" t="n">
+        <v>999.99</v>
+      </c>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="B24" s="15" t="n">
@@ -9313,6 +9520,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AK24" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="18" customHeight="1">
       <c r="B25" s="6" t="n">
@@ -9454,6 +9666,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AK25" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="18" customHeight="1">
       <c r="B26" s="15" t="n">
@@ -9583,6 +9800,9 @@
       <c r="AJ26" s="34" t="n">
         <v>1274.99</v>
       </c>
+      <c r="AK26" s="34" t="n">
+        <v>1274.99</v>
+      </c>
     </row>
     <row r="27" ht="5" customHeight="1"/>
     <row r="28" ht="22" customHeight="1">
@@ -9726,6 +9946,11 @@
       <c r="AJ29" s="34" t="n">
         <v>369.99</v>
       </c>
+      <c r="AK29" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="18" customHeight="1">
       <c r="B30" s="15" t="n">
@@ -9859,6 +10084,9 @@
       <c r="AJ30" s="34" t="n">
         <v>579.99</v>
       </c>
+      <c r="AK30" s="34" t="n">
+        <v>579.99</v>
+      </c>
     </row>
     <row r="31" ht="18" customHeight="1">
       <c r="B31" s="6" t="n">
@@ -9996,6 +10224,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AK31" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="18" customHeight="1">
       <c r="B32" s="15" t="n">
@@ -10129,6 +10362,9 @@
       <c r="AJ32" s="34" t="n">
         <v>759.99</v>
       </c>
+      <c r="AK32" s="34" t="n">
+        <v>759.99</v>
+      </c>
     </row>
     <row r="33" ht="18" customHeight="1">
       <c r="B33" s="6" t="n">
@@ -10266,6 +10502,9 @@
       <c r="AJ33" s="34" t="n">
         <v>799.99</v>
       </c>
+      <c r="AK33" s="34" t="n">
+        <v>799.99</v>
+      </c>
     </row>
     <row r="34" ht="18" customHeight="1">
       <c r="B34" s="15" t="n">
@@ -10395,6 +10634,9 @@
       <c r="AJ34" s="34" t="n">
         <v>1274.99</v>
       </c>
+      <c r="AK34" s="34" t="n">
+        <v>1274.99</v>
+      </c>
     </row>
     <row r="35" ht="18" customHeight="1">
       <c r="B35" s="6" t="n">
@@ -10526,6 +10768,9 @@
       <c r="AJ35" s="13" t="n">
         <v>1399.99</v>
       </c>
+      <c r="AK35" s="13" t="n">
+        <v>1599.99</v>
+      </c>
     </row>
     <row r="36" ht="18" customHeight="1">
       <c r="B36" s="15" t="n">
@@ -10655,6 +10900,9 @@
       <c r="AJ36" s="34" t="n">
         <v>1975.99</v>
       </c>
+      <c r="AK36" s="34" t="n">
+        <v>1975.99</v>
+      </c>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="B37" s="6" t="n">
@@ -10794,6 +11042,9 @@
       <c r="AJ37" s="34" t="n">
         <v>2699.99</v>
       </c>
+      <c r="AK37" s="34" t="n">
+        <v>2699.99</v>
+      </c>
     </row>
     <row r="38" ht="5" customHeight="1"/>
     <row r="39" ht="22" customHeight="1">
@@ -10935,6 +11186,9 @@
       <c r="AJ40" s="34" t="n">
         <v>740.99</v>
       </c>
+      <c r="AK40" s="34" t="n">
+        <v>740.99</v>
+      </c>
     </row>
     <row r="41" ht="18" customHeight="1">
       <c r="B41" s="6" t="n">
@@ -11072,6 +11326,9 @@
       <c r="AJ41" s="13" t="n">
         <v>549.99</v>
       </c>
+      <c r="AK41" s="13" t="n">
+        <v>549.99</v>
+      </c>
     </row>
     <row r="42" ht="18" customHeight="1">
       <c r="B42" s="15" t="n">
@@ -11209,6 +11466,9 @@
       <c r="AJ42" s="34" t="n">
         <v>799.99</v>
       </c>
+      <c r="AK42" s="34" t="n">
+        <v>799.99</v>
+      </c>
     </row>
     <row r="43" ht="18" customHeight="1">
       <c r="B43" s="6" t="n">
@@ -11346,6 +11606,9 @@
       <c r="AJ43" s="34" t="n">
         <v>949.99</v>
       </c>
+      <c r="AK43" s="34" t="n">
+        <v>949.99</v>
+      </c>
     </row>
     <row r="44" ht="18" customHeight="1">
       <c r="B44" s="15" t="n">
@@ -11473,6 +11736,11 @@
       <c r="AJ44" s="34" t="n">
         <v>1139.99</v>
       </c>
+      <c r="AK44" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="45" ht="18" customHeight="1">
       <c r="B45" s="6" t="n">
@@ -11600,6 +11868,9 @@
       <c r="AJ45" s="34" t="n">
         <v>1529.99</v>
       </c>
+      <c r="AK45" s="34" t="n">
+        <v>1529.99</v>
+      </c>
     </row>
     <row r="46" ht="18" customHeight="1">
       <c r="B46" s="15" t="n">
@@ -11757,6 +12028,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AK46" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="47" ht="18" customHeight="1">
       <c r="B47" s="6" t="n">
@@ -11890,6 +12166,9 @@
       <c r="AJ47" s="34" t="n">
         <v>2999.99</v>
       </c>
+      <c r="AK47" s="34" t="n">
+        <v>2999.99</v>
+      </c>
     </row>
     <row r="48" ht="18" customHeight="1">
       <c r="B48" s="15" t="n">
@@ -12029,6 +12308,11 @@
       <c r="AJ48" s="36" t="n">
         <v>3799.99</v>
       </c>
+      <c r="AK48" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="49" ht="5" customHeight="1"/>
     <row r="50" ht="22" customHeight="1">
@@ -12166,6 +12450,9 @@
       <c r="AJ51" s="34" t="n">
         <v>798.99</v>
       </c>
+      <c r="AK51" s="34" t="n">
+        <v>798.99</v>
+      </c>
     </row>
     <row r="52" ht="18" customHeight="1">
       <c r="B52" s="15" t="n">
@@ -12295,6 +12582,9 @@
       <c r="AJ52" s="34" t="n">
         <v>798.99</v>
       </c>
+      <c r="AK52" s="34" t="n">
+        <v>798.99</v>
+      </c>
     </row>
     <row r="53" ht="18" customHeight="1">
       <c r="B53" s="6" t="n">
@@ -12430,6 +12720,11 @@
       <c r="AJ53" s="34" t="n">
         <v>1499.99</v>
       </c>
+      <c r="AK53" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="54" ht="18" customHeight="1">
       <c r="B54" s="15" t="n">
@@ -12559,6 +12854,9 @@
       <c r="AJ54" s="34" t="n">
         <v>899.99</v>
       </c>
+      <c r="AK54" s="34" t="n">
+        <v>899.99</v>
+      </c>
     </row>
     <row r="55" ht="18" customHeight="1">
       <c r="B55" s="6" t="n">
@@ -12690,6 +12988,11 @@
       <c r="AJ55" s="13" t="n">
         <v>1299.99</v>
       </c>
+      <c r="AK55" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="56" ht="18" customHeight="1">
       <c r="B56" s="15" t="n">
@@ -12825,6 +13128,9 @@
       <c r="AJ56" s="34" t="n">
         <v>2799.99</v>
       </c>
+      <c r="AK56" s="34" t="n">
+        <v>2799.99</v>
+      </c>
     </row>
     <row r="57" ht="18" customHeight="1">
       <c r="B57" s="6" t="n">
@@ -12954,6 +13260,9 @@
         </is>
       </c>
       <c r="AJ57" s="13" t="n">
+        <v>1600.99</v>
+      </c>
+      <c r="AK57" s="13" t="n">
         <v>1600.99</v>
       </c>
     </row>
@@ -13153,6 +13462,9 @@
       <c r="AJ61" s="34" t="n">
         <v>999.99</v>
       </c>
+      <c r="AK61" s="34" t="n">
+        <v>999.99</v>
+      </c>
     </row>
     <row r="62" ht="18" customHeight="1">
       <c r="B62" s="15" t="n">
@@ -13346,6 +13658,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AK63" s="34" t="n">
+        <v>1658.99</v>
+      </c>
     </row>
     <row r="64" ht="18" customHeight="1">
       <c r="B64" s="15" t="n">
@@ -13473,6 +13788,9 @@
         <v>2549.99</v>
       </c>
       <c r="AJ64" s="34" t="n">
+        <v>2549.99</v>
+      </c>
+      <c r="AK64" s="34" t="n">
         <v>2549.99</v>
       </c>
     </row>
@@ -13780,6 +14098,9 @@
         <v>1899.99</v>
       </c>
       <c r="AJ70" s="34" t="n">
+        <v>1899.99</v>
+      </c>
+      <c r="AK70" s="34" t="n">
         <v>1899.99</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Price check — 04/02/2026
</commit_message>
<xml_diff>
--- a/PriceBook_Combined_Final.xlsx
+++ b/PriceBook_Combined_Final.xlsx
@@ -709,7 +709,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:AK67"/>
+  <dimension ref="B1:AL67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -749,6 +749,7 @@
     <col width="12" customWidth="1" min="35" max="35"/>
     <col width="12" customWidth="1" min="36" max="36"/>
     <col width="12" customWidth="1" min="37" max="37"/>
+    <col width="12" customWidth="1" min="38" max="38"/>
   </cols>
   <sheetData>
     <row r="1" ht="8" customHeight="1"/>
@@ -948,6 +949,11 @@
           <t>4/1</t>
         </is>
       </c>
+      <c r="AL5" s="33" t="inlineStr">
+        <is>
+          <t>4/2</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="22" customHeight="1">
       <c r="B6" s="5" t="inlineStr">
@@ -1081,6 +1087,9 @@
       <c r="AK7" s="34" t="n">
         <v>449.99</v>
       </c>
+      <c r="AL7" s="34" t="n">
+        <v>449.99</v>
+      </c>
     </row>
     <row r="8" ht="18" customHeight="1">
       <c r="B8" s="15" t="n">
@@ -1237,6 +1246,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AL8" s="36" t="n">
+        <v>809.99</v>
+      </c>
     </row>
     <row r="9" ht="18" customHeight="1">
       <c r="B9" s="6" t="n">
@@ -1393,6 +1405,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AL9" s="36" t="n">
+        <v>809.99</v>
+      </c>
     </row>
     <row r="10" ht="18" customHeight="1">
       <c r="B10" s="15" t="n">
@@ -1519,6 +1534,9 @@
       <c r="AK10" s="34" t="n">
         <v>449.99</v>
       </c>
+      <c r="AL10" s="34" t="n">
+        <v>449.99</v>
+      </c>
     </row>
     <row r="11" ht="18" customHeight="1">
       <c r="B11" s="6" t="n">
@@ -1675,6 +1693,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AL11" s="36" t="n">
+        <v>809.99</v>
+      </c>
     </row>
     <row r="12" ht="18" customHeight="1">
       <c r="B12" s="15" t="n">
@@ -1807,6 +1828,9 @@
       <c r="AK12" s="36" t="n">
         <v>839.99</v>
       </c>
+      <c r="AL12" s="36" t="n">
+        <v>839.99</v>
+      </c>
     </row>
     <row r="13" ht="5" customHeight="1"/>
     <row r="14" ht="22" customHeight="1">
@@ -1957,6 +1981,9 @@
       <c r="AK15" s="34" t="n">
         <v>599.99</v>
       </c>
+      <c r="AL15" s="34" t="n">
+        <v>599.99</v>
+      </c>
     </row>
     <row r="16" ht="18" customHeight="1">
       <c r="B16" s="15" t="n">
@@ -2093,6 +2120,9 @@
       <c r="AK16" s="36" t="n">
         <v>809.99</v>
       </c>
+      <c r="AL16" s="36" t="n">
+        <v>809.99</v>
+      </c>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="B17" s="6" t="n">
@@ -2255,6 +2285,11 @@
         </is>
       </c>
       <c r="AK17" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AL17" s="35" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2449,6 +2484,11 @@
       <c r="AK19" s="34" t="n">
         <v>2199.99</v>
       </c>
+      <c r="AL19" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="5" customHeight="1"/>
     <row r="21" ht="22" customHeight="1">
@@ -2595,6 +2635,9 @@
       <c r="AK22" s="34" t="n">
         <v>1098.99</v>
       </c>
+      <c r="AL22" s="34" t="n">
+        <v>1098.99</v>
+      </c>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="B23" s="6" t="n">
@@ -2735,6 +2778,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AL23" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="B24" s="15" t="n">
@@ -2871,6 +2919,11 @@
         </is>
       </c>
       <c r="AK24" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AL24" s="35" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -3073,6 +3126,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AL26" s="34" t="n">
+        <v>1599.99</v>
+      </c>
     </row>
     <row r="27" ht="18" customHeight="1">
       <c r="B27" s="6" t="n">
@@ -3211,6 +3267,9 @@
       <c r="AK27" s="34" t="n">
         <v>1799.99</v>
       </c>
+      <c r="AL27" s="13" t="n">
+        <v>1649.99</v>
+      </c>
     </row>
     <row r="28" ht="18" customHeight="1">
       <c r="B28" s="15" t="n">
@@ -3343,6 +3402,9 @@
       <c r="AK28" s="34" t="n">
         <v>1479.99</v>
       </c>
+      <c r="AL28" s="34" t="n">
+        <v>1479.99</v>
+      </c>
     </row>
     <row r="29" ht="18" customHeight="1">
       <c r="B29" s="6" t="n">
@@ -3481,6 +3543,9 @@
       <c r="AK29" s="34" t="n">
         <v>1799.99</v>
       </c>
+      <c r="AL29" s="13" t="n">
+        <v>1649.99</v>
+      </c>
     </row>
     <row r="30" ht="18" customHeight="1">
       <c r="B30" s="15" t="n">
@@ -3619,6 +3684,9 @@
       <c r="AK30" s="34" t="n">
         <v>1799.99</v>
       </c>
+      <c r="AL30" s="13" t="n">
+        <v>1649.99</v>
+      </c>
     </row>
     <row r="31" ht="5" customHeight="1"/>
     <row r="32" ht="22" customHeight="1">
@@ -3763,6 +3831,11 @@
       <c r="AK33" s="34" t="n">
         <v>1029.99</v>
       </c>
+      <c r="AL33" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="18" customHeight="1">
       <c r="B34" s="15" t="n">
@@ -3899,6 +3972,11 @@
       <c r="AK34" s="34" t="n">
         <v>1029.99</v>
       </c>
+      <c r="AL34" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="18" customHeight="1">
       <c r="B35" s="6" t="n">
@@ -4041,6 +4119,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AL35" s="34" t="n">
+        <v>1599.99</v>
+      </c>
     </row>
     <row r="36" ht="18" customHeight="1">
       <c r="B36" s="15" t="n">
@@ -4181,6 +4262,9 @@
       <c r="AK36" s="34" t="n">
         <v>1699.99</v>
       </c>
+      <c r="AL36" s="34" t="n">
+        <v>1699.99</v>
+      </c>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="B37" s="6" t="n">
@@ -4315,6 +4399,9 @@
       <c r="AK37" s="36" t="n">
         <v>3399.99</v>
       </c>
+      <c r="AL37" s="36" t="n">
+        <v>3399.99</v>
+      </c>
     </row>
     <row r="38" ht="18" customHeight="1">
       <c r="B38" s="15" t="n">
@@ -4451,6 +4538,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AL38" s="34" t="n">
+        <v>2898.99</v>
+      </c>
     </row>
     <row r="39" ht="18" customHeight="1">
       <c r="B39" s="6" t="n">
@@ -4585,6 +4675,9 @@
       <c r="AK39" s="36" t="n">
         <v>3399.99</v>
       </c>
+      <c r="AL39" s="36" t="n">
+        <v>3399.99</v>
+      </c>
     </row>
     <row r="40" ht="18" customHeight="1">
       <c r="B40" s="15" t="n">
@@ -4721,6 +4814,11 @@
       <c r="AK40" s="34" t="n">
         <v>1029.99</v>
       </c>
+      <c r="AL40" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="18" customHeight="1">
       <c r="B41" s="6" t="n">
@@ -4855,6 +4953,11 @@
       <c r="AK41" s="36" t="n">
         <v>2159.99</v>
       </c>
+      <c r="AL41" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="18" customHeight="1">
       <c r="B42" s="15" t="n">
@@ -4999,6 +5102,9 @@
         <v>1999.99</v>
       </c>
       <c r="AK42" s="36" t="n">
+        <v>1999.99</v>
+      </c>
+      <c r="AL42" s="36" t="n">
         <v>1999.99</v>
       </c>
     </row>
@@ -5191,6 +5297,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AL44" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="45" ht="5" customHeight="1"/>
     <row r="46" ht="22" customHeight="1">
@@ -5345,6 +5456,9 @@
       <c r="AK47" s="36" t="n">
         <v>1999.99</v>
       </c>
+      <c r="AL47" s="36" t="n">
+        <v>1999.99</v>
+      </c>
     </row>
     <row r="48" ht="18" customHeight="1">
       <c r="B48" s="15" t="n">
@@ -5487,6 +5601,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AL48" s="34" t="n">
+        <v>1599.99</v>
+      </c>
     </row>
     <row r="49" ht="18" customHeight="1">
       <c r="B49" s="6" t="n">
@@ -5625,6 +5742,9 @@
       <c r="AK49" s="34" t="n">
         <v>1849.99</v>
       </c>
+      <c r="AL49" s="34" t="n">
+        <v>1849.99</v>
+      </c>
     </row>
     <row r="50" ht="18" customHeight="1">
       <c r="B50" s="15" t="n">
@@ -5757,6 +5877,9 @@
         </is>
       </c>
       <c r="AK50" s="34" t="n">
+        <v>2599.99</v>
+      </c>
+      <c r="AL50" s="34" t="n">
         <v>2599.99</v>
       </c>
     </row>
@@ -5949,6 +6072,9 @@
       <c r="AK52" s="34" t="n">
         <v>2599.99</v>
       </c>
+      <c r="AL52" s="34" t="n">
+        <v>2599.99</v>
+      </c>
     </row>
     <row r="53" ht="18" customHeight="1">
       <c r="B53" s="6" t="n">
@@ -6085,6 +6211,9 @@
       <c r="AK53" s="13" t="n">
         <v>1899.99</v>
       </c>
+      <c r="AL53" s="13" t="n">
+        <v>1899.99</v>
+      </c>
     </row>
     <row r="54" ht="5" customHeight="1"/>
     <row r="55" ht="22" customHeight="1">
@@ -6223,6 +6352,11 @@
         <v>3599.99</v>
       </c>
       <c r="AK56" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AL56" s="35" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -6539,6 +6673,9 @@
       <c r="AK62" s="34" t="n">
         <v>127.99</v>
       </c>
+      <c r="AL62" s="34" t="n">
+        <v>127.99</v>
+      </c>
     </row>
     <row r="63" ht="18" customHeight="1">
       <c r="B63" s="6" t="n">
@@ -6699,6 +6836,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AL63" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="64" ht="18" customHeight="1">
       <c r="B64" s="15" t="n">
@@ -6842,6 +6984,11 @@
       </c>
       <c r="AK64" s="36" t="n">
         <v>599.99</v>
+      </c>
+      <c r="AL64" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
     </row>
     <row r="65" ht="18" customHeight="1">
@@ -7075,7 +7222,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:AK70"/>
+  <dimension ref="B1:AL70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -7115,6 +7262,7 @@
     <col width="12" customWidth="1" min="35" max="35"/>
     <col width="12" customWidth="1" min="36" max="36"/>
     <col width="12" customWidth="1" min="37" max="37"/>
+    <col width="12" customWidth="1" min="38" max="38"/>
   </cols>
   <sheetData>
     <row r="1" ht="8" customHeight="1"/>
@@ -7314,6 +7462,11 @@
           <t>4/1</t>
         </is>
       </c>
+      <c r="AL5" s="33" t="inlineStr">
+        <is>
+          <t>4/2</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="22" customHeight="1">
       <c r="B6" s="5" t="inlineStr">
@@ -7457,6 +7610,9 @@
       <c r="AK7" s="34" t="n">
         <v>89.98999999999999</v>
       </c>
+      <c r="AL7" s="34" t="n">
+        <v>89.98999999999999</v>
+      </c>
     </row>
     <row r="8" ht="18" customHeight="1">
       <c r="B8" s="15" t="n">
@@ -7593,6 +7749,11 @@
       <c r="AK8" s="34" t="n">
         <v>194.99</v>
       </c>
+      <c r="AL8" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="18" customHeight="1">
       <c r="B9" s="6" t="n">
@@ -7753,6 +7914,11 @@
         </is>
       </c>
       <c r="AK9" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AL9" s="35" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -7941,6 +8107,9 @@
       <c r="AK11" s="34" t="n">
         <v>219.99</v>
       </c>
+      <c r="AL11" s="34" t="n">
+        <v>219.99</v>
+      </c>
     </row>
     <row r="12" ht="18" customHeight="1">
       <c r="B12" s="15" t="n">
@@ -8077,6 +8246,11 @@
       <c r="AK12" s="36" t="n">
         <v>379.99</v>
       </c>
+      <c r="AL12" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="18" customHeight="1">
       <c r="B13" s="6" t="n">
@@ -8239,6 +8413,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AL13" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="5" customHeight="1"/>
     <row r="15" ht="22" customHeight="1">
@@ -8411,6 +8590,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AL16" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="B17" s="6" t="n">
@@ -8543,6 +8727,11 @@
       <c r="AK17" s="36" t="n">
         <v>299.99</v>
       </c>
+      <c r="AL17" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="B18" s="15" t="n">
@@ -8683,6 +8872,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AL18" s="34" t="n">
+        <v>399.99</v>
+      </c>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="B19" s="6" t="n">
@@ -8821,6 +9013,11 @@
       <c r="AK19" s="34" t="n">
         <v>249.99</v>
       </c>
+      <c r="AL19" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="B20" s="15" t="n">
@@ -8957,6 +9154,9 @@
       <c r="AK20" s="34" t="n">
         <v>427.99</v>
       </c>
+      <c r="AL20" s="34" t="n">
+        <v>427.99</v>
+      </c>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="B21" s="6" t="n">
@@ -9083,6 +9283,9 @@
       <c r="AK21" s="13" t="n">
         <v>449.99</v>
       </c>
+      <c r="AL21" s="13" t="n">
+        <v>449.99</v>
+      </c>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="B22" s="15" t="n">
@@ -9227,6 +9430,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AL22" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="B23" s="6" t="n">
@@ -9363,6 +9571,9 @@
       <c r="AK23" s="34" t="n">
         <v>999.99</v>
       </c>
+      <c r="AL23" s="34" t="n">
+        <v>999.99</v>
+      </c>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="B24" s="15" t="n">
@@ -9525,6 +9736,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AL24" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="18" customHeight="1">
       <c r="B25" s="6" t="n">
@@ -9671,6 +9887,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AL25" s="34" t="n">
+        <v>1199.99</v>
+      </c>
     </row>
     <row r="26" ht="18" customHeight="1">
       <c r="B26" s="15" t="n">
@@ -9803,6 +10022,9 @@
       <c r="AK26" s="34" t="n">
         <v>1274.99</v>
       </c>
+      <c r="AL26" s="34" t="n">
+        <v>1274.99</v>
+      </c>
     </row>
     <row r="27" ht="5" customHeight="1"/>
     <row r="28" ht="22" customHeight="1">
@@ -9951,6 +10173,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AL29" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="18" customHeight="1">
       <c r="B30" s="15" t="n">
@@ -10087,6 +10314,11 @@
       <c r="AK30" s="34" t="n">
         <v>579.99</v>
       </c>
+      <c r="AL30" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="18" customHeight="1">
       <c r="B31" s="6" t="n">
@@ -10229,6 +10461,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AL31" s="13" t="n">
+        <v>699.99</v>
+      </c>
     </row>
     <row r="32" ht="18" customHeight="1">
       <c r="B32" s="15" t="n">
@@ -10365,6 +10600,9 @@
       <c r="AK32" s="34" t="n">
         <v>759.99</v>
       </c>
+      <c r="AL32" s="34" t="n">
+        <v>759.99</v>
+      </c>
     </row>
     <row r="33" ht="18" customHeight="1">
       <c r="B33" s="6" t="n">
@@ -10505,6 +10743,11 @@
       <c r="AK33" s="34" t="n">
         <v>799.99</v>
       </c>
+      <c r="AL33" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="18" customHeight="1">
       <c r="B34" s="15" t="n">
@@ -10637,6 +10880,9 @@
       <c r="AK34" s="34" t="n">
         <v>1274.99</v>
       </c>
+      <c r="AL34" s="34" t="n">
+        <v>1274.99</v>
+      </c>
     </row>
     <row r="35" ht="18" customHeight="1">
       <c r="B35" s="6" t="n">
@@ -10771,6 +11017,9 @@
       <c r="AK35" s="13" t="n">
         <v>1599.99</v>
       </c>
+      <c r="AL35" s="13" t="n">
+        <v>1599.99</v>
+      </c>
     </row>
     <row r="36" ht="18" customHeight="1">
       <c r="B36" s="15" t="n">
@@ -10903,6 +11152,11 @@
       <c r="AK36" s="34" t="n">
         <v>1975.99</v>
       </c>
+      <c r="AL36" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="B37" s="6" t="n">
@@ -11045,6 +11299,9 @@
       <c r="AK37" s="34" t="n">
         <v>2699.99</v>
       </c>
+      <c r="AL37" s="34" t="n">
+        <v>2699.99</v>
+      </c>
     </row>
     <row r="38" ht="5" customHeight="1"/>
     <row r="39" ht="22" customHeight="1">
@@ -11189,6 +11446,9 @@
       <c r="AK40" s="34" t="n">
         <v>740.99</v>
       </c>
+      <c r="AL40" s="34" t="n">
+        <v>740.99</v>
+      </c>
     </row>
     <row r="41" ht="18" customHeight="1">
       <c r="B41" s="6" t="n">
@@ -11329,6 +11589,11 @@
       <c r="AK41" s="13" t="n">
         <v>549.99</v>
       </c>
+      <c r="AL41" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="18" customHeight="1">
       <c r="B42" s="15" t="n">
@@ -11469,6 +11734,11 @@
       <c r="AK42" s="34" t="n">
         <v>799.99</v>
       </c>
+      <c r="AL42" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="43" ht="18" customHeight="1">
       <c r="B43" s="6" t="n">
@@ -11609,6 +11879,11 @@
       <c r="AK43" s="34" t="n">
         <v>949.99</v>
       </c>
+      <c r="AL43" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="44" ht="18" customHeight="1">
       <c r="B44" s="15" t="n">
@@ -11741,6 +12016,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AL44" s="34" t="n">
+        <v>1139.99</v>
+      </c>
     </row>
     <row r="45" ht="18" customHeight="1">
       <c r="B45" s="6" t="n">
@@ -11871,6 +12149,11 @@
       <c r="AK45" s="34" t="n">
         <v>1529.99</v>
       </c>
+      <c r="AL45" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="46" ht="18" customHeight="1">
       <c r="B46" s="15" t="n">
@@ -12033,6 +12316,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AL46" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="47" ht="18" customHeight="1">
       <c r="B47" s="6" t="n">
@@ -12169,6 +12457,9 @@
       <c r="AK47" s="34" t="n">
         <v>2999.99</v>
       </c>
+      <c r="AL47" s="34" t="n">
+        <v>2999.99</v>
+      </c>
     </row>
     <row r="48" ht="18" customHeight="1">
       <c r="B48" s="15" t="n">
@@ -12313,6 +12604,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AL48" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="49" ht="5" customHeight="1"/>
     <row r="50" ht="22" customHeight="1">
@@ -12453,6 +12749,9 @@
       <c r="AK51" s="34" t="n">
         <v>798.99</v>
       </c>
+      <c r="AL51" s="34" t="n">
+        <v>798.99</v>
+      </c>
     </row>
     <row r="52" ht="18" customHeight="1">
       <c r="B52" s="15" t="n">
@@ -12585,6 +12884,9 @@
       <c r="AK52" s="34" t="n">
         <v>798.99</v>
       </c>
+      <c r="AL52" s="34" t="n">
+        <v>798.99</v>
+      </c>
     </row>
     <row r="53" ht="18" customHeight="1">
       <c r="B53" s="6" t="n">
@@ -12725,6 +13027,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AL53" s="34" t="n">
+        <v>1499.99</v>
+      </c>
     </row>
     <row r="54" ht="18" customHeight="1">
       <c r="B54" s="15" t="n">
@@ -12857,6 +13162,11 @@
       <c r="AK54" s="34" t="n">
         <v>899.99</v>
       </c>
+      <c r="AL54" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="55" ht="18" customHeight="1">
       <c r="B55" s="6" t="n">
@@ -12993,6 +13303,9 @@
           <t>—</t>
         </is>
       </c>
+      <c r="AL55" s="13" t="n">
+        <v>1299.99</v>
+      </c>
     </row>
     <row r="56" ht="18" customHeight="1">
       <c r="B56" s="15" t="n">
@@ -13131,6 +13444,9 @@
       <c r="AK56" s="34" t="n">
         <v>2799.99</v>
       </c>
+      <c r="AL56" s="34" t="n">
+        <v>2799.99</v>
+      </c>
     </row>
     <row r="57" ht="18" customHeight="1">
       <c r="B57" s="6" t="n">
@@ -13264,6 +13580,11 @@
       </c>
       <c r="AK57" s="13" t="n">
         <v>1600.99</v>
+      </c>
+      <c r="AL57" s="35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
     </row>
     <row r="58" ht="18" customHeight="1">
@@ -13465,6 +13786,9 @@
       <c r="AK61" s="34" t="n">
         <v>999.99</v>
       </c>
+      <c r="AL61" s="34" t="n">
+        <v>999.99</v>
+      </c>
     </row>
     <row r="62" ht="18" customHeight="1">
       <c r="B62" s="15" t="n">
@@ -13661,6 +13985,9 @@
       <c r="AK63" s="34" t="n">
         <v>1658.99</v>
       </c>
+      <c r="AL63" s="34" t="n">
+        <v>1658.99</v>
+      </c>
     </row>
     <row r="64" ht="18" customHeight="1">
       <c r="B64" s="15" t="n">
@@ -13791,6 +14118,9 @@
         <v>2549.99</v>
       </c>
       <c r="AK64" s="34" t="n">
+        <v>2549.99</v>
+      </c>
+      <c r="AL64" s="34" t="n">
         <v>2549.99</v>
       </c>
     </row>
@@ -14101,6 +14431,9 @@
         <v>1899.99</v>
       </c>
       <c r="AK70" s="34" t="n">
+        <v>1899.99</v>
+      </c>
+      <c r="AL70" s="34" t="n">
         <v>1899.99</v>
       </c>
     </row>

</xml_diff>